<commit_message>
Cierra Mapa de impacto, matrices, colaboraciones y combinaciones unicas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -511,7 +511,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -653,6 +653,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="45.1640625" customWidth="1" min="1" max="1"/>
@@ -1230,7 +1236,7 @@
       <c r="B8" s="37" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Consultar, organizar y reaprovechar conversaciones anteriores, para tener un historial ordenado que sirva de recurso de aprendizaje y referencia.</t>
+          <t>Acceder a mi cuenta de forma segura, para que mis conversaciones y mi configuracion queden guardadas y solo yo pueda verlas.</t>
         </is>
       </c>
       <c r="D8" s="53" t="inlineStr">
@@ -1250,7 +1256,7 @@
       </c>
       <c r="G8" s="32" t="inlineStr">
         <is>
-          <t>Suena a funcionalidad, el impacto anterior lo cubre mejor?</t>
+          <t>Impacto reescrito para que no suene a funcionalidad. Validar con Farid.</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1340,7 @@
       <c r="G11" s="32" t="n"/>
     </row>
     <row r="12" ht="78" customHeight="1" thickBot="1">
-      <c r="A12" s="54" t="n"/>
+      <c r="A12" s="40" t="n"/>
       <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Administrador</t>
@@ -1365,6 +1371,35 @@
           <t>Puede agregar valor pero esto lo hace un administrador?</t>
         </is>
       </c>
+    </row>
+    <row r="13" ht="78" customHeight="1">
+      <c r="A13" s="54" t="n"/>
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="C13" s="56" t="inlineStr">
+        <is>
+          <t>Revisar los reportes de mala traduccion que envian los clientes, para decidir que mejoras priorizar en el servicio.</t>
+        </is>
+      </c>
+      <c r="D13" s="53" t="inlineStr">
+        <is>
+          <t>Si nadie revisa los reportes de mala traduccion, los errores no se corrigen y no se sabe que mejorar primero.</t>
+        </is>
+      </c>
+      <c r="E13" s="53" t="inlineStr">
+        <is>
+          <t>Mejorar primero lo que mas afecta a los usuarios.</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Revisión de reportes de calidad de traducción</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="n"/>
     </row>
     <row r="14" ht="19" customHeight="1"/>
     <row r="17" ht="16" customHeight="1"/>
@@ -1381,9 +1416,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="C1:E1"/>
+    <mergeCell ref="G1:G3"/>
+    <mergeCell ref="A4:A13"/>
     <mergeCell ref="B4:B10"/>
-    <mergeCell ref="A4:A12"/>
-    <mergeCell ref="G1:G3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F4" location="'Traductor de mensajes'!A1" display="Traductor de mensajes"/>
@@ -1791,10 +1826,11 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!#REF!</f>
-        <v/>
-      </c>
-    </row>
+        <f>'Mapa de Impacto'!C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -1916,7 +1952,7 @@
       </c>
       <c r="C2" s="23" t="inlineStr">
         <is>
-          <t>Recibir entrada del mensaje</t>
+          <t>Ingresar mi mensaje (hablado o escrito)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1946,7 +1982,7 @@
       </c>
       <c r="C3" s="23" t="inlineStr">
         <is>
-          <t>Seleccionar idioma y región destino</t>
+          <t>Seleccionar el idioma y la region destino</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1998,7 +2034,7 @@
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>Consultar idiomas disponibles</t>
+          <t>Consultar los idiomas disponibles</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2028,7 +2064,7 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Crear conversación</t>
+          <t>Crear una conversacion</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2054,7 +2090,7 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Configurar parámetros una sola vez</t>
+          <t>Configurar los parametros una sola vez</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2110,7 +2146,7 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Consultar historial</t>
+          <t>Consultar mi historial</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2136,7 +2172,7 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Abrir una conversación</t>
+          <t>Abrir una conversacion anterior</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2162,7 +2198,7 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Renombrar conversación</t>
+          <t>Renombrar una conversacion</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2188,7 +2224,7 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Eliminar conversación</t>
+          <t>Eliminar una conversacion</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2218,7 +2254,7 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Registro de cuenta</t>
+          <t>Registrarme en la aplicacion</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2244,7 +2280,7 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Inicio de sesión</t>
+          <t>Iniciar sesion</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2270,7 +2306,7 @@
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Recuperación de contraseña</t>
+          <t>Recuperar mi contrasena</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2296,7 +2332,7 @@
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Cierre de sesión</t>
+          <t>Cerrar sesion</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2326,7 +2362,7 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Reproducir audio traducido</t>
+          <t>Reproducir el audio traducido</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2352,7 +2388,7 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Entregar por el mismo canal</t>
+          <t>Recibir la traduccion por el mismo canal que use</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2382,7 +2418,7 @@
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Reportar mala traducción</t>
+          <t>Reportar una mala traduccion</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2412,7 +2448,7 @@
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Recibir mensaje traducido</t>
+          <t>Recibir el mensaje traducido</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2468,7 +2504,7 @@
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Gestionar catálogo de idiomas</t>
+          <t>Gestionar el catalogo de idiomas</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2498,7 +2534,7 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Revisar reportes de mala traducción</t>
+          <t>Revisar los reportes de mala traduccion</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2510,10 +2546,9 @@
         <f>C23</f>
         <v/>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Revisar los reportes de mala traduccion que envian los clientes, para priorizar las mejoras del servicio.</t>
-        </is>
+      <c r="F23">
+        <f>'Mapa de Impacto'!C13</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mapa de Impacto: redacta Problema y Beneficio en tercera persona
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -1166,7 +1166,7 @@
       </c>
       <c r="D5" s="53" t="inlineStr">
         <is>
-          <t>Si cada vez que mando un mensaje tengo que volver a escoger los idiomas, pierdo tiempo y la conversacion se vuelve lenta.</t>
+          <t>Si el usuario tiene que volver a escoger los idiomas cada vez que envia un mensaje, pierde tiempo y la conversacion se vuelve lenta.</t>
         </is>
       </c>
       <c r="E5" s="53" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D7" s="53" t="inlineStr">
         <is>
-          <t>Si las conversaciones no se guardan, al cerrar la app se pierde lo que se dijo y no hay como repasar las frases ni aprender de ellas.</t>
+          <t>Si las conversaciones no se guardan, al cerrar la app se pierde lo que se dijo y el usuario no puede repasar las frases ni aprender de ellas.</t>
         </is>
       </c>
       <c r="E7" s="53" t="inlineStr">
@@ -1236,17 +1236,17 @@
       <c r="B8" s="37" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Acceder a mi cuenta de forma segura, para que mis conversaciones y mi configuracion queden guardadas y solo yo pueda verlas.</t>
+          <t>Acceder a la cuenta de forma segura, para que las conversaciones y la configuracion queden guardadas y solo el usuario pueda verlas.</t>
         </is>
       </c>
       <c r="D8" s="53" t="inlineStr">
         <is>
-          <t>Si no hay una cuenta, las conversaciones no quedan ligadas a nadie: cualquiera con el celular las veria y, si cambio de celular, las pierdo.</t>
+          <t>Si no hay una cuenta, las conversaciones no quedan ligadas a nadie: cualquiera con el celular las podria ver y, si el usuario cambia de celular, las pierde.</t>
         </is>
       </c>
       <c r="E8" s="53" t="inlineStr">
         <is>
-          <t>Tener mis conversaciones guardadas y que sean solo mias.</t>
+          <t>Tener las conversaciones guardadas y que sean solo del usuario.</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="D9" s="53" t="inlineStr">
         <is>
-          <t>Si la traduccion solo sale en texto o con una voz que suena robotica, la otra persona no entiende bien lo que quise decir y todo se siente forzado.</t>
+          <t>Si la traduccion solo sale en texto o con una voz que suena robotica, la otra persona no entiende bien lo que el usuario quiso decir y todo se siente forzado.</t>
         </is>
       </c>
       <c r="E9" s="53" t="inlineStr">
         <is>
-          <t>Hablar y escuchar de forma natural, como en mi propio idioma.</t>
+          <t>Hablar y escuchar de forma natural, como en el propio idioma.</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D10" s="53" t="inlineStr">
         <is>
-          <t>Si no puedo avisar cuando una traduccion sale mal, el error se queda y se repite, y uno termina desconfiando de la app.</t>
+          <t>Si el usuario no puede avisar cuando una traduccion sale mal, el error se queda y se repite, y termina desconfiando de la app.</t>
         </is>
       </c>
       <c r="E10" s="53" t="inlineStr">
@@ -1415,10 +1415,10 @@
     <row r="27" ht="128" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A4:A13"/>
     <mergeCell ref="C1:E1"/>
+    <mergeCell ref="B4:B10"/>
     <mergeCell ref="G1:G3"/>
-    <mergeCell ref="A4:A13"/>
-    <mergeCell ref="B4:B10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F4" location="'Traductor de mensajes'!A1" display="Traductor de mensajes"/>
@@ -1830,7 +1830,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Entregables como epicas (modulos): 7 modulos y 25 HU, una hoja por modulo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -9,16 +9,13 @@
     <sheet name="Mapa de Impacto" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Entregables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Backlog - Historias de Usuario" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Traductor de mensajes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Configuración de idiomas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gestión de conversaciones" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Historial de conversaciones" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gestión de perfil" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Audio traducido" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Reporte mala traducción" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Participación conversación" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Catálogo idiomas (Admin)" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Reportes calidad (Admin)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Traduccion de mensajes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Config. de conversacion" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Historial" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cuenta de usuario" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Participacion interlocutor" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Reportes de calidad" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Admin idiomas y regiones" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1151,7 +1148,7 @@
       </c>
       <c r="F4" s="31" t="inlineStr">
         <is>
-          <t>Traductor de mensajes</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
       <c r="G4" s="32" t="n"/>
@@ -1176,7 +1173,7 @@
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Configuración de idiomas origen–destino</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="G5" s="32" t="n"/>
@@ -1201,7 +1198,7 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Gestión de conversaciones</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="G6" s="32" t="n"/>
@@ -1226,7 +1223,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Historial y gestión de conversaciones traducidas</t>
+          <t>Modulo de historial de conversaciones</t>
         </is>
       </c>
       <c r="G7" s="32" t="n"/>
@@ -1251,7 +1248,7 @@
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="G8" s="32" t="inlineStr">
@@ -1280,7 +1277,7 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Reproducción y personalización de audio traducido</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
       <c r="G9" s="32" t="n"/>
@@ -1305,7 +1302,7 @@
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Reporte de mala traducción</t>
+          <t>Modulo de reportes de calidad</t>
         </is>
       </c>
       <c r="G10" s="32" t="n"/>
@@ -1334,7 +1331,7 @@
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>Participación en la conversación traducida</t>
+          <t>Modulo de participacion del interlocutor</t>
         </is>
       </c>
       <c r="G11" s="32" t="n"/>
@@ -1363,7 +1360,7 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Gestión del catálogo de idiomas y regiones</t>
+          <t>Modulo de administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="G12" s="32" t="inlineStr">
@@ -1396,7 +1393,7 @@
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>Revisión de reportes de calidad de traducción</t>
+          <t>Modulo de reportes de calidad</t>
         </is>
       </c>
       <c r="G13" s="32" t="n"/>
@@ -1420,17 +1417,6 @@
     <mergeCell ref="B4:B10"/>
     <mergeCell ref="G1:G3"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="F4" location="'Traductor de mensajes'!A1" display="Traductor de mensajes"/>
-    <hyperlink ref="F5" location="'Configuración de idiomas'!A1" display="Configuración de idiomas origen–destino"/>
-    <hyperlink ref="F6" location="'Gestión de conversaciones'!A1" display="Gestión de conversaciones"/>
-    <hyperlink ref="F7" location="'Historial de conversaciones'!A1" display="Historial y gestión de conversaciones traducidas"/>
-    <hyperlink ref="F8" location="'Gestión de perfil'!A1" display="Gestión de perfil de usuario"/>
-    <hyperlink ref="F9" location="'Audio traducido'!A1" display="Reproducción y personalización de audio traducido"/>
-    <hyperlink ref="F10" location="'Reporte mala traducción'!A1" display="Reporte de mala traducción"/>
-    <hyperlink ref="F11" location="'Participación conversación'!A1" display="Participación en la conversación traducida"/>
-    <hyperlink ref="F12" location="'Catálogo idiomas (Admin)'!A1" display="Gestión del catálogo de idiomas y regiones"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1441,7 +1427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1457,7 +1443,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Reporte de mala traducción</t>
+          <t>Modulo de administracion de idiomas y regiones</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1455,7 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Cliente Traductor</t>
+          <t>Administrador</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1466,7 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C10</f>
+        <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
     </row>
@@ -1513,377 +1499,80 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="27.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Reportar mala traducción</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>reportar cuando una traducción no fue correcta o natural</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Reportar cuando una traducción no fue correcta o natural, para contribuir a que la calidad del servicio mejore con el tiempo.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C25</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D25</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E25</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C26</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D26</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E26</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="41.5" customHeight="1">
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D10" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Participación en la conversación traducida</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="41.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Recibir mensaje traducido</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>escuchar o leer en mi propio idioma el mensaje que me enviaron</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Recibir en mi propio idioma los mensajes que me envían y responder en el mío, para participar en la conversación de forma natural aunque no comparta el idioma de la otra persona.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.5" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Responder en mi idioma</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>responder hablando o escribiendo en mi propio idioma para que la otra persona lo reciba traducido</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Recibir en mi propio idioma los mensajes que me envían y responder en el mío, para participar en la conversación de forma natural aunque no comparta el idioma de la otra persona.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D11" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Gestión del catálogo de idiomas y regiones</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="41.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Gestionar catálogo de idiomas</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>agregar, activar o desactivar los idiomas, regiones y acentos disponibles</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Gestionar el catálogo de idiomas, regiones y acentos soportados por la aplicación, para mantener actualizada y disponible la oferta de idiomas del servicio.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D12" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Revisión de reportes de calidad de traducción</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="27.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Revisar reportes de mala traducción</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>revisar los reportes de mala traducción enviados por los clientes para priorizar mejoras</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Revisar los reportes de mala traducción enviados por los clientes, para priorizar las mejoras y la evolución de la calidad del servicio.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D13" display="← Volver al Mapa de Impacto"/>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1895,7 +1584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1941,7 +1630,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Traductor de mensajes</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
       <c r="B2" s="33" t="inlineStr">
@@ -1951,7 +1640,7 @@
       </c>
       <c r="C2" s="23" t="inlineStr">
         <is>
-          <t>Ingresar mi mensaje (hablado o escrito)</t>
+          <t>Ingresar mi mensaje hablando</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1969,11 +1658,7 @@
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="33" t="inlineStr">
-        <is>
-          <t>Configuración de idiomas origen–destino</t>
-        </is>
-      </c>
+      <c r="A3" s="34" t="n"/>
       <c r="B3" s="33" t="inlineStr">
         <is>
           <t>HU0002</t>
@@ -1981,7 +1666,7 @@
       </c>
       <c r="C3" s="23" t="inlineStr">
         <is>
-          <t>Seleccionar el idioma y la region destino</t>
+          <t>Ingresar mi mensaje escribiendo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1994,7 +1679,7 @@
         <v/>
       </c>
       <c r="F3">
-        <f>'Mapa de Impacto'!C5</f>
+        <f>'Mapa de Impacto'!C4</f>
         <v/>
       </c>
     </row>
@@ -2007,7 +1692,7 @@
       </c>
       <c r="C4" s="23" t="inlineStr">
         <is>
-          <t>Reconocer el idioma origen</t>
+          <t>Traducir mi mensaje al idioma destino en tiempo real</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2020,12 +1705,12 @@
         <v/>
       </c>
       <c r="F4">
-        <f>'Mapa de Impacto'!C5</f>
+        <f>'Mapa de Impacto'!C4</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="35" t="n"/>
+      <c r="A5" s="34" t="n"/>
       <c r="B5" s="33" t="inlineStr">
         <is>
           <t>HU0004</t>
@@ -2033,7 +1718,7 @@
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>Consultar los idiomas disponibles</t>
+          <t>Escuchar el mensaje traducido</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2046,16 +1731,12 @@
         <v/>
       </c>
       <c r="F5">
-        <f>'Mapa de Impacto'!C5</f>
+        <f>'Mapa de Impacto'!C9</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>Gestión de conversaciones</t>
-        </is>
-      </c>
+      <c r="A6" s="35" t="n"/>
       <c r="B6" s="33" t="inlineStr">
         <is>
           <t>HU0005</t>
@@ -2063,7 +1744,7 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Crear una conversacion</t>
+          <t>Recibir la traduccion por el mismo canal que use</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2076,12 +1757,16 @@
         <v/>
       </c>
       <c r="F6">
-        <f>'Mapa de Impacto'!C6</f>
+        <f>'Mapa de Impacto'!C9</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="34" t="n"/>
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Modulo de configuracion de conversacion</t>
+        </is>
+      </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
           <t>HU0006</t>
@@ -2089,7 +1774,7 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Configurar los parametros una sola vez</t>
+          <t>Seleccionar el idioma y la region destino</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2102,12 +1787,12 @@
         <v/>
       </c>
       <c r="F7">
-        <f>'Mapa de Impacto'!C6</f>
+        <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="35" t="n"/>
+      <c r="A8" s="34" t="n"/>
       <c r="B8" s="33" t="inlineStr">
         <is>
           <t>HU0007</t>
@@ -2115,7 +1800,7 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Mantener el hilo continuo</t>
+          <t>Reconocer el idioma origen</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2128,16 +1813,12 @@
         <v/>
       </c>
       <c r="F8">
-        <f>'Mapa de Impacto'!C6</f>
+        <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>Historial y gestión de conversaciones traducidas</t>
-        </is>
-      </c>
+      <c r="A9" s="34" t="n"/>
       <c r="B9" s="33" t="inlineStr">
         <is>
           <t>HU0008</t>
@@ -2145,7 +1826,7 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Consultar mi historial</t>
+          <t>Consultar los idiomas disponibles</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2158,7 +1839,7 @@
         <v/>
       </c>
       <c r="F9">
-        <f>'Mapa de Impacto'!C7</f>
+        <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
     </row>
@@ -2171,7 +1852,7 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Abrir una conversacion anterior</t>
+          <t>Crear una conversacion</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2184,7 +1865,7 @@
         <v/>
       </c>
       <c r="F10">
-        <f>'Mapa de Impacto'!C7</f>
+        <f>'Mapa de Impacto'!C6</f>
         <v/>
       </c>
     </row>
@@ -2197,7 +1878,7 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Renombrar una conversacion</t>
+          <t>Configurar los parametros una sola vez</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2210,7 +1891,7 @@
         <v/>
       </c>
       <c r="F11">
-        <f>'Mapa de Impacto'!C7</f>
+        <f>'Mapa de Impacto'!C6</f>
         <v/>
       </c>
     </row>
@@ -2223,7 +1904,7 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Eliminar una conversacion</t>
+          <t>Mantener el hilo continuo</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2236,14 +1917,14 @@
         <v/>
       </c>
       <c r="F12">
-        <f>'Mapa de Impacto'!C7</f>
+        <f>'Mapa de Impacto'!C6</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="33" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de historial de conversaciones</t>
         </is>
       </c>
       <c r="B13" s="33" t="inlineStr">
@@ -2253,7 +1934,7 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Registrarme en la aplicacion</t>
+          <t>Consultar mi historial</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2266,7 +1947,7 @@
         <v/>
       </c>
       <c r="F13">
-        <f>'Mapa de Impacto'!C8</f>
+        <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
     </row>
@@ -2279,7 +1960,7 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Iniciar sesion</t>
+          <t>Abrir una conversacion anterior</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2292,7 +1973,7 @@
         <v/>
       </c>
       <c r="F14">
-        <f>'Mapa de Impacto'!C8</f>
+        <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
     </row>
@@ -2305,7 +1986,7 @@
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Recuperar mi contrasena</t>
+          <t>Renombrar una conversacion</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2318,7 +1999,7 @@
         <v/>
       </c>
       <c r="F15">
-        <f>'Mapa de Impacto'!C8</f>
+        <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
     </row>
@@ -2331,7 +2012,7 @@
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Cerrar sesion</t>
+          <t>Eliminar una conversacion</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2344,14 +2025,14 @@
         <v/>
       </c>
       <c r="F16">
-        <f>'Mapa de Impacto'!C8</f>
+        <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="33" t="inlineStr">
         <is>
-          <t>Reproducción y personalización de audio traducido</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="B17" s="33" t="inlineStr">
@@ -2361,7 +2042,7 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Reproducir el audio traducido</t>
+          <t>Registrarme en la aplicacion</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2374,12 +2055,12 @@
         <v/>
       </c>
       <c r="F17">
-        <f>'Mapa de Impacto'!C9</f>
+        <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="35" t="n"/>
+      <c r="A18" s="34" t="n"/>
       <c r="B18" s="33" t="inlineStr">
         <is>
           <t>HU0017</t>
@@ -2387,7 +2068,7 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Recibir la traduccion por el mismo canal que use</t>
+          <t>Iniciar sesion</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2400,16 +2081,12 @@
         <v/>
       </c>
       <c r="F18">
-        <f>'Mapa de Impacto'!C9</f>
+        <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>Reporte de mala traducción</t>
-        </is>
-      </c>
+      <c r="A19" s="34" t="n"/>
       <c r="B19" s="33" t="inlineStr">
         <is>
           <t>HU0018</t>
@@ -2417,7 +2094,7 @@
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Reportar una mala traduccion</t>
+          <t>Recuperar mi contrasena</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2430,16 +2107,12 @@
         <v/>
       </c>
       <c r="F19">
-        <f>'Mapa de Impacto'!C10</f>
+        <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="33" t="inlineStr">
-        <is>
-          <t>Participación en la conversación traducida</t>
-        </is>
-      </c>
+      <c r="A20" s="35" t="n"/>
       <c r="B20" s="33" t="inlineStr">
         <is>
           <t>HU0019</t>
@@ -2447,12 +2120,12 @@
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Recibir el mensaje traducido</t>
+          <t>Cerrar sesion</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Interlocutor</t>
+          <t>Cliente Traductor</t>
         </is>
       </c>
       <c r="E20">
@@ -2460,12 +2133,16 @@
         <v/>
       </c>
       <c r="F20">
-        <f>'Mapa de Impacto'!C11</f>
+        <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="35" t="n"/>
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Modulo de participacion del interlocutor</t>
+        </is>
+      </c>
       <c r="B21" s="33" t="inlineStr">
         <is>
           <t>HU0020</t>
@@ -2473,7 +2150,7 @@
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Responder en mi idioma</t>
+          <t>Recibir el mensaje traducido</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2491,11 +2168,7 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>Gestión del catálogo de idiomas y regiones</t>
-        </is>
-      </c>
+      <c r="A22" s="35" t="n"/>
       <c r="B22" s="33" t="inlineStr">
         <is>
           <t>HU0021</t>
@@ -2503,12 +2176,12 @@
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Gestionar el catalogo de idiomas</t>
+          <t>Responder en mi idioma</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Administrador</t>
+          <t>Interlocutor</t>
         </is>
       </c>
       <c r="E22">
@@ -2516,14 +2189,14 @@
         <v/>
       </c>
       <c r="F22">
-        <f>'Mapa de Impacto'!C12</f>
+        <f>'Mapa de Impacto'!C11</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="33" t="inlineStr">
         <is>
-          <t>Revisión de reportes de calidad de traducción</t>
+          <t>Modulo de reportes de calidad</t>
         </is>
       </c>
       <c r="B23" s="33" t="inlineStr">
@@ -2533,12 +2206,12 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Revisar los reportes de mala traduccion</t>
+          <t>Reportar una mala traduccion</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Administrador</t>
+          <t>Cliente Traductor</t>
         </is>
       </c>
       <c r="E23">
@@ -2546,29 +2219,120 @@
         <v/>
       </c>
       <c r="F23">
+        <f>'Mapa de Impacto'!C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="n"/>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>HU0023</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>Revisar los reportes de mala traduccion</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="E24">
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="F24">
         <f>'Mapa de Impacto'!C13</f>
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>Modulo de administracion de idiomas y regiones</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>HU0024</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Agregar un idioma o una region</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="E25">
+        <f>C25</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>'Mapa de Impacto'!C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="n"/>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>HU0025</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>Activar o desactivar un idioma o una region</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Administrador</t>
+        </is>
+      </c>
+      <c r="E26">
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="F26">
+        <f>'Mapa de Impacto'!C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="60"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A7:A12"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A21:A22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" location="'Traductor de mensajes'!A1" display="Traductor de mensajes"/>
-    <hyperlink ref="A3" location="'Configuración de idiomas'!A1" display="Configuración de idiomas origen–destino"/>
-    <hyperlink ref="A6" location="'Gestión de conversaciones'!A1" display="Gestión de conversaciones"/>
-    <hyperlink ref="A9" location="'Historial de conversaciones'!A1" display="Historial y gestión de conversaciones traducidas"/>
     <hyperlink ref="A13" location="'Gestión de perfil'!A1" display="Gestión de perfil de usuario"/>
     <hyperlink ref="A17" location="'Audio traducido'!A1" display="Reproducción y personalización de audio traducido"/>
-    <hyperlink ref="A19" location="'Reporte mala traducción'!A1" display="Reporte de mala traducción"/>
-    <hyperlink ref="A20" location="'Participación conversación'!A1" display="Participación en la conversación traducida"/>
-    <hyperlink ref="A22" location="'Catálogo idiomas (Admin)'!A1" display="Gestión del catálogo de idiomas y regiones"/>
     <hyperlink ref="A23" location="'Reportes calidad (Admin)'!A1" display="Revisión de reportes de calidad de traducción"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2621,7 +2385,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>Traductor de mensajes</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
       <c r="B2" s="12" t="inlineStr">
@@ -2648,7 +2412,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Traductor de mensajes</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
@@ -2671,7 +2435,7 @@
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Configuración de idiomas origen–destino</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
@@ -2698,7 +2462,7 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Configuración de idiomas origen–destino</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -2721,7 +2485,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Configuración de idiomas origen–destino</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -2744,7 +2508,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Gestión de conversaciones</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -2771,7 +2535,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Gestión de conversaciones</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -2794,7 +2558,7 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Gestión de conversaciones</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2817,7 +2581,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Historial y gestión de conversaciones traducidas</t>
+          <t>Modulo de historial de conversaciones</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -2844,7 +2608,7 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Historial y gestión de conversaciones traducidas</t>
+          <t>Modulo de historial de conversaciones</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -2867,7 +2631,7 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Historial y gestión de conversaciones traducidas</t>
+          <t>Modulo de historial de conversaciones</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -2890,7 +2654,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Historial y gestión de conversaciones traducidas</t>
+          <t>Modulo de historial de conversaciones</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -2913,7 +2677,7 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -2940,7 +2704,7 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2963,7 +2727,7 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -2986,7 +2750,7 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -3009,7 +2773,7 @@
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -3032,7 +2796,7 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -3055,7 +2819,7 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Reproducción y personalización de audio traducido</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -3082,7 +2846,7 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Reproducción y personalización de audio traducido</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -3105,7 +2869,7 @@
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Reporte de mala traducción</t>
+          <t>Modulo de reportes de calidad</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -3132,7 +2896,7 @@
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Participación en la conversación traducida</t>
+          <t>Modulo de participacion del interlocutor</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
@@ -3159,7 +2923,7 @@
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Participación en la conversación traducida</t>
+          <t>Modulo de participacion del interlocutor</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
@@ -3182,7 +2946,7 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Gestión del catálogo de idiomas y regiones</t>
+          <t>Modulo de administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
@@ -3209,7 +2973,7 @@
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Revisión de reportes de calidad de traducción</t>
+          <t>Modulo de reportes de calidad</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
@@ -3253,7 +3017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3269,7 +3033,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Traductor de mensajes</t>
+          <t>Modulo de traduccion de mensajes</t>
         </is>
       </c>
     </row>
@@ -3285,14 +3049,14 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C4</f>
+        <f>'Mapa de Impacto'!C4&amp;CHAR(10)&amp;'Mapa de Impacto'!C9</f>
         <v/>
       </c>
     </row>
@@ -3325,53 +3089,126 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="41.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Recibir entrada del mensaje</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>decir (hablar) el mensaje que quiero traducir</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Traducir un mensaje de un idioma origen a un idioma destino en tiempo real, para comunicarme fácil y rápidamente con personas que hablan otro idioma conservando el contexto cultural, el tono y los modismos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.5" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Recibir entrada del mensaje</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>escribir el mensaje que quiero traducir</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Traducir un mensaje de un idioma origen a un idioma destino en tiempo real, para comunicarme fácil y rápidamente con personas que hablan otro idioma conservando el contexto cultural, el tono y los modismos.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C2</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D2</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E2</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C3</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D3</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E3</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18">
+        <f>Entregables!C4</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D4</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E4</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18">
+        <f>Entregables!C5</f>
+        <v/>
+      </c>
+      <c r="B11" s="18">
+        <f>Entregables!D5</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>Entregables!E5</f>
+        <v/>
+      </c>
+      <c r="D11" s="18">
+        <f>Entregables!F5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="18">
+        <f>Entregables!C6</f>
+        <v/>
+      </c>
+      <c r="B12" s="18">
+        <f>Entregables!D6</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>Entregables!E6</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
+        <f>Entregables!F6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D4" display="← Volver al Mapa de Impacto"/>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3383,7 +3220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3399,7 +3236,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Configuración de idiomas origen–destino</t>
+          <t>Modulo de configuracion de conversacion</t>
         </is>
       </c>
     </row>
@@ -3415,14 +3252,14 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C5</f>
+        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C6</f>
         <v/>
       </c>
     </row>
@@ -3455,75 +3292,143 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="41.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Seleccionar idioma y región destino</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>elegir el idioma y la región a los que quiero traducir</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Definir y conocer los idiomas y regiones con los que me quiero comunicar, para dejar claro desde el inicio qué idioma hablo y a qué idioma/región necesito traducir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.5" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Reconocer el idioma origen</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>empezar a hablar sin tener que indicar manualmente mi idioma de origen, reconociéndolo desde mi primer mensaje de voz (Conversacion-RN-2)</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Definir y conocer los idiomas y regiones con los que me quiero comunicar, para dejar claro desde el inicio qué idioma hablo y a qué idioma/región necesito traducir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="41.5" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Consultar idiomas disponibles</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>ver la lista de idiomas y regiones que TalkLate soporta antes de configurar la conversación</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Definir y conocer los idiomas y regiones con los que me quiero comunicar, para dejar claro desde el inicio qué idioma hablo y a qué idioma/región necesito traducir.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C7</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D7</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E7</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C8</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D8</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E8</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18">
+        <f>Entregables!C9</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D9</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E9</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18">
+        <f>Entregables!C10</f>
+        <v/>
+      </c>
+      <c r="B11" s="18">
+        <f>Entregables!D10</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>Entregables!E10</f>
+        <v/>
+      </c>
+      <c r="D11" s="18">
+        <f>Entregables!F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="18">
+        <f>Entregables!C11</f>
+        <v/>
+      </c>
+      <c r="B12" s="18">
+        <f>Entregables!D11</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>Entregables!E11</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
+        <f>Entregables!F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="18">
+        <f>Entregables!C12</f>
+        <v/>
+      </c>
+      <c r="B13" s="18">
+        <f>Entregables!D12</f>
+        <v/>
+      </c>
+      <c r="C13" s="18">
+        <f>Entregables!E12</f>
+        <v/>
+      </c>
+      <c r="D13" s="18">
+        <f>Entregables!F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D5" display="← Volver al Mapa de Impacto"/>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3535,7 +3440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3551,7 +3456,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Gestión de conversaciones</t>
+          <t>Modulo de historial de conversaciones</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3479,7 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C6</f>
+        <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
     </row>
@@ -3607,75 +3512,109 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="41.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Crear conversación</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>iniciar una nueva conversación con otra persona</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Configurar una conversación una sola vez y mantener su hilo continuo, para conversar de forma fluida y organizada sin reconfigurar nada en cada mensaje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.5" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Configurar parámetros una sola vez</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>definir el idioma y la región destino una única vez al crear la conversación (Conversacion-RN-1)</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Configurar una conversación una sola vez y mantener su hilo continuo, para conversar de forma fluida y organizada sin reconfigurar nada en cada mensaje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="41.5" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Mantener el hilo continuo</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>que cada mensaje que envío o recibo dentro de esa conversación se traduzca automáticamente sin volver a configurar nada</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Configurar una conversación una sola vez y mantener su hilo continuo, para conversar de forma fluida y organizada sin reconfigurar nada en cada mensaje.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C13</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D13</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E13</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C14</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D14</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E14</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18">
+        <f>Entregables!C15</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D15</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E15</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18">
+        <f>Entregables!C16</f>
+        <v/>
+      </c>
+      <c r="B11" s="18">
+        <f>Entregables!D16</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>Entregables!E16</f>
+        <v/>
+      </c>
+      <c r="D11" s="18">
+        <f>Entregables!F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D6" display="← Volver al Mapa de Impacto"/>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3687,7 +3626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3703,7 +3642,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Historial y gestión de conversaciones traducidas</t>
+          <t>Modulo de cuenta de usuario</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3665,7 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C7</f>
+        <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
     </row>
@@ -3759,97 +3698,109 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="41.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Consultar historial</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>ver la lista de mis conversaciones anteriores</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Consultar, organizar y reaprovechar mis conversaciones anteriores, para tener un historial ordenado que me sirva de recurso de aprendizaje y referencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.5" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Abrir una conversación</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>abrir una conversación anterior y ver sus mensajes originales y traducidos</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Consultar, organizar y reaprovechar mis conversaciones anteriores, para tener un historial ordenado que me sirva de recurso de aprendizaje y referencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="41.5" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Renombrar conversación</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>cambiar el nombre de una conversación para identificarla fácilmente</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Consultar, organizar y reaprovechar mis conversaciones anteriores, para tener un historial ordenado que me sirva de recurso de aprendizaje y referencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="41.5" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Eliminar conversación</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>eliminar una conversación que ya no necesito</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Consultar, organizar y reaprovechar mis conversaciones anteriores, para tener un historial ordenado que me sirva de recurso de aprendizaje y referencia.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C17</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D17</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E17</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C18</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D18</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E18</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18">
+        <f>Entregables!C19</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D19</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E19</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18">
+        <f>Entregables!C20</f>
+        <v/>
+      </c>
+      <c r="B11" s="18">
+        <f>Entregables!D20</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>Entregables!E20</f>
+        <v/>
+      </c>
+      <c r="D11" s="18">
+        <f>Entregables!F20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D7" display="← Volver al Mapa de Impacto"/>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3861,7 +3812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3877,7 +3828,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Gestión de perfil de usuario</t>
+          <t>Modulo de participacion del interlocutor</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3840,7 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Cliente Traductor</t>
+          <t>Interlocutor</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3851,7 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C8</f>
+        <f>'Mapa de Impacto'!C11</f>
         <v/>
       </c>
     </row>
@@ -3933,141 +3884,80 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="27.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Registro de cuenta</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>registrarme con mi nombre, apellido, correo y contraseña</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Crear y administrar mi perfil de forma sencilla y segura, para acceder con mi identidad protegida a mis configuraciones y conversaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.5" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Registro de cuenta</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>registrarme indicando mi fecha de nacimiento y que solo se permita el registro si tengo al menos 13 años (Usuario-RN-2)</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Crear y administrar mi perfil de forma sencilla y segura, para acceder con mi identidad protegida a mis configuraciones y conversaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="27.5" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Inicio de sesión</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>iniciar sesión con mi correo y contraseña</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Crear y administrar mi perfil de forma sencilla y segura, para acceder con mi identidad protegida a mis configuraciones y conversaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="27.5" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Recuperación de contraseña</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>solicitar un código de recuperación a mi correo cuando olvide mi contraseña</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Crear y administrar mi perfil de forma sencilla y segura, para acceder con mi identidad protegida a mis configuraciones y conversaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="27.5" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Recuperación de contraseña</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>definir una nueva contraseña usando el código de recuperación recibido</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Crear y administrar mi perfil de forma sencilla y segura, para acceder con mi identidad protegida a mis configuraciones y conversaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="27.5" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Cierre de sesión</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>cerrar mi sesión activa cuando termine de usar la app</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Crear y administrar mi perfil de forma sencilla y segura, para acceder con mi identidad protegida a mis configuraciones y conversaciones.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C21</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D21</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E21</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C22</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D22</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E22</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="41.5" customHeight="1">
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D8" display="← Volver al Mapa de Impacto"/>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4079,7 +3969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4095,7 +3985,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Reproducción y personalización de audio traducido</t>
+          <t>Modulo de reportes de calidad</t>
         </is>
       </c>
     </row>
@@ -4107,18 +3997,18 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
+          <t>Cliente Traductor / Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C9</f>
+        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
         <v/>
       </c>
     </row>
@@ -4151,53 +4041,80 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="41.5" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Reproducir audio traducido</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>escuchar el mensaje traducido en un audio claro y natural</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Escuchar y entregar el mensaje traducido en el mismo canal (voz o texto) de forma clara y natural, para que mi interlocutor lo reciba de forma cómoda y comprensible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="41.5" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Entregar por el mismo canal</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>recibir el mensaje traducido en el mismo formato que usé para enviarlo (audio si hablé, texto si escribí)</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Escuchar y entregar el mensaje traducido en el mismo canal (voz o texto) de forma clara y natural, para que mi interlocutor lo reciba de forma cómoda y comprensible.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C23</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D23</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E23</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C24</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D24</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E24</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="41.5" customHeight="1">
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!D9" display="← Volver al Mapa de Impacto"/>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Epicas sin el prefijo 'Modulo de'
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -1148,7 +1148,7 @@
       </c>
       <c r="F4" s="31" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
       <c r="G4" s="32" t="n"/>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="G5" s="32" t="n"/>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="G6" s="32" t="n"/>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Modulo de historial de conversaciones</t>
+          <t>Historial de conversaciones</t>
         </is>
       </c>
       <c r="G7" s="32" t="n"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="G8" s="32" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
       <c r="G9" s="32" t="n"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Modulo de reportes de calidad</t>
+          <t>Reportes de calidad</t>
         </is>
       </c>
       <c r="G10" s="32" t="n"/>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>Modulo de participacion del interlocutor</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
       <c r="G11" s="32" t="n"/>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Modulo de administracion de idiomas y regiones</t>
+          <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="G12" s="32" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>Modulo de reportes de calidad</t>
+          <t>Reportes de calidad</t>
         </is>
       </c>
       <c r="G13" s="32" t="n"/>
@@ -1427,7 +1427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Modulo de administracion de idiomas y regiones</t>
+          <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
     </row>
@@ -1470,6 +1470,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -1477,6 +1478,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -1541,35 +1543,6 @@
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="18" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -1584,7 +1557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1630,7 +1603,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
       <c r="B2" s="33" t="inlineStr">
@@ -1764,7 +1737,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="33" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="B7" s="33" t="inlineStr">
@@ -1924,7 +1897,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="33" t="inlineStr">
         <is>
-          <t>Modulo de historial de conversaciones</t>
+          <t>Historial de conversaciones</t>
         </is>
       </c>
       <c r="B13" s="33" t="inlineStr">
@@ -2032,7 +2005,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="33" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B17" s="33" t="inlineStr">
@@ -2140,7 +2113,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="33" t="inlineStr">
         <is>
-          <t>Modulo de participacion del interlocutor</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
       <c r="B21" s="33" t="inlineStr">
@@ -2196,7 +2169,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="33" t="inlineStr">
         <is>
-          <t>Modulo de reportes de calidad</t>
+          <t>Reportes de calidad</t>
         </is>
       </c>
       <c r="B23" s="33" t="inlineStr">
@@ -2252,7 +2225,7 @@
     <row r="25">
       <c r="A25" s="33" t="inlineStr">
         <is>
-          <t>Modulo de administracion de idiomas y regiones</t>
+          <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="B25" s="33" t="inlineStr">
@@ -2305,27 +2278,13 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="60"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="A2:A6"/>
     <mergeCell ref="A7:A12"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A17:A20"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A21:A22"/>
   </mergeCells>
@@ -2385,7 +2344,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
       <c r="B2" s="12" t="inlineStr">
@@ -2412,7 +2371,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
@@ -2435,7 +2394,7 @@
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
@@ -2462,7 +2421,7 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -2485,7 +2444,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -2508,7 +2467,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -2535,7 +2494,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -2558,7 +2517,7 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2581,7 +2540,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Modulo de historial de conversaciones</t>
+          <t>Historial de conversaciones</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -2608,7 +2567,7 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Modulo de historial de conversaciones</t>
+          <t>Historial de conversaciones</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -2631,7 +2590,7 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Modulo de historial de conversaciones</t>
+          <t>Historial de conversaciones</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -2654,7 +2613,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Modulo de historial de conversaciones</t>
+          <t>Historial de conversaciones</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -2677,7 +2636,7 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -2704,7 +2663,7 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2727,7 +2686,7 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -2750,7 +2709,7 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -2773,7 +2732,7 @@
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -2796,7 +2755,7 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -2819,7 +2778,7 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -2846,7 +2805,7 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -2869,7 +2828,7 @@
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Modulo de reportes de calidad</t>
+          <t>Reportes de calidad</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -2896,7 +2855,7 @@
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Modulo de participacion del interlocutor</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
@@ -2923,7 +2882,7 @@
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Modulo de participacion del interlocutor</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
@@ -2946,7 +2905,7 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Modulo de administracion de idiomas y regiones</t>
+          <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
@@ -2973,7 +2932,7 @@
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Modulo de reportes de calidad</t>
+          <t>Reportes de calidad</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
@@ -3017,7 +2976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3033,7 +2992,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Modulo de traduccion de mensajes</t>
+          <t>Traduccion de mensajes</t>
         </is>
       </c>
     </row>
@@ -3060,6 +3019,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3067,6 +3027,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3179,33 +3140,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3220,7 +3154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3236,7 +3170,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Modulo de configuracion de conversacion</t>
+          <t>Configuracion de conversacion</t>
         </is>
       </c>
     </row>
@@ -3263,6 +3197,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3270,6 +3205,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3400,32 +3336,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3440,7 +3350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3456,7 +3366,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Modulo de historial de conversaciones</t>
+          <t>Historial de conversaciones</t>
         </is>
       </c>
     </row>
@@ -3483,6 +3393,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3490,6 +3401,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3584,34 +3496,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3626,7 +3510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3642,7 +3526,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Modulo de cuenta de usuario</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
     </row>
@@ -3669,6 +3553,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3676,6 +3561,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3770,34 +3656,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3812,7 +3670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3828,7 +3686,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Modulo de participacion del interlocutor</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
     </row>
@@ -3855,6 +3713,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3862,6 +3721,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3926,35 +3786,6 @@
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="18" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3969,7 +3800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3985,7 +3816,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Modulo de reportes de calidad</t>
+          <t>Reportes de calidad</t>
         </is>
       </c>
     </row>
@@ -4012,6 +3843,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -4019,6 +3851,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -4083,35 +3916,6 @@
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="18" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>

</xml_diff>

<commit_message>
Epicas finales, priorizacion por valor, tallas y sprints; drivers, ADR y stack tecnico
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -8,13 +8,13 @@
   <sheets>
     <sheet name="Mapa de Impacto" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Entregables" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Backlog - Historias de Usuario" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Traduccion de mensajes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Config. de conversacion" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Historial" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Planificacion" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog - Historias de Usuario" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Traduccion de mensajes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gestion de conversaciones" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Cuenta de usuario" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Participacion interlocutor" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Reportes de calidad" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Reportes" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Admin idiomas y regiones" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,8 +104,15 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -150,8 +157,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0092D050"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="28">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -504,11 +516,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -656,6 +682,30 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1173,7 +1223,7 @@
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="G5" s="32" t="n"/>
@@ -1198,7 +1248,7 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="G6" s="32" t="n"/>
@@ -1223,7 +1273,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Historial de conversaciones</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="G7" s="32" t="n"/>
@@ -1302,7 +1352,7 @@
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Reportes de calidad</t>
+          <t>Reportes</t>
         </is>
       </c>
       <c r="G10" s="32" t="n"/>
@@ -1393,7 +1443,7 @@
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
-          <t>Reportes de calidad</t>
+          <t>Reportes</t>
         </is>
       </c>
       <c r="G13" s="32" t="n"/>
@@ -1427,7 +1477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1455,22 +1505,21 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
+          <t>Cliente Traductor / Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4"/>
+        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C12</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -1478,7 +1527,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -1503,46 +1551,92 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C25</f>
+        <f>Entregables!C24</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D25</f>
+        <f>Entregables!D24</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E25</f>
+        <f>Entregables!E24</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F25</f>
+        <f>Entregables!F24</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
+        <f>Entregables!C25</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D25</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E25</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18">
         <f>Entregables!C26</f>
         <v/>
       </c>
-      <c r="B9" s="18">
+      <c r="B10" s="18">
         <f>Entregables!D26</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C10" s="18">
         <f>Entregables!E26</f>
         <v/>
       </c>
-      <c r="D9" s="18">
+      <c r="D10" s="18">
         <f>Entregables!F26</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="41.5" customHeight="1">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -1557,7 +1651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1566,6 +1660,11 @@
     <col width="14.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="22.1640625" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="162.1640625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1599,6 +1698,31 @@
           <t>Para</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Prioridad (valor)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Por que genera valor</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="33" t="inlineStr">
@@ -1628,6 +1752,26 @@
       <c r="F2">
         <f>'Mapa de Impacto'!C4</f>
         <v/>
+      </c>
+      <c r="G2" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" s="57" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I2" s="57">
+        <f>VLOOKUP(H2,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J2" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="58" t="inlineStr">
+        <is>
+          <t>Es la forma natural de usar el producto: hablar y ser entendido sin escribir.</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
@@ -1655,6 +1799,26 @@
         <f>'Mapa de Impacto'!C4</f>
         <v/>
       </c>
+      <c r="G3" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I3" s="57">
+        <f>VLOOKUP(H3,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J3" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="58" t="inlineStr">
+        <is>
+          <t>Es la entrada mas simple y la que permite usar la traduccion desde el primer dia.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="34" t="n"/>
@@ -1681,6 +1845,26 @@
         <f>'Mapa de Impacto'!C4</f>
         <v/>
       </c>
+      <c r="G4" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="57" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="I4" s="57">
+        <f>VLOOKUP(H4,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J4" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="58" t="inlineStr">
+        <is>
+          <t>Es el corazon del producto: sin esto TalkLate no entrega su valor diferencial.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="34" t="n"/>
@@ -1707,6 +1891,26 @@
         <f>'Mapa de Impacto'!C9</f>
         <v/>
       </c>
+      <c r="G5" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I5" s="57">
+        <f>VLOOKUP(H5,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J5" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="58" t="inlineStr">
+        <is>
+          <t>Permite que la otra persona reciba el mensaje de forma comoda y natural.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="35" t="n"/>
@@ -1733,11 +1937,31 @@
         <f>'Mapa de Impacto'!C9</f>
         <v/>
       </c>
+      <c r="G6" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I6" s="57">
+        <f>VLOOKUP(H6,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J6" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="58" t="inlineStr">
+        <is>
+          <t>Mantiene la experiencia coherente: si hablo, escucho; si escribo, leo.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="33" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B7" s="33" t="inlineStr">
@@ -1762,6 +1986,26 @@
       <c r="F7">
         <f>'Mapa de Impacto'!C5</f>
         <v/>
+      </c>
+      <c r="G7" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I7" s="57">
+        <f>VLOOKUP(H7,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J7" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="58" t="inlineStr">
+        <is>
+          <t>Define a que persona y lugar se adapta el mensaje: de ahi sale el matiz cultural.</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
@@ -1789,6 +2033,26 @@
         <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
+      <c r="G8" s="57" t="n">
+        <v>7</v>
+      </c>
+      <c r="H8" s="57" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I8" s="57">
+        <f>VLOOKUP(H8,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J8" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="58" t="inlineStr">
+        <is>
+          <t>Evita configurar a mano el idioma cada vez y acelera la conversacion.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="34" t="n"/>
@@ -1799,7 +2063,7 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Consultar los idiomas disponibles</t>
+          <t>Crear una conversacion</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1812,8 +2076,28 @@
         <v/>
       </c>
       <c r="F9">
-        <f>'Mapa de Impacto'!C5</f>
-        <v/>
+        <f>'Mapa de Impacto'!C6</f>
+        <v/>
+      </c>
+      <c r="G9" s="57" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I9" s="57">
+        <f>VLOOKUP(H9,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J9" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="58" t="inlineStr">
+        <is>
+          <t>Agrupa los mensajes de una misma charla para no perder el contexto.</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
@@ -1825,7 +2109,7 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Crear una conversacion</t>
+          <t>Configurar los parametros una sola vez</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1840,6 +2124,26 @@
       <c r="F10">
         <f>'Mapa de Impacto'!C6</f>
         <v/>
+      </c>
+      <c r="G10" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I10" s="57">
+        <f>VLOOKUP(H10,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J10" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="58" t="inlineStr">
+        <is>
+          <t>Ahorra repetir la configuracion en cada mensaje.</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
@@ -1851,7 +2155,7 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Configurar los parametros una sola vez</t>
+          <t>Mantener el hilo continuo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1867,9 +2171,29 @@
         <f>'Mapa de Impacto'!C6</f>
         <v/>
       </c>
+      <c r="G11" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I11" s="57">
+        <f>VLOOKUP(H11,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J11" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" s="58" t="inlineStr">
+        <is>
+          <t>Hace posible un dialogo fluido, que es lo que busca el usuario.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="35" t="n"/>
+      <c r="A12" s="34" t="n"/>
       <c r="B12" s="33" t="inlineStr">
         <is>
           <t>HU0011</t>
@@ -1877,7 +2201,7 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Mantener el hilo continuo</t>
+          <t>Consultar mi historial</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1890,16 +2214,32 @@
         <v/>
       </c>
       <c r="F12">
-        <f>'Mapa de Impacto'!C6</f>
-        <v/>
+        <f>'Mapa de Impacto'!C7</f>
+        <v/>
+      </c>
+      <c r="G12" s="57" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I12" s="57">
+        <f>VLOOKUP(H12,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J12" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="58" t="inlineStr">
+        <is>
+          <t>Permite repasar y aprender de conversaciones pasadas.</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>Historial de conversaciones</t>
-        </is>
-      </c>
+      <c r="A13" s="34" t="n"/>
       <c r="B13" s="33" t="inlineStr">
         <is>
           <t>HU0012</t>
@@ -1907,7 +2247,7 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Consultar mi historial</t>
+          <t>Abrir una conversacion anterior</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1922,6 +2262,26 @@
       <c r="F13">
         <f>'Mapa de Impacto'!C7</f>
         <v/>
+      </c>
+      <c r="G13" s="57" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" s="57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I13" s="57">
+        <f>VLOOKUP(H13,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J13" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="58" t="inlineStr">
+        <is>
+          <t>Permite retomar una conversacion donde se dejo.</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
@@ -1933,7 +2293,7 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Abrir una conversacion anterior</t>
+          <t>Renombrar una conversacion</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1949,9 +2309,29 @@
         <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
+      <c r="G14" s="57" t="n">
+        <v>19</v>
+      </c>
+      <c r="H14" s="57" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I14" s="57">
+        <f>VLOOKUP(H14,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J14" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="58" t="inlineStr">
+        <is>
+          <t>Ayuda a ubicar conversaciones, pero no cambia el valor central.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="34" t="n"/>
+      <c r="A15" s="35" t="n"/>
       <c r="B15" s="33" t="inlineStr">
         <is>
           <t>HU0014</t>
@@ -1959,7 +2339,7 @@
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>Renombrar una conversacion</t>
+          <t>Eliminar una conversacion</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1975,9 +2355,33 @@
         <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
+      <c r="G15" s="57" t="n">
+        <v>20</v>
+      </c>
+      <c r="H15" s="57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I15" s="57">
+        <f>VLOOKUP(H15,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J15" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="58" t="inlineStr">
+        <is>
+          <t>Da control sobre los datos propios; es de apoyo.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="35" t="n"/>
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
       <c r="B16" s="33" t="inlineStr">
         <is>
           <t>HU0015</t>
@@ -1985,7 +2389,7 @@
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Eliminar una conversacion</t>
+          <t>Registrarme en la aplicacion</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1998,16 +2402,32 @@
         <v/>
       </c>
       <c r="F16">
-        <f>'Mapa de Impacto'!C7</f>
-        <v/>
+        <f>'Mapa de Impacto'!C8</f>
+        <v/>
+      </c>
+      <c r="G16" s="57" t="n">
+        <v>16</v>
+      </c>
+      <c r="H16" s="57" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I16" s="57">
+        <f>VLOOKUP(H16,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J16" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="58" t="inlineStr">
+        <is>
+          <t>Guarda las conversaciones del usuario y protege sus datos; el valor central no depende de esto.</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
+      <c r="A17" s="34" t="n"/>
       <c r="B17" s="33" t="inlineStr">
         <is>
           <t>HU0016</t>
@@ -2015,7 +2435,7 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Registrarme en la aplicacion</t>
+          <t>Iniciar sesion</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2030,6 +2450,26 @@
       <c r="F17">
         <f>'Mapa de Impacto'!C8</f>
         <v/>
+      </c>
+      <c r="G17" s="57" t="n">
+        <v>17</v>
+      </c>
+      <c r="H17" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I17" s="57">
+        <f>VLOOKUP(H17,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J17" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" s="58" t="inlineStr">
+        <is>
+          <t>Da acceso seguro a lo guardado.</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
@@ -2041,7 +2481,7 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Iniciar sesion</t>
+          <t>Recuperar mi contrasena</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2057,9 +2497,29 @@
         <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
+      <c r="G18" s="57" t="n">
+        <v>21</v>
+      </c>
+      <c r="H18" s="57" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I18" s="57">
+        <f>VLOOKUP(H18,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J18" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="58" t="inlineStr">
+        <is>
+          <t>Evita perder la cuenta; es de apoyo.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="34" t="n"/>
+      <c r="A19" s="35" t="n"/>
       <c r="B19" s="33" t="inlineStr">
         <is>
           <t>HU0018</t>
@@ -2067,7 +2527,7 @@
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>Recuperar mi contrasena</t>
+          <t>Cerrar sesion</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2083,9 +2543,33 @@
         <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
+      <c r="G19" s="57" t="n">
+        <v>22</v>
+      </c>
+      <c r="H19" s="57" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I19" s="57">
+        <f>VLOOKUP(H19,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J19" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="58" t="inlineStr">
+        <is>
+          <t>Protege la cuenta en un dispositivo compartido; es de apoyo.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="35" t="n"/>
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>Participacion del interlocutor</t>
+        </is>
+      </c>
       <c r="B20" s="33" t="inlineStr">
         <is>
           <t>HU0019</t>
@@ -2093,12 +2577,12 @@
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Cerrar sesion</t>
+          <t>Recibir el mensaje traducido</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Cliente Traductor</t>
+          <t>Interlocutor</t>
         </is>
       </c>
       <c r="E20">
@@ -2106,16 +2590,32 @@
         <v/>
       </c>
       <c r="F20">
-        <f>'Mapa de Impacto'!C8</f>
-        <v/>
+        <f>'Mapa de Impacto'!C11</f>
+        <v/>
+      </c>
+      <c r="G20" s="57" t="n">
+        <v>11</v>
+      </c>
+      <c r="H20" s="57" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I20" s="57">
+        <f>VLOOKUP(H20,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J20" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="58" t="inlineStr">
+        <is>
+          <t>Hace que la otra persona participe sin instalar ni operar la app.</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>Participacion del interlocutor</t>
-        </is>
-      </c>
+      <c r="A21" s="35" t="n"/>
       <c r="B21" s="33" t="inlineStr">
         <is>
           <t>HU0020</t>
@@ -2123,7 +2623,7 @@
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Recibir el mensaje traducido</t>
+          <t>Responder en mi idioma</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2139,9 +2639,33 @@
         <f>'Mapa de Impacto'!C11</f>
         <v/>
       </c>
+      <c r="G21" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I21" s="57">
+        <f>VLOOKUP(H21,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J21" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="58" t="inlineStr">
+        <is>
+          <t>Cierra el dialogo en ambos sentidos.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="35" t="n"/>
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
       <c r="B22" s="33" t="inlineStr">
         <is>
           <t>HU0021</t>
@@ -2149,12 +2673,12 @@
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Responder en mi idioma</t>
+          <t>Reportar una mala traduccion</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Interlocutor</t>
+          <t>Cliente Traductor</t>
         </is>
       </c>
       <c r="E22">
@@ -2162,16 +2686,32 @@
         <v/>
       </c>
       <c r="F22">
-        <f>'Mapa de Impacto'!C11</f>
-        <v/>
+        <f>'Mapa de Impacto'!C10</f>
+        <v/>
+      </c>
+      <c r="G22" s="57" t="n">
+        <v>18</v>
+      </c>
+      <c r="H22" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I22" s="57">
+        <f>VLOOKUP(H22,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J22" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K22" s="58" t="inlineStr">
+        <is>
+          <t>Alimenta la mejora de calidad con casos reales.</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>Reportes de calidad</t>
-        </is>
-      </c>
+      <c r="A23" s="35" t="n"/>
       <c r="B23" s="33" t="inlineStr">
         <is>
           <t>HU0022</t>
@@ -2179,12 +2719,12 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Reportar una mala traduccion</t>
+          <t>Revisar los reportes de mala traduccion</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Cliente Traductor</t>
+          <t>Administrador</t>
         </is>
       </c>
       <c r="E23">
@@ -2192,12 +2732,36 @@
         <v/>
       </c>
       <c r="F23">
-        <f>'Mapa de Impacto'!C10</f>
-        <v/>
+        <f>'Mapa de Impacto'!C13</f>
+        <v/>
+      </c>
+      <c r="G23" s="57" t="n">
+        <v>23</v>
+      </c>
+      <c r="H23" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I23" s="57">
+        <f>VLOOKUP(H23,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J23" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" s="58" t="inlineStr">
+        <is>
+          <t>Permite priorizar que mejorar primero.</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="35" t="n"/>
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
       <c r="B24" s="33" t="inlineStr">
         <is>
           <t>HU0023</t>
@@ -2205,12 +2769,12 @@
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Revisar los reportes de mala traduccion</t>
+          <t>Consultar los idiomas disponibles</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Administrador</t>
+          <t>Cliente Traductor</t>
         </is>
       </c>
       <c r="E24">
@@ -2218,16 +2782,32 @@
         <v/>
       </c>
       <c r="F24">
-        <f>'Mapa de Impacto'!C13</f>
-        <v/>
+        <f>'Mapa de Impacto'!C5</f>
+        <v/>
+      </c>
+      <c r="G24" s="57" t="n">
+        <v>13</v>
+      </c>
+      <c r="H24" s="57" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I24" s="57">
+        <f>VLOOKUP(H24,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J24" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="58" t="inlineStr">
+        <is>
+          <t>Muestra con que idiomas se puede hablar antes de empezar.</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="33" t="inlineStr">
-        <is>
-          <t>Administracion de idiomas y regiones</t>
-        </is>
-      </c>
+      <c r="A25" s="34" t="n"/>
       <c r="B25" s="33" t="inlineStr">
         <is>
           <t>HU0024</t>
@@ -2250,6 +2830,26 @@
       <c r="F25">
         <f>'Mapa de Impacto'!C12</f>
         <v/>
+      </c>
+      <c r="G25" s="57" t="n">
+        <v>24</v>
+      </c>
+      <c r="H25" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I25" s="57">
+        <f>VLOOKUP(H25,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J25" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K25" s="58" t="inlineStr">
+        <is>
+          <t>Hace crecer el servicio a mas personas.</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -2277,28 +2877,378 @@
         <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
-    </row>
+      <c r="G26" s="57" t="n">
+        <v>25</v>
+      </c>
+      <c r="H26" s="57" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I26" s="57">
+        <f>VLOOKUP(H26,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J26" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="58" t="inlineStr">
+        <is>
+          <t>Controla que idiomas se ofrecen con calidad suficiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A17:A20"/>
+  <mergeCells count="6">
+    <mergeCell ref="A22:A23"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A7:A12"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A7:A15"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A16:A19"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" location="'Traductor de mensajes'!A1" display="Traductor de mensajes"/>
-    <hyperlink ref="A13" location="'Gestión de perfil'!A1" display="Gestión de perfil de usuario"/>
-    <hyperlink ref="A17" location="'Audio traducido'!A1" display="Reproducción y personalización de audio traducido"/>
-    <hyperlink ref="A23" location="'Reportes calidad (Admin)'!A1" display="Revisión de reportes de calidad de traducción"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>Tallas y horas estimadas (una persona desarrolla)</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Capacidad de un sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Dias del sprint</t>
+        </is>
+      </c>
+      <c r="E3" s="62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="61" t="inlineStr">
+        <is>
+          <t>Horas por dia y por persona</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="62" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B5" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="E5" s="62" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="62" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B6" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="61" t="inlineStr">
+        <is>
+          <t>Horas brutas por sprint</t>
+        </is>
+      </c>
+      <c r="E6" s="62">
+        <f>E3*E4*E5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="62" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B7" s="62" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Porcentaje usable (el resto es planeacion, dailies, refinamiento y retrospectiva)</t>
+        </is>
+      </c>
+      <c r="E7" s="63" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="B8" s="62" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="61" t="inlineStr">
+        <is>
+          <t>Horas disponibles por sprint</t>
+        </is>
+      </c>
+      <c r="E8" s="62">
+        <f>E6*E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="62" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="B9" s="62" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="59" t="inlineStr">
+        <is>
+          <t>Plan por sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="60" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>Horas planeadas</t>
+        </is>
+      </c>
+      <c r="C13" s="60" t="inlineStr">
+        <is>
+          <t>Horas disponibles</t>
+        </is>
+      </c>
+      <c r="D13" s="60" t="inlineStr">
+        <is>
+          <t>Diferencia</t>
+        </is>
+      </c>
+      <c r="E13" s="60" t="inlineStr">
+        <is>
+          <t>Historias</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="64">
+        <f>SUMIF(Entregables!$J$2:$J$40,A14,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="C14" s="64">
+        <f>$E$8</f>
+        <v/>
+      </c>
+      <c r="D14" s="64">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="65" t="inlineStr">
+        <is>
+          <t>HU0001, HU0002, HU0003, HU0004, HU0005, HU0006</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="64">
+        <f>SUMIF(Entregables!$J$2:$J$40,A15,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="C15" s="64">
+        <f>$E$8</f>
+        <v/>
+      </c>
+      <c r="D15" s="64">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="65" t="inlineStr">
+        <is>
+          <t>HU0007, HU0008, HU0009, HU0010, HU0011, HU0012, HU0013, HU0018, HU0019, HU0020, HU0023, HU0025</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="64" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="64">
+        <f>SUMIF(Entregables!$J$2:$J$40,A16,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="C16" s="64">
+        <f>$E$8</f>
+        <v/>
+      </c>
+      <c r="D16" s="64">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="65" t="inlineStr">
+        <is>
+          <t>HU0014, HU0015, HU0016, HU0017, HU0021, HU0022, HU0024</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="66" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B17" s="66">
+        <f>SUM(B14:B16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="66" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>La prioridad va por valor para el negocio (no por dependencia): lo que mas valor genera es traducir; registrarse y cerrar sesion son de apoyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Se llenan los sprints de mayor a menor valor hasta quedar cerca de las horas disponibles; si sobra espacio se acomoda una historia pequena de mas abajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Las horas por talla son una estimacion; se pueden ajustar y las formulas recalculan los sprints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Metodologico: el plan de liberaciones se arma con estos sprints.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2394,7 +3344,7 @@
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
@@ -2421,7 +3371,7 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -2444,7 +3394,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -2467,7 +3417,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -2494,7 +3444,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -2517,7 +3467,7 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Configuracion de conversacion</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2540,7 +3490,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Historial de conversaciones</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -2567,7 +3517,7 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Historial de conversaciones</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -2590,7 +3540,7 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Historial de conversaciones</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -2613,7 +3563,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Historial de conversaciones</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -2828,7 +3778,7 @@
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Reportes de calidad</t>
+          <t>Reportes</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -2932,7 +3882,7 @@
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Reportes de calidad</t>
+          <t>Reportes</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
@@ -2970,13 +3920,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3019,7 +3969,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3027,7 +3976,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3140,202 +4088,33 @@
         <v/>
       </c>
     </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Configuracion de conversacion</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="18">
-        <f>Entregables!C7</f>
-        <v/>
-      </c>
-      <c r="B8" s="18">
-        <f>Entregables!D7</f>
-        <v/>
-      </c>
-      <c r="C8" s="18">
-        <f>Entregables!E7</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>Entregables!F7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="18">
-        <f>Entregables!C8</f>
-        <v/>
-      </c>
-      <c r="B9" s="18">
-        <f>Entregables!D8</f>
-        <v/>
-      </c>
-      <c r="C9" s="18">
-        <f>Entregables!E8</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>Entregables!F8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18">
-        <f>Entregables!C9</f>
-        <v/>
-      </c>
-      <c r="B10" s="18">
-        <f>Entregables!D9</f>
-        <v/>
-      </c>
-      <c r="C10" s="18">
-        <f>Entregables!E9</f>
-        <v/>
-      </c>
-      <c r="D10" s="18">
-        <f>Entregables!F9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="18">
-        <f>Entregables!C10</f>
-        <v/>
-      </c>
-      <c r="B11" s="18">
-        <f>Entregables!D10</f>
-        <v/>
-      </c>
-      <c r="C11" s="18">
-        <f>Entregables!E10</f>
-        <v/>
-      </c>
-      <c r="D11" s="18">
-        <f>Entregables!F10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="18">
-        <f>Entregables!C11</f>
-        <v/>
-      </c>
-      <c r="B12" s="18">
-        <f>Entregables!D11</f>
-        <v/>
-      </c>
-      <c r="C12" s="18">
-        <f>Entregables!E11</f>
-        <v/>
-      </c>
-      <c r="D12" s="18">
-        <f>Entregables!F11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="18">
-        <f>Entregables!C12</f>
-        <v/>
-      </c>
-      <c r="B13" s="18">
-        <f>Entregables!D12</f>
-        <v/>
-      </c>
-      <c r="C13" s="18">
-        <f>Entregables!E12</f>
-        <v/>
-      </c>
-      <c r="D13" s="18">
-        <f>Entregables!F12</f>
-        <v/>
-      </c>
-    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3350,7 +4129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3366,7 +4145,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Historial de conversaciones</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
     </row>
@@ -3382,18 +4161,17 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1">
+    <row r="3" ht="135" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4"/>
+        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C6&amp;CHAR(10)&amp;'Mapa de Impacto'!C7</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3401,7 +4179,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3426,76 +4203,189 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C13</f>
+        <f>Entregables!C7</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D13</f>
+        <f>Entregables!D7</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E13</f>
+        <f>Entregables!E7</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F13</f>
+        <f>Entregables!F7</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C14</f>
+        <f>Entregables!C8</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D14</f>
+        <f>Entregables!D8</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E14</f>
+        <f>Entregables!E8</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F14</f>
+        <f>Entregables!F8</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18">
-        <f>Entregables!C15</f>
+        <f>Entregables!C9</f>
         <v/>
       </c>
       <c r="B10" s="18">
-        <f>Entregables!D15</f>
+        <f>Entregables!D9</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>Entregables!E15</f>
+        <f>Entregables!E9</f>
         <v/>
       </c>
       <c r="D10" s="18">
-        <f>Entregables!F15</f>
+        <f>Entregables!F9</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="18">
-        <f>Entregables!C16</f>
+        <f>Entregables!C10</f>
         <v/>
       </c>
       <c r="B11" s="18">
-        <f>Entregables!D16</f>
+        <f>Entregables!D10</f>
         <v/>
       </c>
       <c r="C11" s="18">
-        <f>Entregables!E16</f>
+        <f>Entregables!E10</f>
         <v/>
       </c>
       <c r="D11" s="18">
-        <f>Entregables!F16</f>
-        <v/>
-      </c>
-    </row>
+        <f>Entregables!F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="18">
+        <f>Entregables!C11</f>
+        <v/>
+      </c>
+      <c r="B12" s="18">
+        <f>Entregables!D11</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>Entregables!E11</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
+        <f>Entregables!F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="18">
+        <f>Entregables!C12</f>
+        <v/>
+      </c>
+      <c r="B13" s="18">
+        <f>Entregables!D12</f>
+        <v/>
+      </c>
+      <c r="C13" s="18">
+        <f>Entregables!E12</f>
+        <v/>
+      </c>
+      <c r="D13" s="18">
+        <f>Entregables!F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="18">
+        <f>Entregables!C13</f>
+        <v/>
+      </c>
+      <c r="B14" s="18">
+        <f>Entregables!D13</f>
+        <v/>
+      </c>
+      <c r="C14" s="18">
+        <f>Entregables!E13</f>
+        <v/>
+      </c>
+      <c r="D14" s="18">
+        <f>Entregables!F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="18">
+        <f>Entregables!C14</f>
+        <v/>
+      </c>
+      <c r="B15" s="18">
+        <f>Entregables!D14</f>
+        <v/>
+      </c>
+      <c r="C15" s="18">
+        <f>Entregables!E14</f>
+        <v/>
+      </c>
+      <c r="D15" s="18">
+        <f>Entregables!F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="18">
+        <f>Entregables!C15</f>
+        <v/>
+      </c>
+      <c r="B16" s="18">
+        <f>Entregables!D15</f>
+        <v/>
+      </c>
+      <c r="C16" s="18">
+        <f>Entregables!E15</f>
+        <v/>
+      </c>
+      <c r="D16" s="18">
+        <f>Entregables!F15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3510,7 +4400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3553,7 +4443,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3561,7 +4450,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3586,76 +4474,104 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C17</f>
+        <f>Entregables!C16</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D17</f>
+        <f>Entregables!D16</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E17</f>
+        <f>Entregables!E16</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F17</f>
+        <f>Entregables!F16</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C18</f>
+        <f>Entregables!C17</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D18</f>
+        <f>Entregables!D17</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E18</f>
+        <f>Entregables!E17</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F18</f>
+        <f>Entregables!F17</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18">
-        <f>Entregables!C19</f>
+        <f>Entregables!C18</f>
         <v/>
       </c>
       <c r="B10" s="18">
-        <f>Entregables!D19</f>
+        <f>Entregables!D18</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>Entregables!E19</f>
+        <f>Entregables!E18</f>
         <v/>
       </c>
       <c r="D10" s="18">
-        <f>Entregables!F19</f>
+        <f>Entregables!F18</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="18">
-        <f>Entregables!C20</f>
+        <f>Entregables!C19</f>
         <v/>
       </c>
       <c r="B11" s="18">
-        <f>Entregables!D20</f>
+        <f>Entregables!D19</f>
         <v/>
       </c>
       <c r="C11" s="18">
-        <f>Entregables!E20</f>
+        <f>Entregables!E19</f>
         <v/>
       </c>
       <c r="D11" s="18">
-        <f>Entregables!F20</f>
-        <v/>
-      </c>
-    </row>
+        <f>Entregables!F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3670,7 +4586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3713,7 +4629,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3721,7 +4636,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3746,46 +4660,80 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C21</f>
+        <f>Entregables!C20</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D21</f>
+        <f>Entregables!D20</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E21</f>
+        <f>Entregables!E20</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F21</f>
+        <f>Entregables!F20</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C22</f>
+        <f>Entregables!C21</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D22</f>
+        <f>Entregables!D21</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E22</f>
+        <f>Entregables!E21</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="41.5" customHeight="1">
+        <f>Entregables!F21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18" t="n"/>
       <c r="B10" s="18" t="n"/>
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="18" t="n"/>
     </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3800,7 +4748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3816,7 +4764,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Reportes de calidad</t>
+          <t>Reportes</t>
         </is>
       </c>
     </row>
@@ -3843,7 +4791,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3851,7 +4798,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3876,46 +4822,80 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C23</f>
+        <f>Entregables!C22</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D23</f>
+        <f>Entregables!D22</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E23</f>
+        <f>Entregables!E22</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F23</f>
+        <f>Entregables!F22</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C24</f>
+        <f>Entregables!C23</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D24</f>
+        <f>Entregables!D23</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E24</f>
+        <f>Entregables!E23</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="41.5" customHeight="1">
+        <f>Entregables!F23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18" t="n"/>
       <c r="B10" s="18" t="n"/>
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="18" t="n"/>
     </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>

</xml_diff>

<commit_message>
Limpieza de archivos sin uso, administrador con correo del equipo, ADR como tomadas y lista para validar en la reunion
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -9,13 +9,12 @@
     <sheet name="Mapa de Impacto" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Entregables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Planificacion" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog - Historias de Usuario" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Traduccion de mensajes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gestion de conversaciones" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cuenta de usuario" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Participacion interlocutor" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Reportes" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Admin idiomas y regiones" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Traduccion de mensajes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gestion de conversaciones" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cuenta de usuario" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Participacion interlocutor" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Reportes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Admin idiomas y regiones" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1471,187 +1470,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Administracion de idiomas y regiones</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor / Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="18">
-        <f>Entregables!C24</f>
-        <v/>
-      </c>
-      <c r="B8" s="18">
-        <f>Entregables!D24</f>
-        <v/>
-      </c>
-      <c r="C8" s="18">
-        <f>Entregables!E24</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>Entregables!F24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="18">
-        <f>Entregables!C25</f>
-        <v/>
-      </c>
-      <c r="B9" s="18">
-        <f>Entregables!D25</f>
-        <v/>
-      </c>
-      <c r="C9" s="18">
-        <f>Entregables!E25</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>Entregables!F25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18">
-        <f>Entregables!C26</f>
-        <v/>
-      </c>
-      <c r="B10" s="18">
-        <f>Entregables!D26</f>
-        <v/>
-      </c>
-      <c r="C10" s="18">
-        <f>Entregables!E26</f>
-        <v/>
-      </c>
-      <c r="D10" s="18">
-        <f>Entregables!F26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="18" t="n"/>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2898,39 +2723,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A22:A23"/>
@@ -2975,6 +2767,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="60" t="inlineStr">
         <is>
@@ -3097,6 +2890,8 @@
         <v>12</v>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="59" t="inlineStr">
         <is>
@@ -3208,6 +3003,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="66" t="inlineStr">
         <is>
@@ -3254,668 +3050,174 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="2" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Entregable</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Cliente Traductor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Impacto (para)</t>
+        </is>
+      </c>
+      <c r="B3" s="18">
+        <f>'Mapa de Impacto'!C4&amp;CHAR(10)&amp;'Mapa de Impacto'!C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>← Volver al Mapa de Impacto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Característica</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Como</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>Necesito</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>Para</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Traduccion de mensajes</t>
-        </is>
-      </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Recibir entrada del mensaje</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>decir (hablar) el mensaje que quiero traducir</t>
-        </is>
-      </c>
-      <c r="E2" s="42" t="inlineStr">
-        <is>
-          <t>Traducir un mensaje de un idioma origen a un idioma destino en tiempo real, para comunicarme fácil y rápidamente con personas que hablan otro idioma conservando el contexto cultural, el tono y los modismos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Traduccion de mensajes</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Recibir entrada del mensaje</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>escribir el mensaje que quiero traducir</t>
-        </is>
-      </c>
-      <c r="E3" s="38" t="n"/>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Seleccionar idioma y región destino</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>elegir el idioma y la región a los que quiero traducir</t>
-        </is>
-      </c>
-      <c r="E4" s="42" t="inlineStr">
-        <is>
-          <t>Definir y conocer los idiomas y regiones con los que me quiero comunicar, para dejar claro desde el inicio qué idioma hablo y a qué idioma/región necesito traducir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Reconocer el idioma origen</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>empezar a hablar sin tener que indicar manualmente mi idioma de origen, reconociéndolo desde mi primer mensaje de voz (Conversacion-RN-2)</t>
-        </is>
-      </c>
-      <c r="E5" s="37" t="n"/>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Administracion de idiomas y regiones</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Consultar idiomas disponibles</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>ver la lista de idiomas y regiones que TalkLate soporta antes de configurar la conversación</t>
-        </is>
-      </c>
-      <c r="E6" s="38" t="n"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Crear conversación</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>iniciar una nueva conversación con otra persona</t>
-        </is>
-      </c>
-      <c r="E7" s="42" t="inlineStr">
-        <is>
-          <t>Configurar una conversación una sola vez y mantener su hilo continuo, para conversar de forma fluida y organizada sin reconfigurar nada en cada mensaje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Configurar parámetros una sola vez</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>definir el idioma y la región destino una única vez al crear la conversación (Conversacion-RN-1)</t>
-        </is>
-      </c>
-      <c r="E8" s="37" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Mantener el hilo continuo</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>que cada mensaje que envío o recibo dentro de esa conversación se traduzca automáticamente sin volver a configurar nada</t>
-        </is>
-      </c>
-      <c r="E9" s="38" t="n"/>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>Consultar historial</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>ver la lista de mis conversaciones anteriores</t>
-        </is>
-      </c>
-      <c r="E10" s="42" t="inlineStr">
-        <is>
-          <t>Consultar, organizar y reaprovechar mis conversaciones anteriores, para tener un historial ordenado que me sirva de recurso de aprendizaje y referencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Abrir una conversación</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>abrir una conversación anterior y ver sus mensajes originales y traducidos</t>
-        </is>
-      </c>
-      <c r="E11" s="37" t="n"/>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>Renombrar conversación</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>cambiar el nombre de una conversación para identificarla fácilmente</t>
-        </is>
-      </c>
-      <c r="E12" s="37" t="n"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Gestion de conversaciones</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Eliminar conversación</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>eliminar una conversación que ya no necesito</t>
-        </is>
-      </c>
-      <c r="E13" s="38" t="n"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>Registro de cuenta</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>registrarme con mi nombre, apellido, correo y contraseña</t>
-        </is>
-      </c>
-      <c r="E14" s="42" t="inlineStr">
-        <is>
-          <t>Crear y administrar mi perfil de forma sencilla y segura, para acceder con mi identidad protegida a mis configuraciones y conversaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Registro de cuenta</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>registrarme indicando mi fecha de nacimiento y que solo se permita el registro si tengo al menos 13 años (Usuario-RN-2)</t>
-        </is>
-      </c>
-      <c r="E15" s="37" t="n"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Inicio de sesión</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>iniciar sesión con mi correo y contraseña</t>
-        </is>
-      </c>
-      <c r="E16" s="37" t="n"/>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Recuperación de contraseña</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>solicitar un código de recuperación a mi correo cuando olvide mi contraseña</t>
-        </is>
-      </c>
-      <c r="E17" s="37" t="n"/>
-    </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>Recuperación de contraseña</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>definir una nueva contraseña usando el código de recuperación recibido</t>
-        </is>
-      </c>
-      <c r="E18" s="37" t="n"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Cierre de sesión</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>cerrar mi sesión activa cuando termine de usar la app</t>
-        </is>
-      </c>
-      <c r="E19" s="38" t="n"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Traduccion de mensajes</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>Reproducir audio traducido</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>escuchar el mensaje traducido en un audio claro y natural</t>
-        </is>
-      </c>
-      <c r="E20" s="42" t="inlineStr">
-        <is>
-          <t>Escuchar y entregar el mensaje traducido en el mismo canal (voz o texto) de forma clara y natural, para que mi interlocutor lo reciba de forma cómoda y comprensible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Traduccion de mensajes</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Entregar por el mismo canal</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>recibir el mensaje traducido en el mismo formato que usé para enviarlo (audio si hablé, texto si escribí)</t>
-        </is>
-      </c>
-      <c r="E21" s="38" t="n"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Reportes</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>Reportar mala traducción</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>reportar cuando una traducción no fue correcta o natural</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>Reportar cuando una traducción no fue correcta o natural, para contribuir a que la calidad del servicio mejore con el tiempo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Participacion del interlocutor</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Recibir mensaje traducido</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>escuchar o leer en mi propio idioma el mensaje que me enviaron</t>
-        </is>
-      </c>
-      <c r="E23" s="42" t="inlineStr">
-        <is>
-          <t>Recibir en mi propio idioma los mensajes que me envían y responder en el mío, para participar en la conversación de forma natural aunque no comparta el idioma de la otra persona.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Participacion del interlocutor</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>Responder en mi idioma</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>responder hablando o escribiendo en mi propio idioma para que la otra persona lo reciba traducido</t>
-        </is>
-      </c>
-      <c r="E24" s="38" t="n"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Administracion de idiomas y regiones</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>Gestionar catálogo de idiomas</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>agregar, activar o desactivar los idiomas, regiones y acentos disponibles</t>
-        </is>
-      </c>
-      <c r="E25" s="42" t="inlineStr">
-        <is>
-          <t>Gestionar el catálogo de idiomas, regiones y acentos soportados por la aplicación, para mantener actualizada y disponible la oferta de idiomas del servicio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Reportes</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>Revisar reportes de mala traducción</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>Administrador</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>revisar los reportes de mala traducción enviados por los clientes para priorizar mejoras</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Revisar los reportes de mala traducción enviados por los clientes, para priorizar las mejoras y la evolución de la calidad del servicio.</t>
-        </is>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C2</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D2</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E2</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C3</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D3</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E3</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18">
+        <f>Entregables!C4</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D4</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E4</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18">
+        <f>Entregables!C5</f>
+        <v/>
+      </c>
+      <c r="B11" s="18">
+        <f>Entregables!D5</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>Entregables!E5</f>
+        <v/>
+      </c>
+      <c r="D11" s="18">
+        <f>Entregables!F5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="18">
+        <f>Entregables!C6</f>
+        <v/>
+      </c>
+      <c r="B12" s="18">
+        <f>Entregables!D6</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>Entregables!E6</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
+        <f>Entregables!F6</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E14:E19"/>
-    <mergeCell ref="E10:E13"/>
-  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3926,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3942,7 +3244,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Traduccion de mensajes</t>
+          <t>Gestion de conversaciones</t>
         </is>
       </c>
     </row>
@@ -3958,17 +3260,18 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="90" customHeight="1">
+    <row r="3" ht="135" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C4&amp;CHAR(10)&amp;'Mapa de Impacto'!C9</f>
-        <v/>
-      </c>
-    </row>
+        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C6&amp;CHAR(10)&amp;'Mapa de Impacto'!C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3976,6 +3279,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -4000,121 +3304,166 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C2</f>
+        <f>Entregables!C7</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D2</f>
+        <f>Entregables!D7</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E2</f>
+        <f>Entregables!E7</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F2</f>
+        <f>Entregables!F7</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C3</f>
+        <f>Entregables!C8</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D3</f>
+        <f>Entregables!D8</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E3</f>
+        <f>Entregables!E8</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F3</f>
+        <f>Entregables!F8</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18">
-        <f>Entregables!C4</f>
+        <f>Entregables!C9</f>
         <v/>
       </c>
       <c r="B10" s="18">
-        <f>Entregables!D4</f>
+        <f>Entregables!D9</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>Entregables!E4</f>
+        <f>Entregables!E9</f>
         <v/>
       </c>
       <c r="D10" s="18">
-        <f>Entregables!F4</f>
+        <f>Entregables!F9</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="18">
-        <f>Entregables!C5</f>
+        <f>Entregables!C10</f>
         <v/>
       </c>
       <c r="B11" s="18">
-        <f>Entregables!D5</f>
+        <f>Entregables!D10</f>
         <v/>
       </c>
       <c r="C11" s="18">
-        <f>Entregables!E5</f>
+        <f>Entregables!E10</f>
         <v/>
       </c>
       <c r="D11" s="18">
-        <f>Entregables!F5</f>
+        <f>Entregables!F10</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="18">
-        <f>Entregables!C6</f>
+        <f>Entregables!C11</f>
         <v/>
       </c>
       <c r="B12" s="18">
-        <f>Entregables!D6</f>
+        <f>Entregables!D11</f>
         <v/>
       </c>
       <c r="C12" s="18">
-        <f>Entregables!E6</f>
+        <f>Entregables!E11</f>
         <v/>
       </c>
       <c r="D12" s="18">
-        <f>Entregables!F6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
+        <f>Entregables!F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="18">
+        <f>Entregables!C12</f>
+        <v/>
+      </c>
+      <c r="B13" s="18">
+        <f>Entregables!D12</f>
+        <v/>
+      </c>
+      <c r="C13" s="18">
+        <f>Entregables!E12</f>
+        <v/>
+      </c>
+      <c r="D13" s="18">
+        <f>Entregables!F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="18">
+        <f>Entregables!C13</f>
+        <v/>
+      </c>
+      <c r="B14" s="18">
+        <f>Entregables!D13</f>
+        <v/>
+      </c>
+      <c r="C14" s="18">
+        <f>Entregables!E13</f>
+        <v/>
+      </c>
+      <c r="D14" s="18">
+        <f>Entregables!F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="18">
+        <f>Entregables!C14</f>
+        <v/>
+      </c>
+      <c r="B15" s="18">
+        <f>Entregables!D14</f>
+        <v/>
+      </c>
+      <c r="C15" s="18">
+        <f>Entregables!E14</f>
+        <v/>
+      </c>
+      <c r="D15" s="18">
+        <f>Entregables!F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="18">
+        <f>Entregables!C15</f>
+        <v/>
+      </c>
+      <c r="B16" s="18">
+        <f>Entregables!D15</f>
+        <v/>
+      </c>
+      <c r="C16" s="18">
+        <f>Entregables!E15</f>
+        <v/>
+      </c>
+      <c r="D16" s="18">
+        <f>Entregables!F15</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4129,7 +3478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4145,7 +3494,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Gestion de conversaciones</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
     </row>
@@ -4161,17 +3510,18 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="135" customHeight="1">
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C6&amp;CHAR(10)&amp;'Mapa de Impacto'!C7</f>
-        <v/>
-      </c>
-    </row>
+        <f>'Mapa de Impacto'!C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -4179,6 +3529,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -4203,189 +3554,76 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C7</f>
+        <f>Entregables!C16</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D7</f>
+        <f>Entregables!D16</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E7</f>
+        <f>Entregables!E16</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F7</f>
+        <f>Entregables!F16</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C8</f>
+        <f>Entregables!C17</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D8</f>
+        <f>Entregables!D17</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E8</f>
+        <f>Entregables!E17</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F8</f>
+        <f>Entregables!F17</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18">
-        <f>Entregables!C9</f>
+        <f>Entregables!C18</f>
         <v/>
       </c>
       <c r="B10" s="18">
-        <f>Entregables!D9</f>
+        <f>Entregables!D18</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>Entregables!E9</f>
+        <f>Entregables!E18</f>
         <v/>
       </c>
       <c r="D10" s="18">
-        <f>Entregables!F9</f>
+        <f>Entregables!F18</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="18">
-        <f>Entregables!C10</f>
+        <f>Entregables!C19</f>
         <v/>
       </c>
       <c r="B11" s="18">
-        <f>Entregables!D10</f>
+        <f>Entregables!D19</f>
         <v/>
       </c>
       <c r="C11" s="18">
-        <f>Entregables!E10</f>
+        <f>Entregables!E19</f>
         <v/>
       </c>
       <c r="D11" s="18">
-        <f>Entregables!F10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="18">
-        <f>Entregables!C11</f>
-        <v/>
-      </c>
-      <c r="B12" s="18">
-        <f>Entregables!D11</f>
-        <v/>
-      </c>
-      <c r="C12" s="18">
-        <f>Entregables!E11</f>
-        <v/>
-      </c>
-      <c r="D12" s="18">
-        <f>Entregables!F11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="18">
-        <f>Entregables!C12</f>
-        <v/>
-      </c>
-      <c r="B13" s="18">
-        <f>Entregables!D12</f>
-        <v/>
-      </c>
-      <c r="C13" s="18">
-        <f>Entregables!E12</f>
-        <v/>
-      </c>
-      <c r="D13" s="18">
-        <f>Entregables!F12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="18">
-        <f>Entregables!C13</f>
-        <v/>
-      </c>
-      <c r="B14" s="18">
-        <f>Entregables!D13</f>
-        <v/>
-      </c>
-      <c r="C14" s="18">
-        <f>Entregables!E13</f>
-        <v/>
-      </c>
-      <c r="D14" s="18">
-        <f>Entregables!F13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="18">
-        <f>Entregables!C14</f>
-        <v/>
-      </c>
-      <c r="B15" s="18">
-        <f>Entregables!D14</f>
-        <v/>
-      </c>
-      <c r="C15" s="18">
-        <f>Entregables!E14</f>
-        <v/>
-      </c>
-      <c r="D15" s="18">
-        <f>Entregables!F14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="18">
-        <f>Entregables!C15</f>
-        <v/>
-      </c>
-      <c r="B16" s="18">
-        <f>Entregables!D15</f>
-        <v/>
-      </c>
-      <c r="C16" s="18">
-        <f>Entregables!E15</f>
-        <v/>
-      </c>
-      <c r="D16" s="18">
-        <f>Entregables!F15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
+        <f>Entregables!F19</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4400,7 +3638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4416,7 +3654,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Cuenta de usuario</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
     </row>
@@ -4428,7 +3666,7 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Cliente Traductor</t>
+          <t>Interlocutor</t>
         </is>
       </c>
     </row>
@@ -4439,10 +3677,11 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C8</f>
-        <v/>
-      </c>
-    </row>
+        <f>'Mapa de Impacto'!C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -4450,6 +3689,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -4474,104 +3714,52 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C16</f>
+        <f>Entregables!C20</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D16</f>
+        <f>Entregables!D20</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E16</f>
+        <f>Entregables!E20</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F16</f>
+        <f>Entregables!F20</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C17</f>
+        <f>Entregables!C21</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D17</f>
+        <f>Entregables!D21</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E17</f>
+        <f>Entregables!E21</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F17</f>
+        <f>Entregables!F21</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18">
-        <f>Entregables!C18</f>
-        <v/>
-      </c>
-      <c r="B10" s="18">
-        <f>Entregables!D18</f>
-        <v/>
-      </c>
-      <c r="C10" s="18">
-        <f>Entregables!E18</f>
-        <v/>
-      </c>
-      <c r="D10" s="18">
-        <f>Entregables!F18</f>
-        <v/>
-      </c>
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="18">
-        <f>Entregables!C19</f>
-        <v/>
-      </c>
-      <c r="B11" s="18">
-        <f>Entregables!D19</f>
-        <v/>
-      </c>
-      <c r="C11" s="18">
-        <f>Entregables!E19</f>
-        <v/>
-      </c>
-      <c r="D11" s="18">
-        <f>Entregables!F19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4586,7 +3774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4602,7 +3790,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Participacion del interlocutor</t>
+          <t>Reportes</t>
         </is>
       </c>
     </row>
@@ -4614,21 +3802,22 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
+          <t>Cliente Traductor / Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C11</f>
-        <v/>
-      </c>
-    </row>
+        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -4636,6 +3825,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -4660,37 +3850,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C20</f>
+        <f>Entregables!C22</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D20</f>
+        <f>Entregables!D22</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E20</f>
+        <f>Entregables!E22</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F20</f>
+        <f>Entregables!F22</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C21</f>
+        <f>Entregables!C23</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D21</f>
+        <f>Entregables!D23</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E21</f>
+        <f>Entregables!E23</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F21</f>
+        <f>Entregables!F23</f>
         <v/>
       </c>
     </row>
@@ -4706,34 +3896,6 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4748,7 +3910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4764,7 +3926,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Reportes</t>
+          <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
     </row>
@@ -4787,10 +3949,11 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
-        <v/>
-      </c>
-    </row>
+        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -4798,6 +3961,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -4822,45 +3986,57 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C22</f>
+        <f>Entregables!C24</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D22</f>
+        <f>Entregables!D24</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E22</f>
+        <f>Entregables!E24</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F22</f>
+        <f>Entregables!F24</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C23</f>
+        <f>Entregables!C25</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D23</f>
+        <f>Entregables!D25</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E23</f>
+        <f>Entregables!E25</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F23</f>
+        <f>Entregables!F25</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
+      <c r="A10" s="18">
+        <f>Entregables!C26</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D26</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E26</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F26</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="18" t="n"/>
@@ -4868,34 +4044,6 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>

</xml_diff>

<commit_message>
Plan de liberaciones, criterios de aceptacion y motor Qwen local (Ollama) con Claude Sonnet de respaldo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -9,12 +9,13 @@
     <sheet name="Mapa de Impacto" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Entregables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Planificacion" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Traduccion de mensajes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gestion de conversaciones" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cuenta de usuario" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Participacion interlocutor" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Reportes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Admin idiomas y regiones" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Plan de liberaciones" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Traduccion de mensajes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gestion de conversaciones" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cuenta de usuario" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Participacion interlocutor" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Reportes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Admin idiomas y regiones" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -23,7 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="14">
     <font>
       <name val="Calibri"/>
@@ -533,7 +537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -705,6 +709,30 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1470,13 +1498,159 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Entregable</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Cliente Traductor / Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Impacto (para)</t>
+        </is>
+      </c>
+      <c r="B3" s="18">
+        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>← Volver al Mapa de Impacto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Característica</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Necesito</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Para</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C24</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D24</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E24</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C25</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D25</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E25</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18">
+        <f>Entregables!C26</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D26</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E26</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1490,6 +1664,7 @@
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="95" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1548,33 +1723,38 @@
           <t>Por que genera valor</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Criterios de aceptacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="64" customHeight="1">
+      <c r="A2" s="67" t="inlineStr">
         <is>
           <t>Traduccion de mensajes</t>
         </is>
       </c>
-      <c r="B2" s="33" t="inlineStr">
+      <c r="B2" s="67" t="inlineStr">
         <is>
           <t>HU0001</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
+      <c r="C2" s="68" t="inlineStr">
         <is>
           <t>Ingresar mi mensaje hablando</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E2">
+      <c r="E2" s="58">
         <f>C2</f>
         <v/>
       </c>
-      <c r="F2">
+      <c r="F2" s="58">
         <f>'Mapa de Impacto'!C4</f>
         <v/>
       </c>
@@ -1598,29 +1778,35 @@
           <t>Es la forma natural de usar el producto: hablar y ser entendido sin escribir.</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="34" t="n"/>
-      <c r="B3" s="33" t="inlineStr">
+      <c r="L2" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que estoy en una conversacion en modo voz, cuando dicto mi mensaje (microfono del navegador o del teclado), entonces el texto aparece y se envia por el canal de voz.
+2. Cuando el microfono no esta permitido o el dispositivo no puede dictar, entonces veo un aviso claro y puedo escribir el mensaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="70" t="n"/>
+      <c r="B3" s="67" t="inlineStr">
         <is>
           <t>HU0002</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr">
+      <c r="C3" s="68" t="inlineStr">
         <is>
           <t>Ingresar mi mensaje escribiendo</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E3">
+      <c r="E3" s="58">
         <f>C3</f>
         <v/>
       </c>
-      <c r="F3">
+      <c r="F3" s="58">
         <f>'Mapa de Impacto'!C4</f>
         <v/>
       </c>
@@ -1644,29 +1830,35 @@
           <t>Es la entrada mas simple y la que permite usar la traduccion desde el primer dia.</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="34" t="n"/>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="L3" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que estoy en una conversacion, cuando escribo un mensaje y lo envio, entonces aparecen mi mensaje original y su traduccion.
+2. No se puede enviar un mensaje vacio ni de mas de 5000 caracteres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
+      <c r="A4" s="70" t="n"/>
+      <c r="B4" s="67" t="inlineStr">
         <is>
           <t>HU0003</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="68" t="inlineStr">
         <is>
           <t>Traducir mi mensaje al idioma destino en tiempo real</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E4">
+      <c r="E4" s="58">
         <f>C4</f>
         <v/>
       </c>
-      <c r="F4">
+      <c r="F4" s="58">
         <f>'Mapa de Impacto'!C4</f>
         <v/>
       </c>
@@ -1690,29 +1882,36 @@
           <t>Es el corazon del producto: sin esto TalkLate no entrega su valor diferencial.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="34" t="n"/>
-      <c r="B5" s="33" t="inlineStr">
+      <c r="L4" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado un mensaje con un modismo (ej. 'Hay que ponerse las pilas con el trabajo'), cuando lo envio, entonces la traduccion usa el equivalente cultural en la region destino ('We need to get cracking on the work') y no una version literal.
+2. Cuando se adapto un modismo, entonces puedo ver una nota cultural que lo explica; si quedaron palabras sin traducir, la traduccion se marca como aproximada.
+3. Cuando el servicio no puede traducir, entonces veo un mensaje de error en vez de un resultado vacio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="64" customHeight="1">
+      <c r="A5" s="70" t="n"/>
+      <c r="B5" s="67" t="inlineStr">
         <is>
           <t>HU0004</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="68" t="inlineStr">
         <is>
           <t>Escuchar el mensaje traducido</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E5">
+      <c r="E5" s="58">
         <f>C5</f>
         <v/>
       </c>
-      <c r="F5">
+      <c r="F5" s="58">
         <f>'Mapa de Impacto'!C9</f>
         <v/>
       </c>
@@ -1736,29 +1935,35 @@
           <t>Permite que la otra persona reciba el mensaje de forma comoda y natural.</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="35" t="n"/>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="L5" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado un mensaje traducido, cuando toco 'Escuchar', entonces se reproduce con la voz del idioma y pais destino.
+2. La velocidad y el tono de la voz cambian segun la entonacion detectada (por ejemplo, alegre o preocupado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="71" t="n"/>
+      <c r="B6" s="67" t="inlineStr">
         <is>
           <t>HU0005</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="68" t="inlineStr">
         <is>
           <t>Recibir la traduccion por el mismo canal que use</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E6">
+      <c r="E6" s="58">
         <f>C6</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="58">
         <f>'Mapa de Impacto'!C9</f>
         <v/>
       </c>
@@ -1782,33 +1987,39 @@
           <t>Mantiene la experiencia coherente: si hablo, escucho; si escribo, leo.</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="L6" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que envie el mensaje por voz, entonces la traduccion se reproduce sola y tambien queda escrita.
+2. Dado que envie el mensaje por texto, entonces la traduccion solo se muestra escrita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="67" t="inlineStr">
         <is>
           <t>Gestion de conversaciones</t>
         </is>
       </c>
-      <c r="B7" s="33" t="inlineStr">
+      <c r="B7" s="67" t="inlineStr">
         <is>
           <t>HU0006</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="68" t="inlineStr">
         <is>
           <t>Seleccionar el idioma y la region destino</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E7">
+      <c r="E7" s="58">
         <f>C7</f>
         <v/>
       </c>
-      <c r="F7">
+      <c r="F7" s="58">
         <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
@@ -1832,29 +2043,35 @@
           <t>Define a que persona y lugar se adapta el mensaje: de ahi sale el matiz cultural.</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="34" t="n"/>
-      <c r="B8" s="33" t="inlineStr">
+      <c r="L7" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que creo una conversacion, cuando elijo un idioma de destino, entonces solo veo las regiones validas para ese idioma.
+2. No puedo empezar la conversacion si falta el idioma o la region destino.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="70" t="n"/>
+      <c r="B8" s="67" t="inlineStr">
         <is>
           <t>HU0007</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="68" t="inlineStr">
         <is>
           <t>Reconocer el idioma origen</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E8">
+      <c r="E8" s="58">
         <f>C8</f>
         <v/>
       </c>
-      <c r="F8">
+      <c r="F8" s="58">
         <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
@@ -1878,29 +2095,36 @@
           <t>Evita configurar a mano el idioma cada vez y acelera la conversacion.</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="34" t="n"/>
-      <c r="B9" s="33" t="inlineStr">
+      <c r="L8" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que no elegi mi idioma, cuando envio mi primer mensaje, entonces el sistema lo reconoce y lo muestra en el encabezado de la conversacion.
+2. Una vez reconocido, el idioma de origen no cambia en esa conversacion.
+3. Cuando el mensaje es muy corto para reconocer el idioma, entonces se me pide escribir un poco mas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="70" t="n"/>
+      <c r="B9" s="67" t="inlineStr">
         <is>
           <t>HU0008</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="68" t="inlineStr">
         <is>
           <t>Crear una conversacion</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E9">
+      <c r="E9" s="58">
         <f>C9</f>
         <v/>
       </c>
-      <c r="F9">
+      <c r="F9" s="58">
         <f>'Mapa de Impacto'!C6</f>
         <v/>
       </c>
@@ -1924,29 +2148,35 @@
           <t>Agrupa los mensajes de una misma charla para no perder el contexto.</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="34" t="n"/>
-      <c r="B10" s="33" t="inlineStr">
+      <c r="L9" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando creo una conversacion sin nombre, entonces se llama 'Nueva Conversacion'.
+2. La conversacion creada aparece en el menu lateral y en el historial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="70" t="n"/>
+      <c r="B10" s="67" t="inlineStr">
         <is>
           <t>HU0009</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="68" t="inlineStr">
         <is>
           <t>Configurar los parametros una sola vez</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E10">
+      <c r="E10" s="58">
         <f>C10</f>
         <v/>
       </c>
-      <c r="F10">
+      <c r="F10" s="58">
         <f>'Mapa de Impacto'!C6</f>
         <v/>
       </c>
@@ -1970,29 +2200,35 @@
           <t>Ahorra repetir la configuracion en cada mensaje.</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="34" t="n"/>
-      <c r="B11" s="33" t="inlineStr">
+      <c r="L10" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que ya elegi idioma y region destino al crear la conversacion, entonces los mensajes siguientes no me piden configurar nada.
+2. El destino de la conversacion se mantiene mientras la uso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="70" t="n"/>
+      <c r="B11" s="67" t="inlineStr">
         <is>
           <t>HU0010</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="68" t="inlineStr">
         <is>
           <t>Mantener el hilo continuo</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E11">
+      <c r="E11" s="58">
         <f>C11</f>
         <v/>
       </c>
-      <c r="F11">
+      <c r="F11" s="58">
         <f>'Mapa de Impacto'!C6</f>
         <v/>
       </c>
@@ -2016,29 +2252,35 @@
           <t>Hace posible un dialogo fluido, que es lo que busca el usuario.</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="34" t="n"/>
-      <c r="B12" s="33" t="inlineStr">
+      <c r="L11" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando envio varios mensajes seguidos, entonces cada uno se traduce y queda en el mismo hilo, en orden.
+2. Cuando reabro la conversacion mas tarde, entonces veo todos los mensajes anteriores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="64" customHeight="1">
+      <c r="A12" s="70" t="n"/>
+      <c r="B12" s="67" t="inlineStr">
         <is>
           <t>HU0011</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="68" t="inlineStr">
         <is>
           <t>Consultar mi historial</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E12">
+      <c r="E12" s="58">
         <f>C12</f>
         <v/>
       </c>
-      <c r="F12">
+      <c r="F12" s="58">
         <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
@@ -2062,29 +2304,36 @@
           <t>Permite repasar y aprender de conversaciones pasadas.</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="34" t="n"/>
-      <c r="B13" s="33" t="inlineStr">
+      <c r="L12" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando abro el historial, entonces veo mis conversaciones con su nombre, idiomas, numero de mensajes y ultimo mensaje, las mas recientes primero.
+2. Puedo buscar una conversacion por su nombre.
+3. Solo veo mis propias conversaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="70" t="n"/>
+      <c r="B13" s="67" t="inlineStr">
         <is>
           <t>HU0012</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="68" t="inlineStr">
         <is>
           <t>Abrir una conversacion anterior</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E13">
+      <c r="E13" s="58">
         <f>C13</f>
         <v/>
       </c>
-      <c r="F13">
+      <c r="F13" s="58">
         <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
@@ -2108,29 +2357,35 @@
           <t>Permite retomar una conversacion donde se dejo.</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="34" t="n"/>
-      <c r="B14" s="33" t="inlineStr">
+      <c r="L13" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando toco una conversacion del historial, entonces veo sus mensajes originales y traducidos en orden.
+2. No puedo abrir la conversacion de otra persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="70" t="n"/>
+      <c r="B14" s="67" t="inlineStr">
         <is>
           <t>HU0013</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="68" t="inlineStr">
         <is>
           <t>Renombrar una conversacion</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E14">
+      <c r="E14" s="58">
         <f>C14</f>
         <v/>
       </c>
-      <c r="F14">
+      <c r="F14" s="58">
         <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
@@ -2154,29 +2409,35 @@
           <t>Ayuda a ubicar conversaciones, pero no cambia el valor central.</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="35" t="n"/>
-      <c r="B15" s="33" t="inlineStr">
+      <c r="L14" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando cambio el nombre, entonces debe tener entre 3 y 80 caracteres, sin caracteres especiales ni palabras ofensivas; si no, veo el motivo.
+2. El nombre nuevo se ve en el encabezado, el menu y el historial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="71" t="n"/>
+      <c r="B15" s="67" t="inlineStr">
         <is>
           <t>HU0014</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="68" t="inlineStr">
         <is>
           <t>Eliminar una conversacion</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E15">
+      <c r="E15" s="58">
         <f>C15</f>
         <v/>
       </c>
-      <c r="F15">
+      <c r="F15" s="58">
         <f>'Mapa de Impacto'!C7</f>
         <v/>
       </c>
@@ -2200,33 +2461,39 @@
           <t>Da control sobre los datos propios; es de apoyo.</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="33" t="inlineStr">
+      <c r="L15" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando elijo eliminar, entonces la app me pide confirmar y me avisa que no se puede deshacer.
+2. Al confirmar, la conversacion se borra con sus mensajes y reportes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="67" t="inlineStr">
         <is>
           <t>Cuenta de usuario</t>
         </is>
       </c>
-      <c r="B16" s="33" t="inlineStr">
+      <c r="B16" s="67" t="inlineStr">
         <is>
           <t>HU0015</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="68" t="inlineStr">
         <is>
           <t>Registrarme en la aplicacion</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E16">
+      <c r="E16" s="58">
         <f>C16</f>
         <v/>
       </c>
-      <c r="F16">
+      <c r="F16" s="58">
         <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
@@ -2250,29 +2517,37 @@
           <t>Guarda las conversaciones del usuario y protege sus datos; el valor central no depende de esto.</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="34" t="n"/>
-      <c r="B17" s="33" t="inlineStr">
+      <c r="L16" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando me registro con datos validos, entonces la cuenta se crea y entro a la app.
+2. La contrasena debe tener 8 o mas caracteres, una mayuscula, un numero y un simbolo; el correo debe tener formato valido.
+3. Debo tener 13 anos o mas; si no, veo 'debes tener al menos 13 anos'.
+4. Si el correo ya esta registrado, veo un aviso para iniciar sesion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="64" customHeight="1">
+      <c r="A17" s="70" t="n"/>
+      <c r="B17" s="67" t="inlineStr">
         <is>
           <t>HU0016</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="68" t="inlineStr">
         <is>
           <t>Iniciar sesion</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E17">
+      <c r="E17" s="58">
         <f>C17</f>
         <v/>
       </c>
-      <c r="F17">
+      <c r="F17" s="58">
         <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
@@ -2296,29 +2571,36 @@
           <t>Da acceso seguro a lo guardado.</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="34" t="n"/>
-      <c r="B18" s="33" t="inlineStr">
+      <c r="L17" s="69" t="inlineStr">
+        <is>
+          <t>1. Con correo y contrasena correctos entro a la app; con datos incorrectos veo 'Usuario o contrasena incorrectos'.
+2. Despues de varios intentos fallidos seguidos, el acceso se bloquea unos minutos.
+3. Al cerrar y abrir la app sigo con la sesion iniciada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="96" customHeight="1">
+      <c r="A18" s="70" t="n"/>
+      <c r="B18" s="67" t="inlineStr">
         <is>
           <t>HU0017</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="68" t="inlineStr">
         <is>
           <t>Recuperar mi contrasena</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E18">
+      <c r="E18" s="58">
         <f>C18</f>
         <v/>
       </c>
-      <c r="F18">
+      <c r="F18" s="58">
         <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
@@ -2342,29 +2624,37 @@
           <t>Evita perder la cuenta; es de apoyo.</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="35" t="n"/>
-      <c r="B19" s="33" t="inlineStr">
+      <c r="L18" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando pido recuperar la contrasena con un correo registrado, entonces recibo un codigo de 6 digitos que vence en 15 minutos.
+2. Con un codigo correcto y una contrasena nueva que cumpla las reglas, la contrasena cambia; el codigo solo sirve una vez.
+3. Con un codigo incorrecto o vencido veo que debo pedir uno nuevo.
+4. Si el correo no esta registrado, veo que no hay una cuenta asociada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="71" t="n"/>
+      <c r="B19" s="67" t="inlineStr">
         <is>
           <t>HU0018</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="68" t="inlineStr">
         <is>
           <t>Cerrar sesion</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E19">
+      <c r="E19" s="58">
         <f>C19</f>
         <v/>
       </c>
-      <c r="F19">
+      <c r="F19" s="58">
         <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
@@ -2388,33 +2678,39 @@
           <t>Protege la cuenta en un dispositivo compartido; es de apoyo.</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="33" t="inlineStr">
+      <c r="L19" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando cierro sesion, entonces vuelvo a la pantalla de bienvenida.
+2. El acceso anterior deja de funcionar aunque alguien lo conserve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="67" t="inlineStr">
         <is>
           <t>Participacion del interlocutor</t>
         </is>
       </c>
-      <c r="B20" s="33" t="inlineStr">
+      <c r="B20" s="67" t="inlineStr">
         <is>
           <t>HU0019</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="68" t="inlineStr">
         <is>
           <t>Recibir el mensaje traducido</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="58" t="inlineStr">
         <is>
           <t>Interlocutor</t>
         </is>
       </c>
-      <c r="E20">
+      <c r="E20" s="58">
         <f>C20</f>
         <v/>
       </c>
-      <c r="F20">
+      <c r="F20" s="58">
         <f>'Mapa de Impacto'!C11</f>
         <v/>
       </c>
@@ -2438,29 +2734,35 @@
           <t>Hace que la otra persona participe sin instalar ni operar la app.</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="35" t="n"/>
-      <c r="B21" s="33" t="inlineStr">
+      <c r="L20" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que la otra persona responde (se escribe como 'Otra persona'), entonces su mensaje se traduce a mi idioma y se muestra a la izquierda, junto a su original.
+2. La otra persona no necesita instalar la app ni tener cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="71" t="n"/>
+      <c r="B21" s="67" t="inlineStr">
         <is>
           <t>HU0020</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="68" t="inlineStr">
         <is>
           <t>Responder en mi idioma</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="58" t="inlineStr">
         <is>
           <t>Interlocutor</t>
         </is>
       </c>
-      <c r="E21">
+      <c r="E21" s="58">
         <f>C21</f>
         <v/>
       </c>
-      <c r="F21">
+      <c r="F21" s="58">
         <f>'Mapa de Impacto'!C11</f>
         <v/>
       </c>
@@ -2484,33 +2786,39 @@
           <t>Cierra el dialogo en ambos sentidos.</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="33" t="inlineStr">
+      <c r="L21" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando la otra persona escribe en su propio idioma, entonces su respuesta se traduce al idioma de la conversacion.
+2. Para responder ya debe haberse reconocido mi idioma con mi primer mensaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="67" t="inlineStr">
         <is>
           <t>Reportes</t>
         </is>
       </c>
-      <c r="B22" s="33" t="inlineStr">
+      <c r="B22" s="67" t="inlineStr">
         <is>
           <t>HU0021</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="68" t="inlineStr">
         <is>
           <t>Reportar una mala traduccion</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E22">
+      <c r="E22" s="58">
         <f>C22</f>
         <v/>
       </c>
-      <c r="F22">
+      <c r="F22" s="58">
         <f>'Mapa de Impacto'!C10</f>
         <v/>
       </c>
@@ -2534,29 +2842,35 @@
           <t>Alimenta la mejora de calidad con casos reales.</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="35" t="n"/>
-      <c r="B23" s="33" t="inlineStr">
+      <c r="L22" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando reporto una traduccion con un motivo de 3 a 500 caracteres, entonces el reporte se guarda y el mensaje queda marcado como 'Reportado'.
+2. Solo puedo reportar una vez la misma traduccion y solo las de mis conversaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="64" customHeight="1">
+      <c r="A23" s="71" t="n"/>
+      <c r="B23" s="67" t="inlineStr">
         <is>
           <t>HU0022</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="68" t="inlineStr">
         <is>
           <t>Revisar los reportes de mala traduccion</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E23">
+      <c r="E23" s="58">
         <f>C23</f>
         <v/>
       </c>
-      <c r="F23">
+      <c r="F23" s="58">
         <f>'Mapa de Impacto'!C13</f>
         <v/>
       </c>
@@ -2580,33 +2894,40 @@
           <t>Permite priorizar que mejorar primero.</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="33" t="inlineStr">
+      <c r="L23" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que soy administrador, cuando abro los reportes, entonces veo el original, la traduccion, el motivo y la sugerencia, y puedo filtrar por abiertos, revisados o descartados.
+2. Puedo marcar un reporte como revisado o descartado.
+3. Un cliente que no es administrador no puede ver ni cambiar reportes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="67" t="inlineStr">
         <is>
           <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
-      <c r="B24" s="33" t="inlineStr">
+      <c r="B24" s="67" t="inlineStr">
         <is>
           <t>HU0023</t>
         </is>
       </c>
-      <c r="C24" s="23" t="inlineStr">
+      <c r="C24" s="68" t="inlineStr">
         <is>
           <t>Consultar los idiomas disponibles</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E24">
+      <c r="E24" s="58">
         <f>C24</f>
         <v/>
       </c>
-      <c r="F24">
+      <c r="F24" s="58">
         <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
@@ -2630,29 +2951,35 @@
           <t>Muestra con que idiomas se puede hablar antes de empezar.</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="34" t="n"/>
-      <c r="B25" s="33" t="inlineStr">
+      <c r="L24" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando abro la configuracion de una conversacion, entonces veo solo los idiomas activos con sus regiones.
+2. Los idiomas desactivados no aparecen en la lista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="80" customHeight="1">
+      <c r="A25" s="70" t="n"/>
+      <c r="B25" s="67" t="inlineStr">
         <is>
           <t>HU0024</t>
         </is>
       </c>
-      <c r="C25" s="23" t="inlineStr">
+      <c r="C25" s="68" t="inlineStr">
         <is>
           <t>Agregar un idioma o una region</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E25">
+      <c r="E25" s="58">
         <f>C25</f>
         <v/>
       </c>
-      <c r="F25">
+      <c r="F25" s="58">
         <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
@@ -2676,29 +3003,36 @@
           <t>Hace crecer el servicio a mas personas.</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="35" t="n"/>
-      <c r="B26" s="33" t="inlineStr">
+      <c r="L25" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que soy administrador, cuando agrego un idioma, entonces necesita un nombre unico y un codigo de 2 a 5 letras, y queda desactivado hasta que lo active.
+2. Una region no puede repetirse dentro del mismo pais; si el pais no existe, debo indicar su codigo de 2 letras.
+3. Un cliente que no es administrador no puede agregar idiomas ni regiones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="71" t="n"/>
+      <c r="B26" s="67" t="inlineStr">
         <is>
           <t>HU0025</t>
         </is>
       </c>
-      <c r="C26" s="23" t="inlineStr">
+      <c r="C26" s="68" t="inlineStr">
         <is>
           <t>Activar o desactivar un idioma o una region</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E26">
+      <c r="E26" s="58">
         <f>C26</f>
         <v/>
       </c>
-      <c r="F26">
+      <c r="F26" s="58">
         <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
@@ -2720,6 +3054,12 @@
       <c r="K26" s="58" t="inlineStr">
         <is>
           <t>Controla que idiomas se ofrecen con calidad suficiente.</t>
+        </is>
+      </c>
+      <c r="L26" s="69" t="inlineStr">
+        <is>
+          <t>1. Cuando activo un idioma, entonces aparece en el catalogo para crear conversaciones; cuando lo desactivo, deja de aparecer.
+2. Las conversaciones ya creadas no se ven afectadas.</t>
         </is>
       </c>
     </row>
@@ -2745,7 +3085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2753,6 +3093,9 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2767,7 +3110,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="60" t="inlineStr">
         <is>
@@ -2890,8 +3232,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="59" t="inlineStr">
         <is>
@@ -2923,6 +3263,21 @@
       <c r="E13" s="60" t="inlineStr">
         <is>
           <t>Historias</t>
+        </is>
+      </c>
+      <c r="F13" s="72" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="G13" s="72" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="H13" s="72" t="inlineStr">
+        <is>
+          <t>Liberacion</t>
         </is>
       </c>
     </row>
@@ -2947,6 +3302,17 @@
           <t>HU0001, HU0002, HU0003, HU0004, HU0005, HU0006</t>
         </is>
       </c>
+      <c r="F14" s="73" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G14" s="73" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H14" s="62" t="inlineStr">
+        <is>
+          <t>Liberacion 1</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="64" t="n">
@@ -2969,6 +3335,17 @@
           <t>HU0007, HU0008, HU0009, HU0010, HU0011, HU0012, HU0013, HU0018, HU0019, HU0020, HU0023, HU0025</t>
         </is>
       </c>
+      <c r="F15" s="73" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G15" s="73" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H15" s="62" t="inlineStr">
+        <is>
+          <t>Liberacion 2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="64" t="n">
@@ -2991,6 +3368,17 @@
           <t>HU0014, HU0015, HU0016, HU0017, HU0021, HU0022, HU0024</t>
         </is>
       </c>
+      <c r="F16" s="73" t="n">
+        <v>46328</v>
+      </c>
+      <c r="G16" s="73" t="n">
+        <v>46332</v>
+      </c>
+      <c r="H16" s="62" t="inlineStr">
+        <is>
+          <t>Liberacion 3</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="66" t="inlineStr">
@@ -3003,7 +3391,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="66" t="inlineStr">
         <is>
@@ -3045,6 +3432,198 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>Plan de liberaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cada sprint dura una semana (lunes a viernes) y termina con una liberacion. El primer sprint empieza el lunes 19/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>Liberacion</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="F4" s="60" t="inlineStr">
+        <is>
+          <t>Que recibe el usuario</t>
+        </is>
+      </c>
+      <c r="G4" s="60" t="inlineStr">
+        <is>
+          <t>Historias</t>
+        </is>
+      </c>
+      <c r="H4" s="60" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="64" t="inlineStr">
+        <is>
+          <t>Liberacion 1</t>
+        </is>
+      </c>
+      <c r="B5" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="74" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D5" s="74" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E5" s="65" t="inlineStr">
+        <is>
+          <t>Traduccion funcional</t>
+        </is>
+      </c>
+      <c r="F5" s="65" t="inlineStr">
+        <is>
+          <t>El usuario puede escribir o hablar un mensaje, recibirlo traducido con el tono y los modismos adaptados, escucharlo y obtenerlo por el mismo canal. Es el valor central del producto.</t>
+        </is>
+      </c>
+      <c r="G5" s="65" t="inlineStr">
+        <is>
+          <t>HU0001, HU0002, HU0003, HU0004, HU0005, HU0006</t>
+        </is>
+      </c>
+      <c r="H5" s="64">
+        <f>SUMIF(Entregables!$J$2:$J$40,B5,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
+      <c r="A6" s="64" t="inlineStr">
+        <is>
+          <t>Liberacion 2</t>
+        </is>
+      </c>
+      <c r="B6" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="74" t="n">
+        <v>46321</v>
+      </c>
+      <c r="D6" s="74" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E6" s="65" t="inlineStr">
+        <is>
+          <t>Conversaciones completas</t>
+        </is>
+      </c>
+      <c r="F6" s="65" t="inlineStr">
+        <is>
+          <t>El usuario organiza sus conversaciones (reconocer idioma, crear, hilo continuo, historial, renombrar), la otra persona participa y el administrador controla que idiomas se activan.</t>
+        </is>
+      </c>
+      <c r="G6" s="65" t="inlineStr">
+        <is>
+          <t>HU0007, HU0008, HU0009, HU0010, HU0011, HU0012, HU0013, HU0018, HU0019, HU0020, HU0023, HU0025</t>
+        </is>
+      </c>
+      <c r="H6" s="64">
+        <f>SUMIF(Entregables!$J$2:$J$40,B6,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
+      <c r="A7" s="64" t="inlineStr">
+        <is>
+          <t>Liberacion 3</t>
+        </is>
+      </c>
+      <c r="B7" s="64" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="74" t="n">
+        <v>46328</v>
+      </c>
+      <c r="D7" s="74" t="n">
+        <v>46332</v>
+      </c>
+      <c r="E7" s="65" t="inlineStr">
+        <is>
+          <t>Cuentas, calidad y administracion</t>
+        </is>
+      </c>
+      <c r="F7" s="65" t="inlineStr">
+        <is>
+          <t>Registro, inicio de sesion y recuperacion de contrasena, eliminar conversaciones, reportar y revisar malas traducciones, y agregar idiomas y regiones.</t>
+        </is>
+      </c>
+      <c r="G7" s="65" t="inlineStr">
+        <is>
+          <t>HU0014, HU0015, HU0016, HU0017, HU0021, HU0022, HU0024</t>
+        </is>
+      </c>
+      <c r="H7" s="64">
+        <f>SUMIF(Entregables!$J$2:$J$40,B7,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nota: el orden sale de la prioridad por valor; el plan es metodologico y las horas reales de cada semana pueden variar.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3093,7 +3672,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3101,7 +3679,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3222,7 +3799,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3271,7 +3848,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3279,7 +3855,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3461,166 +4036,6 @@
       </c>
       <c r="D16" s="18">
         <f>Entregables!F15</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Cliente Traductor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="18">
-        <f>Entregables!C16</f>
-        <v/>
-      </c>
-      <c r="B8" s="18">
-        <f>Entregables!D16</f>
-        <v/>
-      </c>
-      <c r="C8" s="18">
-        <f>Entregables!E16</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>Entregables!F16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="18">
-        <f>Entregables!C17</f>
-        <v/>
-      </c>
-      <c r="B9" s="18">
-        <f>Entregables!D17</f>
-        <v/>
-      </c>
-      <c r="C9" s="18">
-        <f>Entregables!E17</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>Entregables!F17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18">
-        <f>Entregables!C18</f>
-        <v/>
-      </c>
-      <c r="B10" s="18">
-        <f>Entregables!D18</f>
-        <v/>
-      </c>
-      <c r="C10" s="18">
-        <f>Entregables!E18</f>
-        <v/>
-      </c>
-      <c r="D10" s="18">
-        <f>Entregables!F18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="18">
-        <f>Entregables!C19</f>
-        <v/>
-      </c>
-      <c r="B11" s="18">
-        <f>Entregables!D19</f>
-        <v/>
-      </c>
-      <c r="C11" s="18">
-        <f>Entregables!E19</f>
-        <v/>
-      </c>
-      <c r="D11" s="18">
-        <f>Entregables!F19</f>
         <v/>
       </c>
     </row>
@@ -3654,7 +4069,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Participacion del interlocutor</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
     </row>
@@ -3666,7 +4081,7 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Interlocutor</t>
+          <t>Cliente Traductor</t>
         </is>
       </c>
     </row>
@@ -3677,11 +4092,10 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4"/>
+        <f>'Mapa de Impacto'!C8</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3689,7 +4103,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3714,51 +4127,75 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C20</f>
+        <f>Entregables!C16</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D20</f>
+        <f>Entregables!D16</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E20</f>
+        <f>Entregables!E16</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F20</f>
+        <f>Entregables!F16</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C21</f>
+        <f>Entregables!C17</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D21</f>
+        <f>Entregables!D17</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E21</f>
+        <f>Entregables!E17</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F21</f>
+        <f>Entregables!F17</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
+      <c r="A10" s="18">
+        <f>Entregables!C18</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>Entregables!D18</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>Entregables!E18</f>
+        <v/>
+      </c>
+      <c r="D10" s="18">
+        <f>Entregables!F18</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="18" t="n"/>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
+      <c r="A11" s="18">
+        <f>Entregables!C19</f>
+        <v/>
+      </c>
+      <c r="B11" s="18">
+        <f>Entregables!D19</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>Entregables!E19</f>
+        <v/>
+      </c>
+      <c r="D11" s="18">
+        <f>Entregables!F19</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3790,7 +4227,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Reportes</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
     </row>
@@ -3802,22 +4239,21 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Cliente Traductor / Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="90" customHeight="1">
+          <t>Interlocutor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4"/>
+        <f>'Mapa de Impacto'!C11</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3825,7 +4261,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3850,37 +4285,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C22</f>
+        <f>Entregables!C20</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D22</f>
+        <f>Entregables!D20</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E22</f>
+        <f>Entregables!E20</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F22</f>
+        <f>Entregables!F20</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C23</f>
+        <f>Entregables!C21</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D23</f>
+        <f>Entregables!D21</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E23</f>
+        <f>Entregables!E21</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F23</f>
+        <f>Entregables!F21</f>
         <v/>
       </c>
     </row>
@@ -3926,7 +4361,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Administracion de idiomas y regiones</t>
+          <t>Reportes</t>
         </is>
       </c>
     </row>
@@ -3949,11 +4384,10 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C5&amp;CHAR(10)&amp;'Mapa de Impacto'!C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4"/>
+        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3961,7 +4395,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
@@ -3986,57 +4419,45 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C24</f>
+        <f>Entregables!C22</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D24</f>
+        <f>Entregables!D22</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E24</f>
+        <f>Entregables!E22</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F24</f>
+        <f>Entregables!F22</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C25</f>
+        <f>Entregables!C23</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D25</f>
+        <f>Entregables!D23</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E25</f>
+        <f>Entregables!E23</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F25</f>
+        <f>Entregables!F23</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18">
-        <f>Entregables!C26</f>
-        <v/>
-      </c>
-      <c r="B10" s="18">
-        <f>Entregables!D26</f>
-        <v/>
-      </c>
-      <c r="C10" s="18">
-        <f>Entregables!E26</f>
-        <v/>
-      </c>
-      <c r="D10" s="18">
-        <f>Entregables!F26</f>
-        <v/>
-      </c>
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="18" t="n"/>

</xml_diff>

<commit_message>
docs: objetivo e impactos SMART, HU0026, requerimientos, matriz de sensibilidad, acta y marco metodologico (#1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -24,9 +24,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -537,7 +536,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -727,10 +726,16 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1098,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="45.1640625" customWidth="1" min="1" max="1"/>
@@ -1108,6 +1113,7 @@
     <col width="48.33203125" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -1138,6 +1144,11 @@
           <t>DUDAS</t>
         </is>
       </c>
+      <c r="H1" s="41" t="inlineStr">
+        <is>
+          <t>Indicador SMART (como se mide y para cuando)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1171,6 +1182,7 @@
         </is>
       </c>
       <c r="G2" s="37" t="n"/>
+      <c r="H2" s="37" t="n"/>
     </row>
     <row r="3" ht="17" customHeight="1" thickBot="1">
       <c r="A3" s="5" t="inlineStr">
@@ -1196,11 +1208,12 @@
         </is>
       </c>
       <c r="G3" s="38" t="n"/>
+      <c r="H3" s="38" t="n"/>
     </row>
     <row r="4" ht="78" customHeight="1">
       <c r="A4" s="39" t="inlineStr">
         <is>
-          <t>Para cualquier persona que necesita expresarse verbal o textualmente en un idioma que no conoce o domina, incluyendo no solo su mensaje sino también cualquier modismo o jerga cultural utilizada sin perder el significado o contexto del mismo, TalkLate es una aplicación móvil que está diseñada para ofrecer una experiencia de traducción que va más allá de la conversión literal de palabras, ya que considera el contexto, las emociones, los matices culturales y las intenciones detrás del lenguaje, permitiendo una comunicación más natural y significativa. A diferencia de Meta Seamless, Deepl Translator, TimeKettle, Lilt y Kudo AI, nuestro producto se distingue por su enfoque en la conexión profunda, permitiendo a los usuarios expresarse auténticamente en otro idioma, con foco inicial en ciertas regiones y acentos específicos del inglés y el español, y con una visión evolutiva para soportar con el paso del tiempo otros lenguajes con sus respectivos modismos y características, sin perder la espontaneidad ni la riqueza de su comunicación original.</t>
+          <t>Objetivo (SMART): al cierre de la liberacion 3 (06/11/2026), al menos 10 personas de prueba sostienen cada una una conversacion de 10 mensajes o mas con alguien que habla otro idioma (espanol-ingles), con menos del 20 % de traducciones reportadas como malas y un tiempo por traduccion de 3 segundos o menos (p95). Vision: ver contexto.md.</t>
         </is>
       </c>
       <c r="B4" s="36" t="inlineStr">
@@ -1229,43 +1242,53 @@
         </is>
       </c>
       <c r="G4" s="32" t="n"/>
+      <c r="H4" s="43" t="inlineStr">
+        <is>
+          <t>Liberacion 1 (23/10/2026): el 80 % de los modismos del glosario de prueba se traducen con su equivalente cultural y en 3 segundos o menos (p95). Se mide con npm run medir.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="78" customHeight="1">
       <c r="A5" s="40" t="n"/>
       <c r="B5" s="37" t="n"/>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Comunicarse de inmediato sin tener que repetir la configuración de idioma en cada mensaje.</t>
+          <t>Empezar a conversar en menos de un minuto, configurando idioma y region destino una sola vez y sin tener que indicar el idioma propio.</t>
         </is>
       </c>
       <c r="D5" s="53" t="inlineStr">
         <is>
-          <t>Si el usuario tiene que volver a escoger los idiomas cada vez que envia un mensaje, pierde tiempo y la conversacion se vuelve lenta.</t>
+          <t>Si el usuario tiene que configurar todo y decir su idioma antes de hablar, pierde tiempo y la conversacion no arranca de inmediato.</t>
         </is>
       </c>
       <c r="E5" s="53" t="inlineStr">
         <is>
-          <t>Empezar a hablar de una vez, sin repetir la configuracion.</t>
+          <t>Empezar a hablar de una vez.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Gestion de conversaciones</t>
+          <t>Gestion de conversaciones / Administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="G5" s="32" t="n"/>
+      <c r="H5" s="53" t="inlineStr">
+        <is>
+          <t>Liberaciones 1 y 2: en la prueba con usuarios, una persona nueva crea la conversacion y envia su primer mensaje en menos de 1 minuto; el idioma de origen se reconoce bien en el 90 % de los primeros mensajes.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="78" customHeight="1">
       <c r="A6" s="40" t="n"/>
       <c r="B6" s="37" t="n"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Conversar de forma fluida y continua sin reconfigurar los idiomas ni los parámetros en cada mensaje.</t>
+          <t>Mantener el contexto de toda la charla, para que cada respuesta se traduzca dentro del mismo hilo sin reconfigurar nada.</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">
         <is>
-          <t>Si la conversacion no guarda la configuracion ni los mensajes juntos, cada mensaje queda suelto y se pierde el hilo de lo que se ha dicho.</t>
+          <t>Si la conversacion no guarda la configuracion ni el hilo, cada mensaje queda suelto y se pierde el contexto de lo que se ha dicho.</t>
         </is>
       </c>
       <c r="E6" s="53" t="inlineStr">
@@ -1279,6 +1302,11 @@
         </is>
       </c>
       <c r="G6" s="32" t="n"/>
+      <c r="H6" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 2 (30/10/2026): en la prueba con usuarios hay conversaciones de 10 mensajes o mas sin reconfigurar idiomas.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="40" t="n"/>
@@ -1304,6 +1332,11 @@
         </is>
       </c>
       <c r="G7" s="32" t="n"/>
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 2: el 100 % de las conversaciones quedan en el historial y se pueden reabrir; en la encuesta final, 7 de cada 10 personas dicen que repasarlas les ayudo.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="40" t="n"/>
@@ -1328,9 +1361,10 @@
           <t>Cuenta de usuario</t>
         </is>
       </c>
-      <c r="G8" s="32" t="inlineStr">
-        <is>
-          <t>Impacto reescrito para que no suene a funcionalidad. Validar con Farid.</t>
+      <c r="G8" s="32" t="n"/>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3 (06/11/2026): 0 accesos de una persona a conversaciones de otra en las pruebas de seguridad; la persona puede eliminar su cuenta con todos sus datos.</t>
         </is>
       </c>
     </row>
@@ -1358,6 +1392,11 @@
         </is>
       </c>
       <c r="G9" s="32" t="n"/>
+      <c r="H9" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 1: el 100 % de los mensajes enviados por voz se escuchan traducidos; 7 de cada 10 personas de prueba califican la voz como comprensible.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1">
       <c r="A10" s="40" t="n"/>
@@ -1383,6 +1422,11 @@
         </is>
       </c>
       <c r="G10" s="32" t="n"/>
+      <c r="H10" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3: cualquier traduccion se reporta en 2 toques o menos y el reporte llega al administrador.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="78" customHeight="1">
       <c r="A11" s="40" t="n"/>
@@ -1393,17 +1437,17 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Participar en la conversación en el propio idioma y en igualdad de condiciones, sin necesidad de conocer ni operar la aplicación.</t>
+          <t>Participar en la conversacion en su propio idioma y en igualdad de condiciones, sin instalar la aplicacion ni crear una cuenta.</t>
         </is>
       </c>
       <c r="D11" s="53" t="inlineStr">
         <is>
-          <t>Si la otra persona tiene que instalar o aprender a manejar la app para contestar, la conversacion no arranca o ella queda en desventaja.</t>
+          <t>Si la otra persona tiene que instalar la app o crear una cuenta para contestar, la conversacion no arranca o ella queda en desventaja.</t>
         </is>
       </c>
       <c r="E11" s="53" t="inlineStr">
         <is>
-          <t>Que la otra persona hable en su idioma sin tocar la app.</t>
+          <t>Que la otra persona hable en su idioma con el celular del usuario, sin cuenta.</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
@@ -1412,6 +1456,11 @@
         </is>
       </c>
       <c r="G11" s="32" t="n"/>
+      <c r="H11" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 2: en la prueba con usuarios, la otra persona responde en su idioma con el celular del usuario, sin cuenta, en el 100 % de los casos.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="78" customHeight="1" thickBot="1">
       <c r="A12" s="40" t="n"/>
@@ -1422,7 +1471,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Gestionar la configuración de la aplicación a nivel de idiomas o regiones</t>
+          <t>Ampliar la oferta de idiomas y regiones con calidad confiable, activando solo los que ya traducen bien.</t>
         </is>
       </c>
       <c r="D12" s="53" t="inlineStr">
@@ -1440,9 +1489,10 @@
           <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
-      <c r="G12" s="32" t="inlineStr">
-        <is>
-          <t>Puede agregar valor pero esto lo hace un administrador?</t>
+      <c r="G12" s="32" t="n"/>
+      <c r="H12" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3: un idioma o region se agrega y activa sin cambiar codigo; solo se activan idiomas que pasan el glosario de prueba con 80 % o mas.</t>
         </is>
       </c>
     </row>
@@ -1474,6 +1524,11 @@
         </is>
       </c>
       <c r="G13" s="32" t="n"/>
+      <c r="H13" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3: el 100 % de los reportes abiertos se revisan (revisado o descartado) en menos de una semana.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="19" customHeight="1"/>
     <row r="17" ht="16" customHeight="1"/>
@@ -1488,11 +1543,12 @@
     <row r="26" ht="144" customHeight="1"/>
     <row r="27" ht="128" customHeight="1"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="G1:G3"/>
+    <mergeCell ref="H1:H3"/>
     <mergeCell ref="A4:A13"/>
-    <mergeCell ref="C1:E1"/>
     <mergeCell ref="B4:B10"/>
-    <mergeCell ref="G1:G3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1504,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1578,55 +1634,55 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C24</f>
+        <f>Entregables!C25</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D24</f>
+        <f>Entregables!D25</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E24</f>
+        <f>Entregables!E25</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F24</f>
+        <f>Entregables!F25</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C25</f>
+        <f>Entregables!C26</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D25</f>
+        <f>Entregables!D26</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E25</f>
+        <f>Entregables!E26</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F25</f>
+        <f>Entregables!F26</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18">
-        <f>Entregables!C26</f>
+        <f>Entregables!C27</f>
         <v/>
       </c>
       <c r="B10" s="18">
-        <f>Entregables!D26</f>
+        <f>Entregables!D27</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>Entregables!E26</f>
+        <f>Entregables!E27</f>
         <v/>
       </c>
       <c r="D10" s="18">
-        <f>Entregables!F26</f>
+        <f>Entregables!F27</f>
         <v/>
       </c>
     </row>
@@ -1636,6 +1692,34 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -1650,7 +1734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1786,7 +1870,7 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="70" t="n"/>
+      <c r="A3" s="34" t="n"/>
       <c r="B3" s="67" t="inlineStr">
         <is>
           <t>HU0002</t>
@@ -1838,7 +1922,7 @@
       </c>
     </row>
     <row r="4" ht="112" customHeight="1">
-      <c r="A4" s="70" t="n"/>
+      <c r="A4" s="34" t="n"/>
       <c r="B4" s="67" t="inlineStr">
         <is>
           <t>HU0003</t>
@@ -1891,7 +1975,7 @@
       </c>
     </row>
     <row r="5" ht="64" customHeight="1">
-      <c r="A5" s="70" t="n"/>
+      <c r="A5" s="34" t="n"/>
       <c r="B5" s="67" t="inlineStr">
         <is>
           <t>HU0004</t>
@@ -1943,7 +2027,7 @@
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="71" t="n"/>
+      <c r="A6" s="35" t="n"/>
       <c r="B6" s="67" t="inlineStr">
         <is>
           <t>HU0005</t>
@@ -2051,7 +2135,7 @@
       </c>
     </row>
     <row r="8" ht="80" customHeight="1">
-      <c r="A8" s="70" t="n"/>
+      <c r="A8" s="34" t="n"/>
       <c r="B8" s="67" t="inlineStr">
         <is>
           <t>HU0007</t>
@@ -2104,7 +2188,7 @@
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="70" t="n"/>
+      <c r="A9" s="34" t="n"/>
       <c r="B9" s="67" t="inlineStr">
         <is>
           <t>HU0008</t>
@@ -2156,7 +2240,7 @@
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="70" t="n"/>
+      <c r="A10" s="34" t="n"/>
       <c r="B10" s="67" t="inlineStr">
         <is>
           <t>HU0009</t>
@@ -2208,7 +2292,7 @@
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="70" t="n"/>
+      <c r="A11" s="34" t="n"/>
       <c r="B11" s="67" t="inlineStr">
         <is>
           <t>HU0010</t>
@@ -2260,7 +2344,7 @@
       </c>
     </row>
     <row r="12" ht="64" customHeight="1">
-      <c r="A12" s="70" t="n"/>
+      <c r="A12" s="34" t="n"/>
       <c r="B12" s="67" t="inlineStr">
         <is>
           <t>HU0011</t>
@@ -2313,7 +2397,7 @@
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="70" t="n"/>
+      <c r="A13" s="34" t="n"/>
       <c r="B13" s="67" t="inlineStr">
         <is>
           <t>HU0012</t>
@@ -2365,7 +2449,7 @@
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="70" t="n"/>
+      <c r="A14" s="34" t="n"/>
       <c r="B14" s="67" t="inlineStr">
         <is>
           <t>HU0013</t>
@@ -2417,7 +2501,7 @@
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="71" t="n"/>
+      <c r="A15" s="35" t="n"/>
       <c r="B15" s="67" t="inlineStr">
         <is>
           <t>HU0014</t>
@@ -2446,7 +2530,7 @@
       </c>
       <c r="H15" s="57" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="I15" s="57">
@@ -2454,7 +2538,7 @@
         <v/>
       </c>
       <c r="J15" s="57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15" s="58" t="inlineStr">
         <is>
@@ -2468,7 +2552,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="80" customHeight="1">
+    <row r="16" ht="112" customHeight="1">
       <c r="A16" s="67" t="inlineStr">
         <is>
           <t>Cuenta de usuario</t>
@@ -2522,12 +2606,13 @@
           <t>1. Cuando me registro con datos validos, entonces la cuenta se crea y entro a la app.
 2. La contrasena debe tener 8 o mas caracteres, una mayuscula, un numero y un simbolo; el correo debe tener formato valido.
 3. Debo tener 13 anos o mas; si no, veo 'debes tener al menos 13 anos'.
-4. Si el correo ya esta registrado, veo un aviso para iniciar sesion.</t>
+4. Si el correo ya esta registrado, veo un aviso para iniciar sesion.
+5. Debo aceptar la politica de tratamiento de datos (Ley 1581 de 2012); si no, no se crea la cuenta.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="64" customHeight="1">
-      <c r="A17" s="70" t="n"/>
+      <c r="A17" s="34" t="n"/>
       <c r="B17" s="67" t="inlineStr">
         <is>
           <t>HU0016</t>
@@ -2580,7 +2665,7 @@
       </c>
     </row>
     <row r="18" ht="96" customHeight="1">
-      <c r="A18" s="70" t="n"/>
+      <c r="A18" s="34" t="n"/>
       <c r="B18" s="67" t="inlineStr">
         <is>
           <t>HU0017</t>
@@ -2634,7 +2719,7 @@
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="71" t="n"/>
+      <c r="A19" s="34" t="n"/>
       <c r="B19" s="67" t="inlineStr">
         <is>
           <t>HU0018</t>
@@ -2671,11 +2756,11 @@
         <v/>
       </c>
       <c r="J19" s="57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" s="58" t="inlineStr">
         <is>
-          <t>Protege la cuenta en un dispositivo compartido; es de apoyo.</t>
+          <t>Protege la cuenta en un dispositivo compartido; solo tiene sentido despues de iniciar sesion, por eso va con ella en el sprint 3.</t>
         </is>
       </c>
       <c r="L19" s="69" t="inlineStr">
@@ -2685,25 +2770,21 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="67" t="inlineStr">
-        <is>
-          <t>Participacion del interlocutor</t>
-        </is>
-      </c>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="35" t="n"/>
       <c r="B20" s="67" t="inlineStr">
         <is>
-          <t>HU0019</t>
+          <t>HU0026</t>
         </is>
       </c>
       <c r="C20" s="68" t="inlineStr">
         <is>
-          <t>Recibir el mensaje traducido</t>
+          <t>Eliminar mi cuenta</t>
         </is>
       </c>
       <c r="D20" s="58" t="inlineStr">
         <is>
-          <t>Interlocutor</t>
+          <t>Cliente Traductor</t>
         </is>
       </c>
       <c r="E20" s="58">
@@ -2711,15 +2792,15 @@
         <v/>
       </c>
       <c r="F20" s="58">
-        <f>'Mapa de Impacto'!C11</f>
+        <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
       <c r="G20" s="57" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="H20" s="57" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="I20" s="57">
@@ -2727,30 +2808,35 @@
         <v/>
       </c>
       <c r="J20" s="57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="58" t="inlineStr">
         <is>
-          <t>Hace que la otra persona participe sin instalar ni operar la app.</t>
+          <t>Cumple el derecho al olvido (Ley 1581 de 2012): la persona controla sus datos.</t>
         </is>
       </c>
       <c r="L20" s="69" t="inlineStr">
         <is>
-          <t>1. Dado que la otra persona responde (se escribe como 'Otra persona'), entonces su mensaje se traduce a mi idioma y se muestra a la izquierda, junto a su original.
-2. La otra persona no necesita instalar la app ni tener cuenta.</t>
+          <t>1. Dado que estoy en mi perfil, cuando elijo eliminar mi cuenta, entonces la app me pide mi contrasena y me avisa que no se puede deshacer.
+2. Al confirmar, se borran mi cuenta, mis conversaciones, mis mensajes y mis reportes, y vuelvo a la pantalla de bienvenida.
+3. Con una contrasena incorrecta la cuenta no se elimina.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="71" t="n"/>
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>Participacion del interlocutor</t>
+        </is>
+      </c>
       <c r="B21" s="67" t="inlineStr">
         <is>
-          <t>HU0020</t>
+          <t>HU0019</t>
         </is>
       </c>
       <c r="C21" s="68" t="inlineStr">
         <is>
-          <t>Responder en mi idioma</t>
+          <t>Recibir el mensaje traducido</t>
         </is>
       </c>
       <c r="D21" s="58" t="inlineStr">
@@ -2767,11 +2853,11 @@
         <v/>
       </c>
       <c r="G21" s="57" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H21" s="57" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I21" s="57">
@@ -2783,118 +2869,170 @@
       </c>
       <c r="K21" s="58" t="inlineStr">
         <is>
+          <t>Hace que la otra persona participe sin instalar ni operar la app.</t>
+        </is>
+      </c>
+      <c r="L21" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que la otra persona responde (se elige 'Otra persona' y se le pasa el celular), entonces su mensaje se traduce a mi idioma y se muestra a la izquierda, junto a su original.
+2. La otra persona no necesita instalar la app ni crear una cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="35" t="n"/>
+      <c r="B22" s="67" t="inlineStr">
+        <is>
+          <t>HU0020</t>
+        </is>
+      </c>
+      <c r="C22" s="68" t="inlineStr">
+        <is>
+          <t>Responder en mi idioma</t>
+        </is>
+      </c>
+      <c r="D22" s="58" t="inlineStr">
+        <is>
+          <t>Interlocutor</t>
+        </is>
+      </c>
+      <c r="E22" s="58">
+        <f>C22</f>
+        <v/>
+      </c>
+      <c r="F22" s="58">
+        <f>'Mapa de Impacto'!C11</f>
+        <v/>
+      </c>
+      <c r="G22" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="H22" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I22" s="57">
+        <f>VLOOKUP(H22,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J22" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="58" t="inlineStr">
+        <is>
           <t>Cierra el dialogo en ambos sentidos.</t>
         </is>
       </c>
-      <c r="L21" s="69" t="inlineStr">
+      <c r="L22" s="69" t="inlineStr">
         <is>
           <t>1. Cuando la otra persona escribe en su propio idioma, entonces su respuesta se traduce al idioma de la conversacion.
 2. Para responder ya debe haberse reconocido mi idioma con mi primer mensaje.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="67" t="inlineStr">
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="67" t="inlineStr">
         <is>
           <t>Reportes</t>
         </is>
       </c>
-      <c r="B22" s="67" t="inlineStr">
+      <c r="B23" s="67" t="inlineStr">
         <is>
           <t>HU0021</t>
         </is>
       </c>
-      <c r="C22" s="68" t="inlineStr">
+      <c r="C23" s="68" t="inlineStr">
         <is>
           <t>Reportar una mala traduccion</t>
         </is>
       </c>
-      <c r="D22" s="58" t="inlineStr">
+      <c r="D23" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E22" s="58">
-        <f>C22</f>
-        <v/>
-      </c>
-      <c r="F22" s="58">
+      <c r="E23" s="58">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="F23" s="58">
         <f>'Mapa de Impacto'!C10</f>
         <v/>
       </c>
-      <c r="G22" s="57" t="n">
+      <c r="G23" s="57" t="n">
         <v>18</v>
       </c>
-      <c r="H22" s="57" t="inlineStr">
+      <c r="H23" s="57" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I22" s="57">
-        <f>VLOOKUP(H22,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J22" s="57" t="n">
+      <c r="I23" s="57">
+        <f>VLOOKUP(H23,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J23" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="K22" s="58" t="inlineStr">
+      <c r="K23" s="58" t="inlineStr">
         <is>
           <t>Alimenta la mejora de calidad con casos reales.</t>
         </is>
       </c>
-      <c r="L22" s="69" t="inlineStr">
+      <c r="L23" s="69" t="inlineStr">
         <is>
           <t>1. Cuando reporto una traduccion con un motivo de 3 a 500 caracteres, entonces el reporte se guarda y el mensaje queda marcado como 'Reportado'.
 2. Solo puedo reportar una vez la misma traduccion y solo las de mis conversaciones.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="64" customHeight="1">
-      <c r="A23" s="71" t="n"/>
-      <c r="B23" s="67" t="inlineStr">
+    <row r="24" ht="64" customHeight="1">
+      <c r="A24" s="35" t="n"/>
+      <c r="B24" s="67" t="inlineStr">
         <is>
           <t>HU0022</t>
         </is>
       </c>
-      <c r="C23" s="68" t="inlineStr">
+      <c r="C24" s="68" t="inlineStr">
         <is>
           <t>Revisar los reportes de mala traduccion</t>
         </is>
       </c>
-      <c r="D23" s="58" t="inlineStr">
+      <c r="D24" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E23" s="58">
-        <f>C23</f>
-        <v/>
-      </c>
-      <c r="F23" s="58">
+      <c r="E24" s="58">
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="F24" s="58">
         <f>'Mapa de Impacto'!C13</f>
         <v/>
       </c>
-      <c r="G23" s="57" t="n">
+      <c r="G24" s="57" t="n">
         <v>23</v>
       </c>
-      <c r="H23" s="57" t="inlineStr">
+      <c r="H24" s="57" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I23" s="57">
-        <f>VLOOKUP(H23,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J23" s="57" t="n">
+      <c r="I24" s="57">
+        <f>VLOOKUP(H24,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J24" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="K23" s="58" t="inlineStr">
+      <c r="K24" s="58" t="inlineStr">
         <is>
           <t>Permite priorizar que mejorar primero.</t>
         </is>
       </c>
-      <c r="L23" s="69" t="inlineStr">
+      <c r="L24" s="69" t="inlineStr">
         <is>
           <t>1. Dado que soy administrador, cuando abro los reportes, entonces veo el original, la traduccion, el motivo y la sugerencia, y puedo filtrar por abiertos, revisados o descartados.
 2. Puedo marcar un reporte como revisado o descartado.
@@ -2902,108 +3040,108 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="67" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="67" t="inlineStr">
         <is>
           <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
-      <c r="B24" s="67" t="inlineStr">
+      <c r="B25" s="67" t="inlineStr">
         <is>
           <t>HU0023</t>
         </is>
       </c>
-      <c r="C24" s="68" t="inlineStr">
+      <c r="C25" s="68" t="inlineStr">
         <is>
           <t>Consultar los idiomas disponibles</t>
         </is>
       </c>
-      <c r="D24" s="58" t="inlineStr">
+      <c r="D25" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E24" s="58">
-        <f>C24</f>
-        <v/>
-      </c>
-      <c r="F24" s="58">
+      <c r="E25" s="58">
+        <f>C25</f>
+        <v/>
+      </c>
+      <c r="F25" s="58">
         <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
-      <c r="G24" s="57" t="n">
+      <c r="G25" s="57" t="n">
         <v>13</v>
       </c>
-      <c r="H24" s="57" t="inlineStr">
+      <c r="H25" s="57" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="I24" s="57">
-        <f>VLOOKUP(H24,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J24" s="57" t="n">
+      <c r="I25" s="57">
+        <f>VLOOKUP(H25,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J25" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="K24" s="58" t="inlineStr">
+      <c r="K25" s="58" t="inlineStr">
         <is>
           <t>Muestra con que idiomas se puede hablar antes de empezar.</t>
         </is>
       </c>
-      <c r="L24" s="69" t="inlineStr">
+      <c r="L25" s="69" t="inlineStr">
         <is>
           <t>1. Cuando abro la configuracion de una conversacion, entonces veo solo los idiomas activos con sus regiones.
 2. Los idiomas desactivados no aparecen en la lista.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="80" customHeight="1">
-      <c r="A25" s="70" t="n"/>
-      <c r="B25" s="67" t="inlineStr">
+    <row r="26" ht="80" customHeight="1">
+      <c r="A26" s="34" t="n"/>
+      <c r="B26" s="67" t="inlineStr">
         <is>
           <t>HU0024</t>
         </is>
       </c>
-      <c r="C25" s="68" t="inlineStr">
+      <c r="C26" s="68" t="inlineStr">
         <is>
           <t>Agregar un idioma o una region</t>
         </is>
       </c>
-      <c r="D25" s="58" t="inlineStr">
+      <c r="D26" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E25" s="58">
-        <f>C25</f>
-        <v/>
-      </c>
-      <c r="F25" s="58">
+      <c r="E26" s="58">
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="F26" s="58">
         <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
-      <c r="G25" s="57" t="n">
+      <c r="G26" s="57" t="n">
         <v>24</v>
       </c>
-      <c r="H25" s="57" t="inlineStr">
+      <c r="H26" s="57" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I25" s="57">
-        <f>VLOOKUP(H25,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J25" s="57" t="n">
+      <c r="I26" s="57">
+        <f>VLOOKUP(H26,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J26" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="K25" s="58" t="inlineStr">
+      <c r="K26" s="58" t="inlineStr">
         <is>
           <t>Hace crecer el servicio a mas personas.</t>
         </is>
       </c>
-      <c r="L25" s="69" t="inlineStr">
+      <c r="L26" s="69" t="inlineStr">
         <is>
           <t>1. Dado que soy administrador, cuando agrego un idioma, entonces necesita un nombre unico y un codigo de 2 a 5 letras, y queda desactivado hasta que lo active.
 2. Una region no puede repetirse dentro del mismo pais; si el pais no existe, debo indicar su codigo de 2 letras.
@@ -3011,66 +3149,98 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="71" t="n"/>
-      <c r="B26" s="67" t="inlineStr">
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="35" t="n"/>
+      <c r="B27" s="67" t="inlineStr">
         <is>
           <t>HU0025</t>
         </is>
       </c>
-      <c r="C26" s="68" t="inlineStr">
+      <c r="C27" s="68" t="inlineStr">
         <is>
           <t>Activar o desactivar un idioma o una region</t>
         </is>
       </c>
-      <c r="D26" s="58" t="inlineStr">
+      <c r="D27" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E26" s="58">
-        <f>C26</f>
-        <v/>
-      </c>
-      <c r="F26" s="58">
+      <c r="E27" s="58">
+        <f>C27</f>
+        <v/>
+      </c>
+      <c r="F27" s="58">
         <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
-      <c r="G26" s="57" t="n">
+      <c r="G27" s="57" t="n">
         <v>25</v>
       </c>
-      <c r="H26" s="57" t="inlineStr">
+      <c r="H27" s="57" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="I26" s="57">
-        <f>VLOOKUP(H26,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J26" s="57" t="n">
+      <c r="I27" s="57">
+        <f>VLOOKUP(H27,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J27" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="K26" s="58" t="inlineStr">
+      <c r="K27" s="58" t="inlineStr">
         <is>
           <t>Controla que idiomas se ofrecen con calidad suficiente.</t>
         </is>
       </c>
-      <c r="L26" s="69" t="inlineStr">
+      <c r="L27" s="69" t="inlineStr">
         <is>
           <t>1. Cuando activo un idioma, entonces aparece en el catalogo para crear conversaciones; cuando lo desactivo, deja de aparecer.
 2. Las conversaciones ya creadas no se ven afectadas.</t>
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A25:A27"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A16:A20"/>
+    <mergeCell ref="A23:A24"/>
     <mergeCell ref="A7:A15"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A21:A22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" location="'Traductor de mensajes'!A1" display="Traductor de mensajes"/>
@@ -3299,13 +3469,13 @@
       </c>
       <c r="E14" s="65" t="inlineStr">
         <is>
-          <t>HU0001, HU0002, HU0003, HU0004, HU0005, HU0006</t>
-        </is>
-      </c>
-      <c r="F14" s="73" t="n">
+          <t>HU0003, HU0002, HU0001, HU0004, HU0005, HU0006</t>
+        </is>
+      </c>
+      <c r="F14" s="75" t="n">
         <v>46314</v>
       </c>
-      <c r="G14" s="73" t="n">
+      <c r="G14" s="75" t="n">
         <v>46318</v>
       </c>
       <c r="H14" s="62" t="inlineStr">
@@ -3332,13 +3502,13 @@
       </c>
       <c r="E15" s="65" t="inlineStr">
         <is>
-          <t>HU0007, HU0008, HU0009, HU0010, HU0011, HU0012, HU0013, HU0018, HU0019, HU0020, HU0023, HU0025</t>
-        </is>
-      </c>
-      <c r="F15" s="73" t="n">
+          <t>HU0007, HU0008, HU0009, HU0010, HU0019, HU0020, HU0023, HU0011, HU0012, HU0013, HU0014, HU0025</t>
+        </is>
+      </c>
+      <c r="F15" s="75" t="n">
         <v>46321</v>
       </c>
-      <c r="G15" s="73" t="n">
+      <c r="G15" s="75" t="n">
         <v>46325</v>
       </c>
       <c r="H15" s="62" t="inlineStr">
@@ -3365,13 +3535,13 @@
       </c>
       <c r="E16" s="65" t="inlineStr">
         <is>
-          <t>HU0014, HU0015, HU0016, HU0017, HU0021, HU0022, HU0024</t>
-        </is>
-      </c>
-      <c r="F16" s="73" t="n">
+          <t>HU0015, HU0016, HU0021, HU0017, HU0018, HU0022, HU0024, HU0026</t>
+        </is>
+      </c>
+      <c r="F16" s="75" t="n">
         <v>46328</v>
       </c>
-      <c r="G16" s="73" t="n">
+      <c r="G16" s="75" t="n">
         <v>46332</v>
       </c>
       <c r="H16" s="62" t="inlineStr">
@@ -3515,10 +3685,10 @@
       <c r="B5" s="64" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="74" t="n">
+      <c r="C5" s="76" t="n">
         <v>46314</v>
       </c>
-      <c r="D5" s="74" t="n">
+      <c r="D5" s="76" t="n">
         <v>46318</v>
       </c>
       <c r="E5" s="65" t="inlineStr">
@@ -3533,7 +3703,7 @@
       </c>
       <c r="G5" s="65" t="inlineStr">
         <is>
-          <t>HU0001, HU0002, HU0003, HU0004, HU0005, HU0006</t>
+          <t>HU0003, HU0002, HU0001, HU0004, HU0005, HU0006</t>
         </is>
       </c>
       <c r="H5" s="64">
@@ -3550,10 +3720,10 @@
       <c r="B6" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="76" t="n">
         <v>46321</v>
       </c>
-      <c r="D6" s="74" t="n">
+      <c r="D6" s="76" t="n">
         <v>46325</v>
       </c>
       <c r="E6" s="65" t="inlineStr">
@@ -3563,12 +3733,12 @@
       </c>
       <c r="F6" s="65" t="inlineStr">
         <is>
-          <t>El usuario organiza sus conversaciones (reconocer idioma, crear, hilo continuo, historial, renombrar), la otra persona participa y el administrador controla que idiomas se activan.</t>
+          <t>El usuario organiza sus conversaciones (reconocer idioma, crear, hilo continuo, historial, renombrar y eliminar), la otra persona participa y el administrador controla que idiomas se activan.</t>
         </is>
       </c>
       <c r="G6" s="65" t="inlineStr">
         <is>
-          <t>HU0007, HU0008, HU0009, HU0010, HU0011, HU0012, HU0013, HU0018, HU0019, HU0020, HU0023, HU0025</t>
+          <t>HU0007, HU0008, HU0009, HU0010, HU0019, HU0020, HU0023, HU0011, HU0012, HU0013, HU0014, HU0025</t>
         </is>
       </c>
       <c r="H6" s="64">
@@ -3585,10 +3755,10 @@
       <c r="B7" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="74" t="n">
+      <c r="C7" s="76" t="n">
         <v>46328</v>
       </c>
-      <c r="D7" s="74" t="n">
+      <c r="D7" s="76" t="n">
         <v>46332</v>
       </c>
       <c r="E7" s="65" t="inlineStr">
@@ -3598,12 +3768,12 @@
       </c>
       <c r="F7" s="65" t="inlineStr">
         <is>
-          <t>Registro, inicio de sesion y recuperacion de contrasena, eliminar conversaciones, reportar y revisar malas traducciones, y agregar idiomas y regiones.</t>
+          <t>Registro con consentimiento de datos, inicio y cierre de sesion, recuperacion de contrasena, eliminar la cuenta, reportar y revisar malas traducciones, y agregar idiomas y regiones.</t>
         </is>
       </c>
       <c r="G7" s="65" t="inlineStr">
         <is>
-          <t>HU0014, HU0015, HU0016, HU0017, HU0021, HU0022, HU0024</t>
+          <t>HU0015, HU0016, HU0021, HU0017, HU0018, HU0022, HU0024, HU0026</t>
         </is>
       </c>
       <c r="H7" s="64">
@@ -3629,7 +3799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3791,6 +3961,33 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -3805,7 +4002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4039,6 +4236,29 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4053,7 +4273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4197,6 +4417,51 @@
         <v/>
       </c>
     </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="18">
+        <f>Entregables!C20</f>
+        <v/>
+      </c>
+      <c r="B12" s="18">
+        <f>Entregables!D20</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>Entregables!E20</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
+        <f>Entregables!F20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4211,7 +4476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4285,37 +4550,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C20</f>
+        <f>Entregables!C21</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D20</f>
+        <f>Entregables!D21</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E20</f>
+        <f>Entregables!E21</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F20</f>
+        <f>Entregables!F21</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C21</f>
+        <f>Entregables!C22</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D21</f>
+        <f>Entregables!D22</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E21</f>
+        <f>Entregables!E22</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F21</f>
+        <f>Entregables!F22</f>
         <v/>
       </c>
     </row>
@@ -4331,6 +4596,34 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4345,7 +4638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4419,37 +4712,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C22</f>
+        <f>Entregables!C23</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D22</f>
+        <f>Entregables!D23</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E22</f>
+        <f>Entregables!E23</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F22</f>
+        <f>Entregables!F23</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C23</f>
+        <f>Entregables!C24</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D23</f>
+        <f>Entregables!D24</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E23</f>
+        <f>Entregables!E24</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F23</f>
+        <f>Entregables!F24</f>
         <v/>
       </c>
     </row>
@@ -4465,6 +4758,34 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>

</xml_diff>

<commit_message>
docs(requerimientos): impactos sin doble 'para' y HU0022 sin repetir la historia (#1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -1223,7 +1223,7 @@
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
-          <t>Traducir un mensaje de un idioma origen a un idioma destino en tiempo real, para interactuar fácil y rápidamente con personas que hablan otro idioma conservando el contexto cultural, el tono y los modismos.</t>
+          <t>Interactuar facil y rapidamente con personas que hablan otro idioma, traduciendo cada mensaje en tiempo real y conservando el contexto cultural, el tono y los modismos.</t>
         </is>
       </c>
       <c r="D4" s="43" t="inlineStr">
@@ -1283,7 +1283,7 @@
       <c r="B6" s="37" t="n"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Mantener el contexto de toda la charla, para que cada respuesta se traduzca dentro del mismo hilo sin reconfigurar nada.</t>
+          <t>Mantener el contexto de toda la charla, de modo que cada respuesta se traduzca dentro del mismo hilo sin reconfigurar nada.</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">
@@ -1343,7 +1343,7 @@
       <c r="B8" s="37" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Acceder a la cuenta de forma segura, para que las conversaciones y la configuracion queden guardadas y solo el usuario pueda verlas.</t>
+          <t>Tener las conversaciones y la configuracion guardadas en una cuenta segura que solo el usuario puede ver.</t>
         </is>
       </c>
       <c r="D8" s="53" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C13" s="56" t="inlineStr">
         <is>
-          <t>Revisar los reportes de mala traduccion que envian los clientes, para decidir que mejoras priorizar en el servicio.</t>
+          <t>Decidir que mejoras priorizar en el servicio a partir de los reportes de mala traduccion que envian los clientes.</t>
         </is>
       </c>
       <c r="D13" s="53" t="inlineStr">
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1692,34 +1692,6 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -1734,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3201,38 +3173,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A25:A27"/>
@@ -3799,7 +3739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3961,33 +3901,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4002,7 +3915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4236,29 +4149,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4273,7 +4163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4435,33 +4325,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4476,7 +4339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4596,34 +4459,6 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
@@ -4638,7 +4473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4758,34 +4593,6 @@
       <c r="C11" s="18" t="n"/>
       <c r="D11" s="18" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>

</xml_diff>

<commit_message>
fix: correcciones de la revision para la sustentacion (#28)
Closes #1

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -24,9 +24,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -537,7 +536,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -727,10 +726,16 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1098,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="45.1640625" customWidth="1" min="1" max="1"/>
@@ -1108,6 +1113,7 @@
     <col width="48.33203125" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -1138,6 +1144,11 @@
           <t>DUDAS</t>
         </is>
       </c>
+      <c r="H1" s="41" t="inlineStr">
+        <is>
+          <t>Indicador SMART (como se mide y para cuando)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1171,6 +1182,7 @@
         </is>
       </c>
       <c r="G2" s="37" t="n"/>
+      <c r="H2" s="37" t="n"/>
     </row>
     <row r="3" ht="17" customHeight="1" thickBot="1">
       <c r="A3" s="5" t="inlineStr">
@@ -1196,11 +1208,12 @@
         </is>
       </c>
       <c r="G3" s="38" t="n"/>
+      <c r="H3" s="38" t="n"/>
     </row>
     <row r="4" ht="78" customHeight="1">
       <c r="A4" s="39" t="inlineStr">
         <is>
-          <t>Para cualquier persona que necesita expresarse verbal o textualmente en un idioma que no conoce o domina, incluyendo no solo su mensaje sino también cualquier modismo o jerga cultural utilizada sin perder el significado o contexto del mismo, TalkLate es una aplicación móvil que está diseñada para ofrecer una experiencia de traducción que va más allá de la conversión literal de palabras, ya que considera el contexto, las emociones, los matices culturales y las intenciones detrás del lenguaje, permitiendo una comunicación más natural y significativa. A diferencia de Meta Seamless, Deepl Translator, TimeKettle, Lilt y Kudo AI, nuestro producto se distingue por su enfoque en la conexión profunda, permitiendo a los usuarios expresarse auténticamente en otro idioma, con foco inicial en ciertas regiones y acentos específicos del inglés y el español, y con una visión evolutiva para soportar con el paso del tiempo otros lenguajes con sus respectivos modismos y características, sin perder la espontaneidad ni la riqueza de su comunicación original.</t>
+          <t>Objetivo (SMART): al cierre de la liberacion 3 (06/11/2026), al menos 10 personas de prueba sostienen cada una una conversacion de 10 mensajes o mas con alguien que habla otro idioma (espanol-ingles), con menos del 20 % de traducciones reportadas como malas y un tiempo por traduccion de 3 segundos o menos (p95). Vision: ver contexto.md.</t>
         </is>
       </c>
       <c r="B4" s="36" t="inlineStr">
@@ -1210,7 +1223,7 @@
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
-          <t>Traducir un mensaje de un idioma origen a un idioma destino en tiempo real, para interactuar fácil y rápidamente con personas que hablan otro idioma conservando el contexto cultural, el tono y los modismos.</t>
+          <t>Interactuar facil y rapidamente con personas que hablan otro idioma, traduciendo cada mensaje en tiempo real y conservando el contexto cultural, el tono y los modismos.</t>
         </is>
       </c>
       <c r="D4" s="43" t="inlineStr">
@@ -1229,43 +1242,53 @@
         </is>
       </c>
       <c r="G4" s="32" t="n"/>
+      <c r="H4" s="43" t="inlineStr">
+        <is>
+          <t>Liberacion 1 (23/10/2026): el 80 % de los modismos del glosario de prueba se traducen con su equivalente cultural y en 3 segundos o menos (p95). Se mide con npm run medir.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="78" customHeight="1">
       <c r="A5" s="40" t="n"/>
       <c r="B5" s="37" t="n"/>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Comunicarse de inmediato sin tener que repetir la configuración de idioma en cada mensaje.</t>
+          <t>Empezar a conversar en menos de un minuto, configurando idioma y region destino una sola vez y sin tener que indicar el idioma propio.</t>
         </is>
       </c>
       <c r="D5" s="53" t="inlineStr">
         <is>
-          <t>Si el usuario tiene que volver a escoger los idiomas cada vez que envia un mensaje, pierde tiempo y la conversacion se vuelve lenta.</t>
+          <t>Si el usuario tiene que configurar todo y decir su idioma antes de hablar, pierde tiempo y la conversacion no arranca de inmediato.</t>
         </is>
       </c>
       <c r="E5" s="53" t="inlineStr">
         <is>
-          <t>Empezar a hablar de una vez, sin repetir la configuracion.</t>
+          <t>Empezar a hablar de una vez.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Gestion de conversaciones</t>
+          <t>Gestion de conversaciones / Administracion de idiomas y regiones</t>
         </is>
       </c>
       <c r="G5" s="32" t="n"/>
+      <c r="H5" s="53" t="inlineStr">
+        <is>
+          <t>Liberaciones 1 y 2: en la prueba con usuarios, una persona nueva crea la conversacion y envia su primer mensaje en menos de 1 minuto; el idioma de origen se reconoce bien en el 90 % de los primeros mensajes.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="78" customHeight="1">
       <c r="A6" s="40" t="n"/>
       <c r="B6" s="37" t="n"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Conversar de forma fluida y continua sin reconfigurar los idiomas ni los parámetros en cada mensaje.</t>
+          <t>Mantener el contexto de toda la charla, de modo que cada respuesta se traduzca dentro del mismo hilo sin reconfigurar nada.</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">
         <is>
-          <t>Si la conversacion no guarda la configuracion ni los mensajes juntos, cada mensaje queda suelto y se pierde el hilo de lo que se ha dicho.</t>
+          <t>Si la conversacion no guarda la configuracion ni el hilo, cada mensaje queda suelto y se pierde el contexto de lo que se ha dicho.</t>
         </is>
       </c>
       <c r="E6" s="53" t="inlineStr">
@@ -1279,6 +1302,11 @@
         </is>
       </c>
       <c r="G6" s="32" t="n"/>
+      <c r="H6" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 2 (30/10/2026): en la prueba con usuarios hay conversaciones de 10 mensajes o mas sin reconfigurar idiomas.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="40" t="n"/>
@@ -1304,13 +1332,18 @@
         </is>
       </c>
       <c r="G7" s="32" t="n"/>
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 2: el 100 % de las conversaciones quedan en el historial y se pueden reabrir; en la encuesta final, 7 de cada 10 personas dicen que repasarlas les ayudo.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="40" t="n"/>
       <c r="B8" s="37" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Acceder a la cuenta de forma segura, para que las conversaciones y la configuracion queden guardadas y solo el usuario pueda verlas.</t>
+          <t>Tener las conversaciones y la configuracion guardadas en una cuenta segura que solo el usuario puede ver.</t>
         </is>
       </c>
       <c r="D8" s="53" t="inlineStr">
@@ -1328,9 +1361,10 @@
           <t>Cuenta de usuario</t>
         </is>
       </c>
-      <c r="G8" s="32" t="inlineStr">
-        <is>
-          <t>Impacto reescrito para que no suene a funcionalidad. Validar con Farid.</t>
+      <c r="G8" s="32" t="n"/>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3 (06/11/2026): 0 accesos de una persona a conversaciones de otra en las pruebas de seguridad; la persona puede eliminar su cuenta con todos sus datos.</t>
         </is>
       </c>
     </row>
@@ -1358,6 +1392,11 @@
         </is>
       </c>
       <c r="G9" s="32" t="n"/>
+      <c r="H9" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 1: el 100 % de los mensajes enviados por voz se escuchan traducidos; 7 de cada 10 personas de prueba califican la voz como comprensible.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1">
       <c r="A10" s="40" t="n"/>
@@ -1383,6 +1422,11 @@
         </is>
       </c>
       <c r="G10" s="32" t="n"/>
+      <c r="H10" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3: cualquier traduccion se reporta en 2 toques o menos y el reporte llega al administrador.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="78" customHeight="1">
       <c r="A11" s="40" t="n"/>
@@ -1393,17 +1437,17 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Participar en la conversación en el propio idioma y en igualdad de condiciones, sin necesidad de conocer ni operar la aplicación.</t>
+          <t>Participar en la conversacion en su propio idioma y en igualdad de condiciones, sin instalar la aplicacion ni crear una cuenta.</t>
         </is>
       </c>
       <c r="D11" s="53" t="inlineStr">
         <is>
-          <t>Si la otra persona tiene que instalar o aprender a manejar la app para contestar, la conversacion no arranca o ella queda en desventaja.</t>
+          <t>Si la otra persona tiene que instalar la app o crear una cuenta para contestar, la conversacion no arranca o ella queda en desventaja.</t>
         </is>
       </c>
       <c r="E11" s="53" t="inlineStr">
         <is>
-          <t>Que la otra persona hable en su idioma sin tocar la app.</t>
+          <t>Que la otra persona hable en su idioma con el celular del usuario, sin cuenta.</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
@@ -1412,6 +1456,11 @@
         </is>
       </c>
       <c r="G11" s="32" t="n"/>
+      <c r="H11" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 2: en la prueba con usuarios, la otra persona responde en su idioma con el celular del usuario, sin cuenta, en el 100 % de los casos.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="78" customHeight="1" thickBot="1">
       <c r="A12" s="40" t="n"/>
@@ -1422,7 +1471,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Gestionar la configuración de la aplicación a nivel de idiomas o regiones</t>
+          <t>Ampliar la oferta de idiomas y regiones con calidad confiable, activando solo los que ya traducen bien.</t>
         </is>
       </c>
       <c r="D12" s="53" t="inlineStr">
@@ -1440,9 +1489,10 @@
           <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
-      <c r="G12" s="32" t="inlineStr">
-        <is>
-          <t>Puede agregar valor pero esto lo hace un administrador?</t>
+      <c r="G12" s="32" t="n"/>
+      <c r="H12" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3: un idioma o region se agrega y activa sin cambiar codigo; solo se activan idiomas que pasan el glosario de prueba con 80 % o mas.</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1505,7 @@
       </c>
       <c r="C13" s="56" t="inlineStr">
         <is>
-          <t>Revisar los reportes de mala traduccion que envian los clientes, para decidir que mejoras priorizar en el servicio.</t>
+          <t>Decidir que mejoras priorizar en el servicio a partir de los reportes de mala traduccion que envian los clientes.</t>
         </is>
       </c>
       <c r="D13" s="53" t="inlineStr">
@@ -1474,6 +1524,11 @@
         </is>
       </c>
       <c r="G13" s="32" t="n"/>
+      <c r="H13" s="53" t="inlineStr">
+        <is>
+          <t>Liberacion 3: el 100 % de los reportes abiertos se revisan (revisado o descartado) en menos de una semana.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="19" customHeight="1"/>
     <row r="17" ht="16" customHeight="1"/>
@@ -1488,11 +1543,12 @@
     <row r="26" ht="144" customHeight="1"/>
     <row r="27" ht="128" customHeight="1"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="G1:G3"/>
+    <mergeCell ref="H1:H3"/>
     <mergeCell ref="A4:A13"/>
-    <mergeCell ref="C1:E1"/>
     <mergeCell ref="B4:B10"/>
-    <mergeCell ref="G1:G3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1578,55 +1634,55 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C24</f>
+        <f>Entregables!C25</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D24</f>
+        <f>Entregables!D25</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E24</f>
+        <f>Entregables!E25</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F24</f>
+        <f>Entregables!F25</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C25</f>
+        <f>Entregables!C26</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D25</f>
+        <f>Entregables!D26</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E25</f>
+        <f>Entregables!E26</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F25</f>
+        <f>Entregables!F26</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="18">
-        <f>Entregables!C26</f>
+        <f>Entregables!C27</f>
         <v/>
       </c>
       <c r="B10" s="18">
-        <f>Entregables!D26</f>
+        <f>Entregables!D27</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>Entregables!E26</f>
+        <f>Entregables!E27</f>
         <v/>
       </c>
       <c r="D10" s="18">
-        <f>Entregables!F26</f>
+        <f>Entregables!F27</f>
         <v/>
       </c>
     </row>
@@ -1650,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="40" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1786,7 +1842,7 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="70" t="n"/>
+      <c r="A3" s="34" t="n"/>
       <c r="B3" s="67" t="inlineStr">
         <is>
           <t>HU0002</t>
@@ -1838,7 +1894,7 @@
       </c>
     </row>
     <row r="4" ht="112" customHeight="1">
-      <c r="A4" s="70" t="n"/>
+      <c r="A4" s="34" t="n"/>
       <c r="B4" s="67" t="inlineStr">
         <is>
           <t>HU0003</t>
@@ -1891,7 +1947,7 @@
       </c>
     </row>
     <row r="5" ht="64" customHeight="1">
-      <c r="A5" s="70" t="n"/>
+      <c r="A5" s="34" t="n"/>
       <c r="B5" s="67" t="inlineStr">
         <is>
           <t>HU0004</t>
@@ -1943,7 +1999,7 @@
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="71" t="n"/>
+      <c r="A6" s="35" t="n"/>
       <c r="B6" s="67" t="inlineStr">
         <is>
           <t>HU0005</t>
@@ -2051,7 +2107,7 @@
       </c>
     </row>
     <row r="8" ht="80" customHeight="1">
-      <c r="A8" s="70" t="n"/>
+      <c r="A8" s="34" t="n"/>
       <c r="B8" s="67" t="inlineStr">
         <is>
           <t>HU0007</t>
@@ -2104,7 +2160,7 @@
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="70" t="n"/>
+      <c r="A9" s="34" t="n"/>
       <c r="B9" s="67" t="inlineStr">
         <is>
           <t>HU0008</t>
@@ -2156,7 +2212,7 @@
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="70" t="n"/>
+      <c r="A10" s="34" t="n"/>
       <c r="B10" s="67" t="inlineStr">
         <is>
           <t>HU0009</t>
@@ -2208,7 +2264,7 @@
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="70" t="n"/>
+      <c r="A11" s="34" t="n"/>
       <c r="B11" s="67" t="inlineStr">
         <is>
           <t>HU0010</t>
@@ -2260,7 +2316,7 @@
       </c>
     </row>
     <row r="12" ht="64" customHeight="1">
-      <c r="A12" s="70" t="n"/>
+      <c r="A12" s="34" t="n"/>
       <c r="B12" s="67" t="inlineStr">
         <is>
           <t>HU0011</t>
@@ -2313,7 +2369,7 @@
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="70" t="n"/>
+      <c r="A13" s="34" t="n"/>
       <c r="B13" s="67" t="inlineStr">
         <is>
           <t>HU0012</t>
@@ -2365,7 +2421,7 @@
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="70" t="n"/>
+      <c r="A14" s="34" t="n"/>
       <c r="B14" s="67" t="inlineStr">
         <is>
           <t>HU0013</t>
@@ -2417,7 +2473,7 @@
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="71" t="n"/>
+      <c r="A15" s="35" t="n"/>
       <c r="B15" s="67" t="inlineStr">
         <is>
           <t>HU0014</t>
@@ -2446,7 +2502,7 @@
       </c>
       <c r="H15" s="57" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="I15" s="57">
@@ -2454,7 +2510,7 @@
         <v/>
       </c>
       <c r="J15" s="57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15" s="58" t="inlineStr">
         <is>
@@ -2468,7 +2524,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="80" customHeight="1">
+    <row r="16" ht="112" customHeight="1">
       <c r="A16" s="67" t="inlineStr">
         <is>
           <t>Cuenta de usuario</t>
@@ -2522,12 +2578,13 @@
           <t>1. Cuando me registro con datos validos, entonces la cuenta se crea y entro a la app.
 2. La contrasena debe tener 8 o mas caracteres, una mayuscula, un numero y un simbolo; el correo debe tener formato valido.
 3. Debo tener 13 anos o mas; si no, veo 'debes tener al menos 13 anos'.
-4. Si el correo ya esta registrado, veo un aviso para iniciar sesion.</t>
+4. Si el correo ya esta registrado, veo un aviso para iniciar sesion.
+5. Debo aceptar la politica de tratamiento de datos (Ley 1581 de 2012); si no, no se crea la cuenta.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="64" customHeight="1">
-      <c r="A17" s="70" t="n"/>
+      <c r="A17" s="34" t="n"/>
       <c r="B17" s="67" t="inlineStr">
         <is>
           <t>HU0016</t>
@@ -2580,7 +2637,7 @@
       </c>
     </row>
     <row r="18" ht="96" customHeight="1">
-      <c r="A18" s="70" t="n"/>
+      <c r="A18" s="34" t="n"/>
       <c r="B18" s="67" t="inlineStr">
         <is>
           <t>HU0017</t>
@@ -2634,7 +2691,7 @@
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="71" t="n"/>
+      <c r="A19" s="34" t="n"/>
       <c r="B19" s="67" t="inlineStr">
         <is>
           <t>HU0018</t>
@@ -2671,11 +2728,11 @@
         <v/>
       </c>
       <c r="J19" s="57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" s="58" t="inlineStr">
         <is>
-          <t>Protege la cuenta en un dispositivo compartido; es de apoyo.</t>
+          <t>Protege la cuenta en un dispositivo compartido; solo tiene sentido despues de iniciar sesion, por eso va con ella en el sprint 3.</t>
         </is>
       </c>
       <c r="L19" s="69" t="inlineStr">
@@ -2685,25 +2742,21 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="67" t="inlineStr">
-        <is>
-          <t>Participacion del interlocutor</t>
-        </is>
-      </c>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="35" t="n"/>
       <c r="B20" s="67" t="inlineStr">
         <is>
-          <t>HU0019</t>
+          <t>HU0026</t>
         </is>
       </c>
       <c r="C20" s="68" t="inlineStr">
         <is>
-          <t>Recibir el mensaje traducido</t>
+          <t>Eliminar mi cuenta</t>
         </is>
       </c>
       <c r="D20" s="58" t="inlineStr">
         <is>
-          <t>Interlocutor</t>
+          <t>Cliente Traductor</t>
         </is>
       </c>
       <c r="E20" s="58">
@@ -2711,15 +2764,15 @@
         <v/>
       </c>
       <c r="F20" s="58">
-        <f>'Mapa de Impacto'!C11</f>
+        <f>'Mapa de Impacto'!C8</f>
         <v/>
       </c>
       <c r="G20" s="57" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="H20" s="57" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="I20" s="57">
@@ -2727,30 +2780,35 @@
         <v/>
       </c>
       <c r="J20" s="57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="58" t="inlineStr">
         <is>
-          <t>Hace que la otra persona participe sin instalar ni operar la app.</t>
+          <t>Cumple el derecho al olvido (Ley 1581 de 2012): la persona controla sus datos.</t>
         </is>
       </c>
       <c r="L20" s="69" t="inlineStr">
         <is>
-          <t>1. Dado que la otra persona responde (se escribe como 'Otra persona'), entonces su mensaje se traduce a mi idioma y se muestra a la izquierda, junto a su original.
-2. La otra persona no necesita instalar la app ni tener cuenta.</t>
+          <t>1. Dado que estoy en mi perfil, cuando elijo eliminar mi cuenta, entonces la app me pide mi contrasena y me avisa que no se puede deshacer.
+2. Al confirmar, se borran mi cuenta, mis conversaciones, mis mensajes y mis reportes, y vuelvo a la pantalla de bienvenida.
+3. Con una contrasena incorrecta la cuenta no se elimina.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="71" t="n"/>
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>Participacion del interlocutor</t>
+        </is>
+      </c>
       <c r="B21" s="67" t="inlineStr">
         <is>
-          <t>HU0020</t>
+          <t>HU0019</t>
         </is>
       </c>
       <c r="C21" s="68" t="inlineStr">
         <is>
-          <t>Responder en mi idioma</t>
+          <t>Recibir el mensaje traducido</t>
         </is>
       </c>
       <c r="D21" s="58" t="inlineStr">
@@ -2767,11 +2825,11 @@
         <v/>
       </c>
       <c r="G21" s="57" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H21" s="57" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I21" s="57">
@@ -2783,118 +2841,170 @@
       </c>
       <c r="K21" s="58" t="inlineStr">
         <is>
+          <t>Hace que la otra persona participe sin instalar ni operar la app.</t>
+        </is>
+      </c>
+      <c r="L21" s="69" t="inlineStr">
+        <is>
+          <t>1. Dado que la otra persona responde (se elige 'Otra persona' y se le pasa el celular), entonces su mensaje se traduce a mi idioma y se muestra a la izquierda, junto a su original.
+2. La otra persona no necesita instalar la app ni crear una cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="35" t="n"/>
+      <c r="B22" s="67" t="inlineStr">
+        <is>
+          <t>HU0020</t>
+        </is>
+      </c>
+      <c r="C22" s="68" t="inlineStr">
+        <is>
+          <t>Responder en mi idioma</t>
+        </is>
+      </c>
+      <c r="D22" s="58" t="inlineStr">
+        <is>
+          <t>Interlocutor</t>
+        </is>
+      </c>
+      <c r="E22" s="58">
+        <f>C22</f>
+        <v/>
+      </c>
+      <c r="F22" s="58">
+        <f>'Mapa de Impacto'!C11</f>
+        <v/>
+      </c>
+      <c r="G22" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="H22" s="57" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I22" s="57">
+        <f>VLOOKUP(H22,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J22" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="58" t="inlineStr">
+        <is>
           <t>Cierra el dialogo en ambos sentidos.</t>
         </is>
       </c>
-      <c r="L21" s="69" t="inlineStr">
+      <c r="L22" s="69" t="inlineStr">
         <is>
           <t>1. Cuando la otra persona escribe en su propio idioma, entonces su respuesta se traduce al idioma de la conversacion.
 2. Para responder ya debe haberse reconocido mi idioma con mi primer mensaje.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="67" t="inlineStr">
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="67" t="inlineStr">
         <is>
           <t>Reportes</t>
         </is>
       </c>
-      <c r="B22" s="67" t="inlineStr">
+      <c r="B23" s="67" t="inlineStr">
         <is>
           <t>HU0021</t>
         </is>
       </c>
-      <c r="C22" s="68" t="inlineStr">
+      <c r="C23" s="68" t="inlineStr">
         <is>
           <t>Reportar una mala traduccion</t>
         </is>
       </c>
-      <c r="D22" s="58" t="inlineStr">
+      <c r="D23" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E22" s="58">
-        <f>C22</f>
-        <v/>
-      </c>
-      <c r="F22" s="58">
+      <c r="E23" s="58">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="F23" s="58">
         <f>'Mapa de Impacto'!C10</f>
         <v/>
       </c>
-      <c r="G22" s="57" t="n">
+      <c r="G23" s="57" t="n">
         <v>18</v>
       </c>
-      <c r="H22" s="57" t="inlineStr">
+      <c r="H23" s="57" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I22" s="57">
-        <f>VLOOKUP(H22,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J22" s="57" t="n">
+      <c r="I23" s="57">
+        <f>VLOOKUP(H23,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J23" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="K22" s="58" t="inlineStr">
+      <c r="K23" s="58" t="inlineStr">
         <is>
           <t>Alimenta la mejora de calidad con casos reales.</t>
         </is>
       </c>
-      <c r="L22" s="69" t="inlineStr">
+      <c r="L23" s="69" t="inlineStr">
         <is>
           <t>1. Cuando reporto una traduccion con un motivo de 3 a 500 caracteres, entonces el reporte se guarda y el mensaje queda marcado como 'Reportado'.
 2. Solo puedo reportar una vez la misma traduccion y solo las de mis conversaciones.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="64" customHeight="1">
-      <c r="A23" s="71" t="n"/>
-      <c r="B23" s="67" t="inlineStr">
+    <row r="24" ht="64" customHeight="1">
+      <c r="A24" s="35" t="n"/>
+      <c r="B24" s="67" t="inlineStr">
         <is>
           <t>HU0022</t>
         </is>
       </c>
-      <c r="C23" s="68" t="inlineStr">
+      <c r="C24" s="68" t="inlineStr">
         <is>
           <t>Revisar los reportes de mala traduccion</t>
         </is>
       </c>
-      <c r="D23" s="58" t="inlineStr">
+      <c r="D24" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E23" s="58">
-        <f>C23</f>
-        <v/>
-      </c>
-      <c r="F23" s="58">
+      <c r="E24" s="58">
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="F24" s="58">
         <f>'Mapa de Impacto'!C13</f>
         <v/>
       </c>
-      <c r="G23" s="57" t="n">
+      <c r="G24" s="57" t="n">
         <v>23</v>
       </c>
-      <c r="H23" s="57" t="inlineStr">
+      <c r="H24" s="57" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I23" s="57">
-        <f>VLOOKUP(H23,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J23" s="57" t="n">
+      <c r="I24" s="57">
+        <f>VLOOKUP(H24,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J24" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="K23" s="58" t="inlineStr">
+      <c r="K24" s="58" t="inlineStr">
         <is>
           <t>Permite priorizar que mejorar primero.</t>
         </is>
       </c>
-      <c r="L23" s="69" t="inlineStr">
+      <c r="L24" s="69" t="inlineStr">
         <is>
           <t>1. Dado que soy administrador, cuando abro los reportes, entonces veo el original, la traduccion, el motivo y la sugerencia, y puedo filtrar por abiertos, revisados o descartados.
 2. Puedo marcar un reporte como revisado o descartado.
@@ -2902,108 +3012,108 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="67" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="67" t="inlineStr">
         <is>
           <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
-      <c r="B24" s="67" t="inlineStr">
+      <c r="B25" s="67" t="inlineStr">
         <is>
           <t>HU0023</t>
         </is>
       </c>
-      <c r="C24" s="68" t="inlineStr">
+      <c r="C25" s="68" t="inlineStr">
         <is>
           <t>Consultar los idiomas disponibles</t>
         </is>
       </c>
-      <c r="D24" s="58" t="inlineStr">
+      <c r="D25" s="58" t="inlineStr">
         <is>
           <t>Cliente Traductor</t>
         </is>
       </c>
-      <c r="E24" s="58">
-        <f>C24</f>
-        <v/>
-      </c>
-      <c r="F24" s="58">
+      <c r="E25" s="58">
+        <f>C25</f>
+        <v/>
+      </c>
+      <c r="F25" s="58">
         <f>'Mapa de Impacto'!C5</f>
         <v/>
       </c>
-      <c r="G24" s="57" t="n">
+      <c r="G25" s="57" t="n">
         <v>13</v>
       </c>
-      <c r="H24" s="57" t="inlineStr">
+      <c r="H25" s="57" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="I24" s="57">
-        <f>VLOOKUP(H24,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J24" s="57" t="n">
+      <c r="I25" s="57">
+        <f>VLOOKUP(H25,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J25" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="K24" s="58" t="inlineStr">
+      <c r="K25" s="58" t="inlineStr">
         <is>
           <t>Muestra con que idiomas se puede hablar antes de empezar.</t>
         </is>
       </c>
-      <c r="L24" s="69" t="inlineStr">
+      <c r="L25" s="69" t="inlineStr">
         <is>
           <t>1. Cuando abro la configuracion de una conversacion, entonces veo solo los idiomas activos con sus regiones.
 2. Los idiomas desactivados no aparecen en la lista.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="80" customHeight="1">
-      <c r="A25" s="70" t="n"/>
-      <c r="B25" s="67" t="inlineStr">
+    <row r="26" ht="80" customHeight="1">
+      <c r="A26" s="34" t="n"/>
+      <c r="B26" s="67" t="inlineStr">
         <is>
           <t>HU0024</t>
         </is>
       </c>
-      <c r="C25" s="68" t="inlineStr">
+      <c r="C26" s="68" t="inlineStr">
         <is>
           <t>Agregar un idioma o una region</t>
         </is>
       </c>
-      <c r="D25" s="58" t="inlineStr">
+      <c r="D26" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E25" s="58">
-        <f>C25</f>
-        <v/>
-      </c>
-      <c r="F25" s="58">
+      <c r="E26" s="58">
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="F26" s="58">
         <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
-      <c r="G25" s="57" t="n">
+      <c r="G26" s="57" t="n">
         <v>24</v>
       </c>
-      <c r="H25" s="57" t="inlineStr">
+      <c r="H26" s="57" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I25" s="57">
-        <f>VLOOKUP(H25,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J25" s="57" t="n">
+      <c r="I26" s="57">
+        <f>VLOOKUP(H26,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J26" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="K25" s="58" t="inlineStr">
+      <c r="K26" s="58" t="inlineStr">
         <is>
           <t>Hace crecer el servicio a mas personas.</t>
         </is>
       </c>
-      <c r="L25" s="69" t="inlineStr">
+      <c r="L26" s="69" t="inlineStr">
         <is>
           <t>1. Dado que soy administrador, cuando agrego un idioma, entonces necesita un nombre unico y un codigo de 2 a 5 letras, y queda desactivado hasta que lo active.
 2. Una region no puede repetirse dentro del mismo pais; si el pais no existe, debo indicar su codigo de 2 letras.
@@ -3011,52 +3121,52 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="71" t="n"/>
-      <c r="B26" s="67" t="inlineStr">
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="35" t="n"/>
+      <c r="B27" s="67" t="inlineStr">
         <is>
           <t>HU0025</t>
         </is>
       </c>
-      <c r="C26" s="68" t="inlineStr">
+      <c r="C27" s="68" t="inlineStr">
         <is>
           <t>Activar o desactivar un idioma o una region</t>
         </is>
       </c>
-      <c r="D26" s="58" t="inlineStr">
+      <c r="D27" s="58" t="inlineStr">
         <is>
           <t>Administrador</t>
         </is>
       </c>
-      <c r="E26" s="58">
-        <f>C26</f>
-        <v/>
-      </c>
-      <c r="F26" s="58">
+      <c r="E27" s="58">
+        <f>C27</f>
+        <v/>
+      </c>
+      <c r="F27" s="58">
         <f>'Mapa de Impacto'!C12</f>
         <v/>
       </c>
-      <c r="G26" s="57" t="n">
+      <c r="G27" s="57" t="n">
         <v>25</v>
       </c>
-      <c r="H26" s="57" t="inlineStr">
+      <c r="H27" s="57" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="I26" s="57">
-        <f>VLOOKUP(H26,Planificacion!$A$4:$B$9,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="J26" s="57" t="n">
+      <c r="I27" s="57">
+        <f>VLOOKUP(H27,Planificacion!$A$4:$B$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J27" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="K26" s="58" t="inlineStr">
+      <c r="K27" s="58" t="inlineStr">
         <is>
           <t>Controla que idiomas se ofrecen con calidad suficiente.</t>
         </is>
       </c>
-      <c r="L26" s="69" t="inlineStr">
+      <c r="L27" s="69" t="inlineStr">
         <is>
           <t>1. Cuando activo un idioma, entonces aparece en el catalogo para crear conversaciones; cuando lo desactivo, deja de aparecer.
 2. Las conversaciones ya creadas no se ven afectadas.</t>
@@ -3065,12 +3175,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A25:A27"/>
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A16:A20"/>
+    <mergeCell ref="A23:A24"/>
     <mergeCell ref="A7:A15"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A21:A22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" location="'Traductor de mensajes'!A1" display="Traductor de mensajes"/>
@@ -3299,13 +3409,13 @@
       </c>
       <c r="E14" s="65" t="inlineStr">
         <is>
-          <t>HU0001, HU0002, HU0003, HU0004, HU0005, HU0006</t>
-        </is>
-      </c>
-      <c r="F14" s="73" t="n">
+          <t>HU0003, HU0002, HU0001, HU0004, HU0005, HU0006</t>
+        </is>
+      </c>
+      <c r="F14" s="75" t="n">
         <v>46314</v>
       </c>
-      <c r="G14" s="73" t="n">
+      <c r="G14" s="75" t="n">
         <v>46318</v>
       </c>
       <c r="H14" s="62" t="inlineStr">
@@ -3332,13 +3442,13 @@
       </c>
       <c r="E15" s="65" t="inlineStr">
         <is>
-          <t>HU0007, HU0008, HU0009, HU0010, HU0011, HU0012, HU0013, HU0018, HU0019, HU0020, HU0023, HU0025</t>
-        </is>
-      </c>
-      <c r="F15" s="73" t="n">
+          <t>HU0007, HU0008, HU0009, HU0010, HU0019, HU0020, HU0023, HU0011, HU0012, HU0013, HU0014, HU0025</t>
+        </is>
+      </c>
+      <c r="F15" s="75" t="n">
         <v>46321</v>
       </c>
-      <c r="G15" s="73" t="n">
+      <c r="G15" s="75" t="n">
         <v>46325</v>
       </c>
       <c r="H15" s="62" t="inlineStr">
@@ -3365,13 +3475,13 @@
       </c>
       <c r="E16" s="65" t="inlineStr">
         <is>
-          <t>HU0014, HU0015, HU0016, HU0017, HU0021, HU0022, HU0024</t>
-        </is>
-      </c>
-      <c r="F16" s="73" t="n">
+          <t>HU0015, HU0016, HU0021, HU0017, HU0018, HU0022, HU0024, HU0026</t>
+        </is>
+      </c>
+      <c r="F16" s="75" t="n">
         <v>46328</v>
       </c>
-      <c r="G16" s="73" t="n">
+      <c r="G16" s="75" t="n">
         <v>46332</v>
       </c>
       <c r="H16" s="62" t="inlineStr">
@@ -3515,10 +3625,10 @@
       <c r="B5" s="64" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="74" t="n">
+      <c r="C5" s="76" t="n">
         <v>46314</v>
       </c>
-      <c r="D5" s="74" t="n">
+      <c r="D5" s="76" t="n">
         <v>46318</v>
       </c>
       <c r="E5" s="65" t="inlineStr">
@@ -3533,7 +3643,7 @@
       </c>
       <c r="G5" s="65" t="inlineStr">
         <is>
-          <t>HU0001, HU0002, HU0003, HU0004, HU0005, HU0006</t>
+          <t>HU0003, HU0002, HU0001, HU0004, HU0005, HU0006</t>
         </is>
       </c>
       <c r="H5" s="64">
@@ -3550,10 +3660,10 @@
       <c r="B6" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="76" t="n">
         <v>46321</v>
       </c>
-      <c r="D6" s="74" t="n">
+      <c r="D6" s="76" t="n">
         <v>46325</v>
       </c>
       <c r="E6" s="65" t="inlineStr">
@@ -3563,12 +3673,12 @@
       </c>
       <c r="F6" s="65" t="inlineStr">
         <is>
-          <t>El usuario organiza sus conversaciones (reconocer idioma, crear, hilo continuo, historial, renombrar), la otra persona participa y el administrador controla que idiomas se activan.</t>
+          <t>El usuario organiza sus conversaciones (reconocer idioma, crear, hilo continuo, historial, renombrar y eliminar), la otra persona participa y el administrador controla que idiomas se activan.</t>
         </is>
       </c>
       <c r="G6" s="65" t="inlineStr">
         <is>
-          <t>HU0007, HU0008, HU0009, HU0010, HU0011, HU0012, HU0013, HU0018, HU0019, HU0020, HU0023, HU0025</t>
+          <t>HU0007, HU0008, HU0009, HU0010, HU0019, HU0020, HU0023, HU0011, HU0012, HU0013, HU0014, HU0025</t>
         </is>
       </c>
       <c r="H6" s="64">
@@ -3585,10 +3695,10 @@
       <c r="B7" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="74" t="n">
+      <c r="C7" s="76" t="n">
         <v>46328</v>
       </c>
-      <c r="D7" s="74" t="n">
+      <c r="D7" s="76" t="n">
         <v>46332</v>
       </c>
       <c r="E7" s="65" t="inlineStr">
@@ -3598,12 +3708,12 @@
       </c>
       <c r="F7" s="65" t="inlineStr">
         <is>
-          <t>Registro, inicio de sesion y recuperacion de contrasena, eliminar conversaciones, reportar y revisar malas traducciones, y agregar idiomas y regiones.</t>
+          <t>Registro con consentimiento de datos, inicio y cierre de sesion, recuperacion de contrasena, eliminar la cuenta, reportar y revisar malas traducciones, y agregar idiomas y regiones.</t>
         </is>
       </c>
       <c r="G7" s="65" t="inlineStr">
         <is>
-          <t>HU0014, HU0015, HU0016, HU0017, HU0021, HU0022, HU0024</t>
+          <t>HU0015, HU0016, HU0021, HU0017, HU0018, HU0022, HU0024, HU0026</t>
         </is>
       </c>
       <c r="H7" s="64">
@@ -4053,7 +4163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4194,6 +4304,24 @@
       </c>
       <c r="D11" s="18">
         <f>Entregables!F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="18">
+        <f>Entregables!C20</f>
+        <v/>
+      </c>
+      <c r="B12" s="18">
+        <f>Entregables!D20</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>Entregables!E20</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
+        <f>Entregables!F20</f>
         <v/>
       </c>
     </row>
@@ -4285,37 +4413,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C20</f>
+        <f>Entregables!C21</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D20</f>
+        <f>Entregables!D21</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E20</f>
+        <f>Entregables!E21</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F20</f>
+        <f>Entregables!F21</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C21</f>
+        <f>Entregables!C22</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D21</f>
+        <f>Entregables!D22</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E21</f>
+        <f>Entregables!E22</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F21</f>
+        <f>Entregables!F22</f>
         <v/>
       </c>
     </row>
@@ -4419,37 +4547,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C22</f>
+        <f>Entregables!C23</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D22</f>
+        <f>Entregables!D23</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E22</f>
+        <f>Entregables!E23</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F22</f>
+        <f>Entregables!F23</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C23</f>
+        <f>Entregables!C24</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D23</f>
+        <f>Entregables!D24</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E23</f>
+        <f>Entregables!E24</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F23</f>
+        <f>Entregables!F24</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(planificacion): hoja Resumen sprints en el Mapa de Impacto
Junta en una sola hoja las tallas y horas, la capacidad del sprint
(2 x 4 h x 5 dias x 75 % = 30 h), el resumen por sprint con fechas y
liberacion, y las historias de cada sprint ordenadas por valor. Todo sale
por formulas de Entregables, Planificacion y Plan de liberaciones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -3,19 +3,20 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="160" yWindow="940" windowWidth="35680" windowHeight="22280" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="160" yWindow="940" windowWidth="35680" windowHeight="22280" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Mapa de Impacto" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Entregables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Planificacion" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Plan de liberaciones" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Traduccion de mensajes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gestion de conversaciones" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cuenta de usuario" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Participacion interlocutor" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Reportes" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Admin idiomas y regiones" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Resumen sprints" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Traduccion de mensajes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gestion de conversaciones" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cuenta de usuario" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Participacion interlocutor" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Reportes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Admin idiomas y regiones" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,8 +114,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -164,8 +169,13 @@
         <fgColor rgb="0092D050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="29">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -532,11 +542,45 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -736,6 +780,49 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1576,6 +1663,140 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Cliente Traductor / Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Impacto (para)</t>
+        </is>
+      </c>
+      <c r="B3" s="18">
+        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>← Volver al Mapa de Impacto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Característica</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Necesito</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Para</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C23</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D23</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E23</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C24</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D24</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E24</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Entregable</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
           <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
@@ -3737,6 +3958,1727 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>Resumen de sprints: prioridad por valor, tallas y horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="69" t="inlineStr">
+        <is>
+          <t>Vista para revisar con el mentor. Los datos salen de las hojas Entregables y Planificacion: si se cambia una talla o un sprint alla, esta hoja se recalcula sola.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>1. Tallas y horas (una persona desarrolla)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B5" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="C5" s="78" t="inlineStr">
+        <is>
+          <t>Historias</t>
+        </is>
+      </c>
+      <c r="D5" s="78" t="inlineStr">
+        <is>
+          <t>Horas en total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="B6" s="80">
+        <f>Planificacion!B4</f>
+        <v/>
+      </c>
+      <c r="C6" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="80">
+        <f>B6*C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="79" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B7" s="80">
+        <f>Planificacion!B5</f>
+        <v/>
+      </c>
+      <c r="C7" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="80">
+        <f>B7*C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="79" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B8" s="80">
+        <f>Planificacion!B6</f>
+        <v/>
+      </c>
+      <c r="C8" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="80">
+        <f>B8*C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B9" s="80">
+        <f>Planificacion!B7</f>
+        <v/>
+      </c>
+      <c r="C9" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="80">
+        <f>B9*C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="79" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="B10" s="80">
+        <f>Planificacion!B8</f>
+        <v/>
+      </c>
+      <c r="C10" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="80">
+        <f>B10*C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="79" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="B11" s="80">
+        <f>Planificacion!B9</f>
+        <v/>
+      </c>
+      <c r="C11" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="80">
+        <f>B11*C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B12" s="82" t="inlineStr"/>
+      <c r="C12" s="83">
+        <f>SUM(C6:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="83">
+        <f>SUM(D6:D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="59" t="inlineStr">
+        <is>
+          <t>2. Capacidad de un sprint (1 semana)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="78" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B15" s="84" t="n"/>
+      <c r="C15" s="85" t="n"/>
+      <c r="D15" s="78" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="86" t="inlineStr">
+        <is>
+          <t>Dias del sprint (lunes a viernes)</t>
+        </is>
+      </c>
+      <c r="B16" s="84" t="n"/>
+      <c r="C16" s="85" t="n"/>
+      <c r="D16" s="87">
+        <f>Planificacion!E3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="86" t="inlineStr">
+        <is>
+          <t>Horas por dia y por persona</t>
+        </is>
+      </c>
+      <c r="B17" s="84" t="n"/>
+      <c r="C17" s="85" t="n"/>
+      <c r="D17" s="87">
+        <f>Planificacion!E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="86" t="inlineStr">
+        <is>
+          <t>Personas (Julian y Diego)</t>
+        </is>
+      </c>
+      <c r="B18" s="84" t="n"/>
+      <c r="C18" s="85" t="n"/>
+      <c r="D18" s="87">
+        <f>Planificacion!E5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="86" t="inlineStr">
+        <is>
+          <t>Horas brutas (5 x 4 x 2)</t>
+        </is>
+      </c>
+      <c r="B19" s="84" t="n"/>
+      <c r="C19" s="85" t="n"/>
+      <c r="D19" s="87">
+        <f>Planificacion!E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="86" t="inlineStr">
+        <is>
+          <t>Porcentaje usable (el resto: planeacion, dailies, refinamiento y retro)</t>
+        </is>
+      </c>
+      <c r="B20" s="84" t="n"/>
+      <c r="C20" s="85" t="n"/>
+      <c r="D20" s="88">
+        <f>Planificacion!E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="81" t="inlineStr">
+        <is>
+          <t>Horas disponibles por sprint</t>
+        </is>
+      </c>
+      <c r="B21" s="84" t="n"/>
+      <c r="C21" s="85" t="n"/>
+      <c r="D21" s="89">
+        <f>Planificacion!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="59" t="inlineStr">
+        <is>
+          <t>3. Resumen por sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="78" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B25" s="78" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="C25" s="78" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="D25" s="78" t="inlineStr">
+        <is>
+          <t>Liberacion</t>
+        </is>
+      </c>
+      <c r="E25" s="78" t="inlineStr">
+        <is>
+          <t>Historias</t>
+        </is>
+      </c>
+      <c r="F25" s="78" t="inlineStr">
+        <is>
+          <t>Horas planeadas</t>
+        </is>
+      </c>
+      <c r="G25" s="78" t="inlineStr">
+        <is>
+          <t>Horas disponibles</t>
+        </is>
+      </c>
+      <c r="H25" s="78" t="inlineStr">
+        <is>
+          <t>Holgura</t>
+        </is>
+      </c>
+      <c r="I25" s="78" t="inlineStr">
+        <is>
+          <t>Uso de la capacidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="90">
+        <f>'Plan de liberaciones'!C5</f>
+        <v/>
+      </c>
+      <c r="C26" s="90">
+        <f>'Plan de liberaciones'!D5</f>
+        <v/>
+      </c>
+      <c r="D26" s="86">
+        <f>'Plan de liberaciones'!A5&amp;": "&amp;'Plan de liberaciones'!E5</f>
+        <v/>
+      </c>
+      <c r="E26" s="80">
+        <f>COUNTIF(Entregables!$J$2:$J$40,A26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="80">
+        <f>SUMIF(Entregables!$J$2:$J$40,A26,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="G26" s="80">
+        <f>Planificacion!$E$8</f>
+        <v/>
+      </c>
+      <c r="H26" s="80">
+        <f>G26-F26</f>
+        <v/>
+      </c>
+      <c r="I26" s="88">
+        <f>F26/G26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="90">
+        <f>'Plan de liberaciones'!C6</f>
+        <v/>
+      </c>
+      <c r="C27" s="90">
+        <f>'Plan de liberaciones'!D6</f>
+        <v/>
+      </c>
+      <c r="D27" s="86">
+        <f>'Plan de liberaciones'!A6&amp;": "&amp;'Plan de liberaciones'!E6</f>
+        <v/>
+      </c>
+      <c r="E27" s="80">
+        <f>COUNTIF(Entregables!$J$2:$J$40,A27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="80">
+        <f>SUMIF(Entregables!$J$2:$J$40,A27,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="G27" s="80">
+        <f>Planificacion!$E$8</f>
+        <v/>
+      </c>
+      <c r="H27" s="80">
+        <f>G27-F27</f>
+        <v/>
+      </c>
+      <c r="I27" s="88">
+        <f>F27/G27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="90">
+        <f>'Plan de liberaciones'!C7</f>
+        <v/>
+      </c>
+      <c r="C28" s="90">
+        <f>'Plan de liberaciones'!D7</f>
+        <v/>
+      </c>
+      <c r="D28" s="86">
+        <f>'Plan de liberaciones'!A7&amp;": "&amp;'Plan de liberaciones'!E7</f>
+        <v/>
+      </c>
+      <c r="E28" s="80">
+        <f>COUNTIF(Entregables!$J$2:$J$40,A28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="80">
+        <f>SUMIF(Entregables!$J$2:$J$40,A28,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="G28" s="80">
+        <f>Planificacion!$E$8</f>
+        <v/>
+      </c>
+      <c r="H28" s="80">
+        <f>G28-F28</f>
+        <v/>
+      </c>
+      <c r="I28" s="88">
+        <f>F28/G28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="81" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B29" s="82" t="inlineStr"/>
+      <c r="C29" s="82" t="inlineStr"/>
+      <c r="D29" s="82" t="inlineStr"/>
+      <c r="E29" s="83">
+        <f>SUM(E26:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="83">
+        <f>SUM(F26:F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="83">
+        <f>SUM(G26:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="83">
+        <f>G29-F29</f>
+        <v/>
+      </c>
+      <c r="I29" s="91">
+        <f>F29/G29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="59" t="inlineStr">
+        <is>
+          <t>4. Historias de cada sprint, de mayor a menor valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="92">
+        <f>"Sprint 1  |  "&amp;TEXT(B26,"dd/mm/yyyy")&amp;" al "&amp;TEXT(C26,"dd/mm/yyyy")&amp;"  |  "&amp;D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="78" t="inlineStr">
+        <is>
+          <t>Prioridad (valor)</t>
+        </is>
+      </c>
+      <c r="B34" s="78" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="C34" s="78" t="inlineStr">
+        <is>
+          <t>Historia de usuario</t>
+        </is>
+      </c>
+      <c r="D34" s="78" t="inlineStr">
+        <is>
+          <t>Epica</t>
+        </is>
+      </c>
+      <c r="E34" s="78" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="F34" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="G34" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="H34" s="78" t="inlineStr">
+        <is>
+          <t>Por que genera valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B35" s="79" t="inlineStr">
+        <is>
+          <t>HU0003</t>
+        </is>
+      </c>
+      <c r="C35" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D35" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E35" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F35" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G35" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H35" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B36" s="79" t="inlineStr">
+        <is>
+          <t>HU0002</t>
+        </is>
+      </c>
+      <c r="C36" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D36" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E36" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F36" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G36" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H36" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B37" s="79" t="inlineStr">
+        <is>
+          <t>HU0001</t>
+        </is>
+      </c>
+      <c r="C37" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D37" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E37" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F37" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G37" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H37" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B38" s="79" t="inlineStr">
+        <is>
+          <t>HU0004</t>
+        </is>
+      </c>
+      <c r="C38" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D38" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E38" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F38" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G38" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H38" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B39" s="79" t="inlineStr">
+        <is>
+          <t>HU0005</t>
+        </is>
+      </c>
+      <c r="C39" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D39" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E39" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F39" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G39" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H39" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B40" s="79" t="inlineStr">
+        <is>
+          <t>HU0006</t>
+        </is>
+      </c>
+      <c r="C40" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D40" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E40" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F40" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G40" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H40" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="81" t="inlineStr">
+        <is>
+          <t>Total sprint 1</t>
+        </is>
+      </c>
+      <c r="B41" s="82" t="inlineStr"/>
+      <c r="C41" s="82">
+        <f>"Disponibles: "&amp;Planificacion!$E$8&amp;" h  |  Holgura: "&amp;(Planificacion!$E$8-G41)&amp;" h"</f>
+        <v/>
+      </c>
+      <c r="D41" s="82" t="inlineStr"/>
+      <c r="E41" s="82" t="inlineStr"/>
+      <c r="F41" s="93" t="inlineStr">
+        <is>
+          <t>6 HU</t>
+        </is>
+      </c>
+      <c r="G41" s="83">
+        <f>SUM(G35:G40)</f>
+        <v/>
+      </c>
+      <c r="H41" s="82" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="92">
+        <f>"Sprint 2  |  "&amp;TEXT(B27,"dd/mm/yyyy")&amp;" al "&amp;TEXT(C27,"dd/mm/yyyy")&amp;"  |  "&amp;D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="78" t="inlineStr">
+        <is>
+          <t>Prioridad (valor)</t>
+        </is>
+      </c>
+      <c r="B44" s="78" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="C44" s="78" t="inlineStr">
+        <is>
+          <t>Historia de usuario</t>
+        </is>
+      </c>
+      <c r="D44" s="78" t="inlineStr">
+        <is>
+          <t>Epica</t>
+        </is>
+      </c>
+      <c r="E44" s="78" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="F44" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="G44" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="H44" s="78" t="inlineStr">
+        <is>
+          <t>Por que genera valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B45" s="79" t="inlineStr">
+        <is>
+          <t>HU0007</t>
+        </is>
+      </c>
+      <c r="C45" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D45" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E45" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F45" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G45" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H45" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B46" s="79" t="inlineStr">
+        <is>
+          <t>HU0008</t>
+        </is>
+      </c>
+      <c r="C46" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D46" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E46" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F46" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G46" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H46" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B47" s="79" t="inlineStr">
+        <is>
+          <t>HU0009</t>
+        </is>
+      </c>
+      <c r="C47" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D47" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E47" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F47" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G47" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H47" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B48" s="79" t="inlineStr">
+        <is>
+          <t>HU0010</t>
+        </is>
+      </c>
+      <c r="C48" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D48" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E48" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F48" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G48" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H48" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B49" s="79" t="inlineStr">
+        <is>
+          <t>HU0019</t>
+        </is>
+      </c>
+      <c r="C49" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D49" s="86" t="inlineStr">
+        <is>
+          <t>Participacion del interlocutor</t>
+        </is>
+      </c>
+      <c r="E49" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F49" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G49" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H49" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B50" s="79" t="inlineStr">
+        <is>
+          <t>HU0020</t>
+        </is>
+      </c>
+      <c r="C50" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D50" s="86" t="inlineStr">
+        <is>
+          <t>Participacion del interlocutor</t>
+        </is>
+      </c>
+      <c r="E50" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F50" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G50" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H50" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B51" s="79" t="inlineStr">
+        <is>
+          <t>HU0023</t>
+        </is>
+      </c>
+      <c r="C51" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D51" s="86" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
+      <c r="E51" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F51" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G51" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H51" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B52" s="79" t="inlineStr">
+        <is>
+          <t>HU0011</t>
+        </is>
+      </c>
+      <c r="C52" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D52" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E52" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F52" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G52" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H52" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B53" s="79" t="inlineStr">
+        <is>
+          <t>HU0012</t>
+        </is>
+      </c>
+      <c r="C53" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D53" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E53" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F53" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G53" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H53" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B54" s="79" t="inlineStr">
+        <is>
+          <t>HU0013</t>
+        </is>
+      </c>
+      <c r="C54" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D54" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E54" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F54" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G54" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H54" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B55" s="79" t="inlineStr">
+        <is>
+          <t>HU0014</t>
+        </is>
+      </c>
+      <c r="C55" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D55" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E55" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F55" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G55" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H55" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B56" s="79" t="inlineStr">
+        <is>
+          <t>HU0025</t>
+        </is>
+      </c>
+      <c r="C56" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D56" s="86" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
+      <c r="E56" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F56" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G56" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H56" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="81" t="inlineStr">
+        <is>
+          <t>Total sprint 2</t>
+        </is>
+      </c>
+      <c r="B57" s="82" t="inlineStr"/>
+      <c r="C57" s="82">
+        <f>"Disponibles: "&amp;Planificacion!$E$8&amp;" h  |  Holgura: "&amp;(Planificacion!$E$8-G57)&amp;" h"</f>
+        <v/>
+      </c>
+      <c r="D57" s="82" t="inlineStr"/>
+      <c r="E57" s="82" t="inlineStr"/>
+      <c r="F57" s="93" t="inlineStr">
+        <is>
+          <t>12 HU</t>
+        </is>
+      </c>
+      <c r="G57" s="83">
+        <f>SUM(G45:G56)</f>
+        <v/>
+      </c>
+      <c r="H57" s="82" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="92">
+        <f>"Sprint 3  |  "&amp;TEXT(B28,"dd/mm/yyyy")&amp;" al "&amp;TEXT(C28,"dd/mm/yyyy")&amp;"  |  "&amp;D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="78" t="inlineStr">
+        <is>
+          <t>Prioridad (valor)</t>
+        </is>
+      </c>
+      <c r="B60" s="78" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="C60" s="78" t="inlineStr">
+        <is>
+          <t>Historia de usuario</t>
+        </is>
+      </c>
+      <c r="D60" s="78" t="inlineStr">
+        <is>
+          <t>Epica</t>
+        </is>
+      </c>
+      <c r="E60" s="78" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="F60" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="G60" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="H60" s="78" t="inlineStr">
+        <is>
+          <t>Por que genera valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B61" s="79" t="inlineStr">
+        <is>
+          <t>HU0015</t>
+        </is>
+      </c>
+      <c r="C61" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D61" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E61" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F61" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G61" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H61" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B62" s="79" t="inlineStr">
+        <is>
+          <t>HU0016</t>
+        </is>
+      </c>
+      <c r="C62" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E62" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F62" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G62" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H62" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B63" s="79" t="inlineStr">
+        <is>
+          <t>HU0021</t>
+        </is>
+      </c>
+      <c r="C63" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D63" s="86" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="E63" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F63" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G63" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H63" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B64" s="79" t="inlineStr">
+        <is>
+          <t>HU0017</t>
+        </is>
+      </c>
+      <c r="C64" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D64" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E64" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F64" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G64" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H64" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B65" s="79" t="inlineStr">
+        <is>
+          <t>HU0018</t>
+        </is>
+      </c>
+      <c r="C65" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D65" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E65" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F65" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G65" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H65" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B66" s="79" t="inlineStr">
+        <is>
+          <t>HU0022</t>
+        </is>
+      </c>
+      <c r="C66" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D66" s="86" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="E66" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F66" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G66" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H66" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B67" s="79" t="inlineStr">
+        <is>
+          <t>HU0024</t>
+        </is>
+      </c>
+      <c r="C67" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D67" s="86" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
+      <c r="E67" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F67" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G67" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H67" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B68" s="79" t="inlineStr">
+        <is>
+          <t>HU0026</t>
+        </is>
+      </c>
+      <c r="C68" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D68" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E68" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F68" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G68" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H68" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="81" t="inlineStr">
+        <is>
+          <t>Total sprint 3</t>
+        </is>
+      </c>
+      <c r="B69" s="82" t="inlineStr"/>
+      <c r="C69" s="82">
+        <f>"Disponibles: "&amp;Planificacion!$E$8&amp;" h  |  Holgura: "&amp;(Planificacion!$E$8-G69)&amp;" h"</f>
+        <v/>
+      </c>
+      <c r="D69" s="82" t="inlineStr"/>
+      <c r="E69" s="82" t="inlineStr"/>
+      <c r="F69" s="93" t="inlineStr">
+        <is>
+          <t>8 HU</t>
+        </is>
+      </c>
+      <c r="G69" s="83">
+        <f>SUM(G61:G68)</f>
+        <v/>
+      </c>
+      <c r="H69" s="82" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="59" t="inlineStr">
+        <is>
+          <t>5. Como se armo</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="69" t="inlineStr">
+        <is>
+          <t>1. La prioridad va por valor para el negocio, no por dependencia: lo que mas valor genera es traducir (HU0003 es la 1); registrarse y cerrar sesion son de apoyo y van al final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="69" t="inlineStr">
+        <is>
+          <t>2. Cada historia se talla con tallas de ropa (XS a XXL) y cada talla tiene horas para una persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="69" t="inlineStr">
+        <is>
+          <t>3. Los sprints duran una semana. Capacidad: 2 personas x 4 horas x 5 dias = 40 horas; se usa el 75 % = 30 horas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="69" t="inlineStr">
+        <is>
+          <t>4. Se llenan los sprints de mayor a menor valor hasta quedar cerca de 30 horas; si sobra espacio se acomoda una historia pequena de mas abajo. Ejemplo: con las prioridades 7 a 15 el sprint 2 llega a 27 horas; las siguientes (HU0015 de 6 h, HU0016 y HU0021 de 4 h) no caben en las 3 horas que quedan, por eso entran HU0013, HU0014 y HU0025 (1 h cada una) y las otras pasan al sprint 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="69" t="inlineStr">
+        <is>
+          <t>5. Con los sprints sale el plan de liberaciones: cada sprint termina con una liberacion. El primero empieza el lunes 19/10/2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A73:I73"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A75:I75"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A76:I76"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A74:I74"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A72:I72"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I26:I28">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FF92D050"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
@@ -3909,7 +5851,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4157,7 +6099,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4324,140 +6266,6 @@
         <f>Entregables!F20</f>
         <v/>
       </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Participacion del interlocutor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="18">
-        <f>Entregables!C21</f>
-        <v/>
-      </c>
-      <c r="B8" s="18">
-        <f>Entregables!D21</f>
-        <v/>
-      </c>
-      <c r="C8" s="18">
-        <f>Entregables!E21</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>Entregables!F21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="18">
-        <f>Entregables!C22</f>
-        <v/>
-      </c>
-      <c r="B9" s="18">
-        <f>Entregables!D22</f>
-        <v/>
-      </c>
-      <c r="C9" s="18">
-        <f>Entregables!E22</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>Entregables!F22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="18" t="n"/>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4489,7 +6297,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Reportes</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
     </row>
@@ -4501,18 +6309,18 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Cliente Traductor / Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="90" customHeight="1">
+          <t>Interlocutor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
+        <f>'Mapa de Impacto'!C11</f>
         <v/>
       </c>
     </row>
@@ -4547,37 +6355,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C23</f>
+        <f>Entregables!C21</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D23</f>
+        <f>Entregables!D21</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E23</f>
+        <f>Entregables!E21</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F23</f>
+        <f>Entregables!F21</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C24</f>
+        <f>Entregables!C22</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D24</f>
+        <f>Entregables!D22</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E24</f>
+        <f>Entregables!E22</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F24</f>
+        <f>Entregables!F22</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(planificacion): hoja Resumen sprints en el Mapa de Impacto (#32)
Junta en una sola hoja las tallas y horas, la capacidad del sprint
(2 x 4 h x 5 dias x 75 % = 30 h), el resumen por sprint con fechas y
liberacion, y las historias de cada sprint ordenadas por valor. Todo sale
por formulas de Entregables, Planificacion y Plan de liberaciones.


Claude-Session: https://claude.ai/code/session_013unzkPcqnbmvPCQVENgdiE

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
+++ b/seguimiento/mapa_impacto/Mapa de Impacto.xlsx
@@ -3,19 +3,20 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="160" yWindow="940" windowWidth="35680" windowHeight="22280" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="160" yWindow="940" windowWidth="35680" windowHeight="22280" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Mapa de Impacto" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Entregables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Planificacion" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Plan de liberaciones" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Traduccion de mensajes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gestion de conversaciones" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cuenta de usuario" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Participacion interlocutor" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Reportes" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Admin idiomas y regiones" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Resumen sprints" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Traduccion de mensajes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gestion de conversaciones" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cuenta de usuario" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Participacion interlocutor" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Reportes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Admin idiomas y regiones" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,8 +114,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -164,8 +169,13 @@
         <fgColor rgb="0092D050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="29">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -532,11 +542,45 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -736,6 +780,49 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1576,6 +1663,140 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Cliente Traductor / Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Impacto (para)</t>
+        </is>
+      </c>
+      <c r="B3" s="18">
+        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>← Volver al Mapa de Impacto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Característica</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Necesito</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Para</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18">
+        <f>Entregables!C23</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>Entregables!D23</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>Entregables!E23</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>Entregables!F23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="18">
+        <f>Entregables!C24</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>Entregables!D24</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>Entregables!E24</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>Entregables!F24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Entregable</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
           <t>Administracion de idiomas y regiones</t>
         </is>
       </c>
@@ -3737,6 +3958,1727 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>Resumen de sprints: prioridad por valor, tallas y horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="69" t="inlineStr">
+        <is>
+          <t>Vista para revisar con el mentor. Los datos salen de las hojas Entregables y Planificacion: si se cambia una talla o un sprint alla, esta hoja se recalcula sola.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>1. Tallas y horas (una persona desarrolla)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B5" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="C5" s="78" t="inlineStr">
+        <is>
+          <t>Historias</t>
+        </is>
+      </c>
+      <c r="D5" s="78" t="inlineStr">
+        <is>
+          <t>Horas en total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="B6" s="80">
+        <f>Planificacion!B4</f>
+        <v/>
+      </c>
+      <c r="C6" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="80">
+        <f>B6*C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="79" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B7" s="80">
+        <f>Planificacion!B5</f>
+        <v/>
+      </c>
+      <c r="C7" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="80">
+        <f>B7*C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="79" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B8" s="80">
+        <f>Planificacion!B6</f>
+        <v/>
+      </c>
+      <c r="C8" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="80">
+        <f>B8*C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B9" s="80">
+        <f>Planificacion!B7</f>
+        <v/>
+      </c>
+      <c r="C9" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="80">
+        <f>B9*C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="79" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="B10" s="80">
+        <f>Planificacion!B8</f>
+        <v/>
+      </c>
+      <c r="C10" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="80">
+        <f>B10*C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="79" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="B11" s="80">
+        <f>Planificacion!B9</f>
+        <v/>
+      </c>
+      <c r="C11" s="80">
+        <f>COUNTIF(Entregables!$H$2:$H$40,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="80">
+        <f>B11*C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B12" s="82" t="inlineStr"/>
+      <c r="C12" s="83">
+        <f>SUM(C6:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="83">
+        <f>SUM(D6:D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="59" t="inlineStr">
+        <is>
+          <t>2. Capacidad de un sprint (1 semana)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="78" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B15" s="84" t="n"/>
+      <c r="C15" s="85" t="n"/>
+      <c r="D15" s="78" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="86" t="inlineStr">
+        <is>
+          <t>Dias del sprint (lunes a viernes)</t>
+        </is>
+      </c>
+      <c r="B16" s="84" t="n"/>
+      <c r="C16" s="85" t="n"/>
+      <c r="D16" s="87">
+        <f>Planificacion!E3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="86" t="inlineStr">
+        <is>
+          <t>Horas por dia y por persona</t>
+        </is>
+      </c>
+      <c r="B17" s="84" t="n"/>
+      <c r="C17" s="85" t="n"/>
+      <c r="D17" s="87">
+        <f>Planificacion!E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="86" t="inlineStr">
+        <is>
+          <t>Personas (Julian y Diego)</t>
+        </is>
+      </c>
+      <c r="B18" s="84" t="n"/>
+      <c r="C18" s="85" t="n"/>
+      <c r="D18" s="87">
+        <f>Planificacion!E5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="86" t="inlineStr">
+        <is>
+          <t>Horas brutas (5 x 4 x 2)</t>
+        </is>
+      </c>
+      <c r="B19" s="84" t="n"/>
+      <c r="C19" s="85" t="n"/>
+      <c r="D19" s="87">
+        <f>Planificacion!E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="86" t="inlineStr">
+        <is>
+          <t>Porcentaje usable (el resto: planeacion, dailies, refinamiento y retro)</t>
+        </is>
+      </c>
+      <c r="B20" s="84" t="n"/>
+      <c r="C20" s="85" t="n"/>
+      <c r="D20" s="88">
+        <f>Planificacion!E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="81" t="inlineStr">
+        <is>
+          <t>Horas disponibles por sprint</t>
+        </is>
+      </c>
+      <c r="B21" s="84" t="n"/>
+      <c r="C21" s="85" t="n"/>
+      <c r="D21" s="89">
+        <f>Planificacion!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="59" t="inlineStr">
+        <is>
+          <t>3. Resumen por sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="78" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B25" s="78" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="C25" s="78" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="D25" s="78" t="inlineStr">
+        <is>
+          <t>Liberacion</t>
+        </is>
+      </c>
+      <c r="E25" s="78" t="inlineStr">
+        <is>
+          <t>Historias</t>
+        </is>
+      </c>
+      <c r="F25" s="78" t="inlineStr">
+        <is>
+          <t>Horas planeadas</t>
+        </is>
+      </c>
+      <c r="G25" s="78" t="inlineStr">
+        <is>
+          <t>Horas disponibles</t>
+        </is>
+      </c>
+      <c r="H25" s="78" t="inlineStr">
+        <is>
+          <t>Holgura</t>
+        </is>
+      </c>
+      <c r="I25" s="78" t="inlineStr">
+        <is>
+          <t>Uso de la capacidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="90">
+        <f>'Plan de liberaciones'!C5</f>
+        <v/>
+      </c>
+      <c r="C26" s="90">
+        <f>'Plan de liberaciones'!D5</f>
+        <v/>
+      </c>
+      <c r="D26" s="86">
+        <f>'Plan de liberaciones'!A5&amp;": "&amp;'Plan de liberaciones'!E5</f>
+        <v/>
+      </c>
+      <c r="E26" s="80">
+        <f>COUNTIF(Entregables!$J$2:$J$40,A26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="80">
+        <f>SUMIF(Entregables!$J$2:$J$40,A26,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="G26" s="80">
+        <f>Planificacion!$E$8</f>
+        <v/>
+      </c>
+      <c r="H26" s="80">
+        <f>G26-F26</f>
+        <v/>
+      </c>
+      <c r="I26" s="88">
+        <f>F26/G26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="90">
+        <f>'Plan de liberaciones'!C6</f>
+        <v/>
+      </c>
+      <c r="C27" s="90">
+        <f>'Plan de liberaciones'!D6</f>
+        <v/>
+      </c>
+      <c r="D27" s="86">
+        <f>'Plan de liberaciones'!A6&amp;": "&amp;'Plan de liberaciones'!E6</f>
+        <v/>
+      </c>
+      <c r="E27" s="80">
+        <f>COUNTIF(Entregables!$J$2:$J$40,A27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="80">
+        <f>SUMIF(Entregables!$J$2:$J$40,A27,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="G27" s="80">
+        <f>Planificacion!$E$8</f>
+        <v/>
+      </c>
+      <c r="H27" s="80">
+        <f>G27-F27</f>
+        <v/>
+      </c>
+      <c r="I27" s="88">
+        <f>F27/G27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="90">
+        <f>'Plan de liberaciones'!C7</f>
+        <v/>
+      </c>
+      <c r="C28" s="90">
+        <f>'Plan de liberaciones'!D7</f>
+        <v/>
+      </c>
+      <c r="D28" s="86">
+        <f>'Plan de liberaciones'!A7&amp;": "&amp;'Plan de liberaciones'!E7</f>
+        <v/>
+      </c>
+      <c r="E28" s="80">
+        <f>COUNTIF(Entregables!$J$2:$J$40,A28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="80">
+        <f>SUMIF(Entregables!$J$2:$J$40,A28,Entregables!$I$2:$I$40)</f>
+        <v/>
+      </c>
+      <c r="G28" s="80">
+        <f>Planificacion!$E$8</f>
+        <v/>
+      </c>
+      <c r="H28" s="80">
+        <f>G28-F28</f>
+        <v/>
+      </c>
+      <c r="I28" s="88">
+        <f>F28/G28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="81" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B29" s="82" t="inlineStr"/>
+      <c r="C29" s="82" t="inlineStr"/>
+      <c r="D29" s="82" t="inlineStr"/>
+      <c r="E29" s="83">
+        <f>SUM(E26:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="83">
+        <f>SUM(F26:F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="83">
+        <f>SUM(G26:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="83">
+        <f>G29-F29</f>
+        <v/>
+      </c>
+      <c r="I29" s="91">
+        <f>F29/G29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="59" t="inlineStr">
+        <is>
+          <t>4. Historias de cada sprint, de mayor a menor valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="92">
+        <f>"Sprint 1  |  "&amp;TEXT(B26,"dd/mm/yyyy")&amp;" al "&amp;TEXT(C26,"dd/mm/yyyy")&amp;"  |  "&amp;D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="78" t="inlineStr">
+        <is>
+          <t>Prioridad (valor)</t>
+        </is>
+      </c>
+      <c r="B34" s="78" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="C34" s="78" t="inlineStr">
+        <is>
+          <t>Historia de usuario</t>
+        </is>
+      </c>
+      <c r="D34" s="78" t="inlineStr">
+        <is>
+          <t>Epica</t>
+        </is>
+      </c>
+      <c r="E34" s="78" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="F34" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="G34" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="H34" s="78" t="inlineStr">
+        <is>
+          <t>Por que genera valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B35" s="79" t="inlineStr">
+        <is>
+          <t>HU0003</t>
+        </is>
+      </c>
+      <c r="C35" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D35" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E35" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F35" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G35" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H35" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B35,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B36" s="79" t="inlineStr">
+        <is>
+          <t>HU0002</t>
+        </is>
+      </c>
+      <c r="C36" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D36" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E36" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F36" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G36" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H36" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B36,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B37" s="79" t="inlineStr">
+        <is>
+          <t>HU0001</t>
+        </is>
+      </c>
+      <c r="C37" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D37" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E37" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F37" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G37" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H37" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B37,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B38" s="79" t="inlineStr">
+        <is>
+          <t>HU0004</t>
+        </is>
+      </c>
+      <c r="C38" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D38" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E38" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F38" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G38" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H38" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B38,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B39" s="79" t="inlineStr">
+        <is>
+          <t>HU0005</t>
+        </is>
+      </c>
+      <c r="C39" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D39" s="86" t="inlineStr">
+        <is>
+          <t>Traduccion de mensajes</t>
+        </is>
+      </c>
+      <c r="E39" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F39" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G39" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H39" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B39,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B40" s="79" t="inlineStr">
+        <is>
+          <t>HU0006</t>
+        </is>
+      </c>
+      <c r="C40" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D40" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E40" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F40" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G40" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H40" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B40,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="81" t="inlineStr">
+        <is>
+          <t>Total sprint 1</t>
+        </is>
+      </c>
+      <c r="B41" s="82" t="inlineStr"/>
+      <c r="C41" s="82">
+        <f>"Disponibles: "&amp;Planificacion!$E$8&amp;" h  |  Holgura: "&amp;(Planificacion!$E$8-G41)&amp;" h"</f>
+        <v/>
+      </c>
+      <c r="D41" s="82" t="inlineStr"/>
+      <c r="E41" s="82" t="inlineStr"/>
+      <c r="F41" s="93" t="inlineStr">
+        <is>
+          <t>6 HU</t>
+        </is>
+      </c>
+      <c r="G41" s="83">
+        <f>SUM(G35:G40)</f>
+        <v/>
+      </c>
+      <c r="H41" s="82" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="92">
+        <f>"Sprint 2  |  "&amp;TEXT(B27,"dd/mm/yyyy")&amp;" al "&amp;TEXT(C27,"dd/mm/yyyy")&amp;"  |  "&amp;D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="78" t="inlineStr">
+        <is>
+          <t>Prioridad (valor)</t>
+        </is>
+      </c>
+      <c r="B44" s="78" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="C44" s="78" t="inlineStr">
+        <is>
+          <t>Historia de usuario</t>
+        </is>
+      </c>
+      <c r="D44" s="78" t="inlineStr">
+        <is>
+          <t>Epica</t>
+        </is>
+      </c>
+      <c r="E44" s="78" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="F44" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="G44" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="H44" s="78" t="inlineStr">
+        <is>
+          <t>Por que genera valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B45" s="79" t="inlineStr">
+        <is>
+          <t>HU0007</t>
+        </is>
+      </c>
+      <c r="C45" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D45" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E45" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F45" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G45" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H45" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B45,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B46" s="79" t="inlineStr">
+        <is>
+          <t>HU0008</t>
+        </is>
+      </c>
+      <c r="C46" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D46" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E46" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F46" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G46" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H46" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B46,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B47" s="79" t="inlineStr">
+        <is>
+          <t>HU0009</t>
+        </is>
+      </c>
+      <c r="C47" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D47" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E47" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F47" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G47" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H47" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B47,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B48" s="79" t="inlineStr">
+        <is>
+          <t>HU0010</t>
+        </is>
+      </c>
+      <c r="C48" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D48" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E48" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F48" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G48" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H48" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B48,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B49" s="79" t="inlineStr">
+        <is>
+          <t>HU0019</t>
+        </is>
+      </c>
+      <c r="C49" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D49" s="86" t="inlineStr">
+        <is>
+          <t>Participacion del interlocutor</t>
+        </is>
+      </c>
+      <c r="E49" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F49" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G49" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H49" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B49,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B50" s="79" t="inlineStr">
+        <is>
+          <t>HU0020</t>
+        </is>
+      </c>
+      <c r="C50" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D50" s="86" t="inlineStr">
+        <is>
+          <t>Participacion del interlocutor</t>
+        </is>
+      </c>
+      <c r="E50" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F50" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G50" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H50" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B50,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B51" s="79" t="inlineStr">
+        <is>
+          <t>HU0023</t>
+        </is>
+      </c>
+      <c r="C51" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D51" s="86" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
+      <c r="E51" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F51" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G51" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H51" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B51,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B52" s="79" t="inlineStr">
+        <is>
+          <t>HU0011</t>
+        </is>
+      </c>
+      <c r="C52" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D52" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E52" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F52" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G52" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H52" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B52,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B53" s="79" t="inlineStr">
+        <is>
+          <t>HU0012</t>
+        </is>
+      </c>
+      <c r="C53" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D53" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E53" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F53" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G53" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H53" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B53,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B54" s="79" t="inlineStr">
+        <is>
+          <t>HU0013</t>
+        </is>
+      </c>
+      <c r="C54" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D54" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E54" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F54" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G54" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H54" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B54,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B55" s="79" t="inlineStr">
+        <is>
+          <t>HU0014</t>
+        </is>
+      </c>
+      <c r="C55" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D55" s="86" t="inlineStr">
+        <is>
+          <t>Gestion de conversaciones</t>
+        </is>
+      </c>
+      <c r="E55" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F55" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G55" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H55" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B55,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B56" s="79" t="inlineStr">
+        <is>
+          <t>HU0025</t>
+        </is>
+      </c>
+      <c r="C56" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D56" s="86" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
+      <c r="E56" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F56" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G56" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H56" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B56,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="81" t="inlineStr">
+        <is>
+          <t>Total sprint 2</t>
+        </is>
+      </c>
+      <c r="B57" s="82" t="inlineStr"/>
+      <c r="C57" s="82">
+        <f>"Disponibles: "&amp;Planificacion!$E$8&amp;" h  |  Holgura: "&amp;(Planificacion!$E$8-G57)&amp;" h"</f>
+        <v/>
+      </c>
+      <c r="D57" s="82" t="inlineStr"/>
+      <c r="E57" s="82" t="inlineStr"/>
+      <c r="F57" s="93" t="inlineStr">
+        <is>
+          <t>12 HU</t>
+        </is>
+      </c>
+      <c r="G57" s="83">
+        <f>SUM(G45:G56)</f>
+        <v/>
+      </c>
+      <c r="H57" s="82" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="92">
+        <f>"Sprint 3  |  "&amp;TEXT(B28,"dd/mm/yyyy")&amp;" al "&amp;TEXT(C28,"dd/mm/yyyy")&amp;"  |  "&amp;D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="78" t="inlineStr">
+        <is>
+          <t>Prioridad (valor)</t>
+        </is>
+      </c>
+      <c r="B60" s="78" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="C60" s="78" t="inlineStr">
+        <is>
+          <t>Historia de usuario</t>
+        </is>
+      </c>
+      <c r="D60" s="78" t="inlineStr">
+        <is>
+          <t>Epica</t>
+        </is>
+      </c>
+      <c r="E60" s="78" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="F60" s="78" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="G60" s="78" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="H60" s="78" t="inlineStr">
+        <is>
+          <t>Por que genera valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B61" s="79" t="inlineStr">
+        <is>
+          <t>HU0015</t>
+        </is>
+      </c>
+      <c r="C61" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D61" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E61" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F61" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G61" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H61" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B61,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B62" s="79" t="inlineStr">
+        <is>
+          <t>HU0016</t>
+        </is>
+      </c>
+      <c r="C62" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E62" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F62" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G62" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H62" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B62,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B63" s="79" t="inlineStr">
+        <is>
+          <t>HU0021</t>
+        </is>
+      </c>
+      <c r="C63" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D63" s="86" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="E63" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F63" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G63" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H63" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B63,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B64" s="79" t="inlineStr">
+        <is>
+          <t>HU0017</t>
+        </is>
+      </c>
+      <c r="C64" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D64" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E64" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F64" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G64" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H64" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B64,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B65" s="79" t="inlineStr">
+        <is>
+          <t>HU0018</t>
+        </is>
+      </c>
+      <c r="C65" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D65" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E65" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F65" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G65" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H65" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B65,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B66" s="79" t="inlineStr">
+        <is>
+          <t>HU0022</t>
+        </is>
+      </c>
+      <c r="C66" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D66" s="86" t="inlineStr">
+        <is>
+          <t>Reportes</t>
+        </is>
+      </c>
+      <c r="E66" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F66" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G66" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H66" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B66,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B67" s="79" t="inlineStr">
+        <is>
+          <t>HU0024</t>
+        </is>
+      </c>
+      <c r="C67" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D67" s="86" t="inlineStr">
+        <is>
+          <t>Administracion de idiomas y regiones</t>
+        </is>
+      </c>
+      <c r="E67" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F67" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G67" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H67" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B67,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="80">
+        <f>INDEX(Entregables!$G$2:$G$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="B68" s="79" t="inlineStr">
+        <is>
+          <t>HU0026</t>
+        </is>
+      </c>
+      <c r="C68" s="86">
+        <f>INDEX(Entregables!$C$2:$C$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="D68" s="86" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario</t>
+        </is>
+      </c>
+      <c r="E68" s="86">
+        <f>INDEX(Entregables!$D$2:$D$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="F68" s="80">
+        <f>INDEX(Entregables!$H$2:$H$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="G68" s="80">
+        <f>INDEX(Entregables!$I$2:$I$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+      <c r="H68" s="86">
+        <f>INDEX(Entregables!$K$2:$K$40,MATCH($B68,Entregables!$B$2:$B$40,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="81" t="inlineStr">
+        <is>
+          <t>Total sprint 3</t>
+        </is>
+      </c>
+      <c r="B69" s="82" t="inlineStr"/>
+      <c r="C69" s="82">
+        <f>"Disponibles: "&amp;Planificacion!$E$8&amp;" h  |  Holgura: "&amp;(Planificacion!$E$8-G69)&amp;" h"</f>
+        <v/>
+      </c>
+      <c r="D69" s="82" t="inlineStr"/>
+      <c r="E69" s="82" t="inlineStr"/>
+      <c r="F69" s="93" t="inlineStr">
+        <is>
+          <t>8 HU</t>
+        </is>
+      </c>
+      <c r="G69" s="83">
+        <f>SUM(G61:G68)</f>
+        <v/>
+      </c>
+      <c r="H69" s="82" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="59" t="inlineStr">
+        <is>
+          <t>5. Como se armo</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="69" t="inlineStr">
+        <is>
+          <t>1. La prioridad va por valor para el negocio, no por dependencia: lo que mas valor genera es traducir (HU0003 es la 1); registrarse y cerrar sesion son de apoyo y van al final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="69" t="inlineStr">
+        <is>
+          <t>2. Cada historia se talla con tallas de ropa (XS a XXL) y cada talla tiene horas para una persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="69" t="inlineStr">
+        <is>
+          <t>3. Los sprints duran una semana. Capacidad: 2 personas x 4 horas x 5 dias = 40 horas; se usa el 75 % = 30 horas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="69" t="inlineStr">
+        <is>
+          <t>4. Se llenan los sprints de mayor a menor valor hasta quedar cerca de 30 horas; si sobra espacio se acomoda una historia pequena de mas abajo. Ejemplo: con las prioridades 7 a 15 el sprint 2 llega a 27 horas; las siguientes (HU0015 de 6 h, HU0016 y HU0021 de 4 h) no caben en las 3 horas que quedan, por eso entran HU0013, HU0014 y HU0025 (1 h cada una) y las otras pasan al sprint 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="69" t="inlineStr">
+        <is>
+          <t>5. Con los sprints sale el plan de liberaciones: cada sprint termina con una liberacion. El primero empieza el lunes 19/10/2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A73:I73"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A75:I75"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A76:I76"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A74:I74"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A72:I72"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I26:I28">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FF92D050"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
@@ -3909,7 +5851,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4157,7 +6099,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4324,140 +6266,6 @@
         <f>Entregables!F20</f>
         <v/>
       </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Mapa de Impacto'!A1" display="← Volver al Mapa de Impacto"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Entregable</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="inlineStr">
-        <is>
-          <t>Participacion del interlocutor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Interlocutor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Impacto (para)</t>
-        </is>
-      </c>
-      <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>← Volver al Mapa de Impacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Característica</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Como</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Necesito</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Para</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="18">
-        <f>Entregables!C21</f>
-        <v/>
-      </c>
-      <c r="B8" s="18">
-        <f>Entregables!D21</f>
-        <v/>
-      </c>
-      <c r="C8" s="18">
-        <f>Entregables!E21</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>Entregables!F21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="18">
-        <f>Entregables!C22</f>
-        <v/>
-      </c>
-      <c r="B9" s="18">
-        <f>Entregables!D22</f>
-        <v/>
-      </c>
-      <c r="C9" s="18">
-        <f>Entregables!E22</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>Entregables!F22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="18" t="n"/>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4489,7 +6297,7 @@
       </c>
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>Reportes</t>
+          <t>Participacion del interlocutor</t>
         </is>
       </c>
     </row>
@@ -4501,18 +6309,18 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Cliente Traductor / Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="90" customHeight="1">
+          <t>Interlocutor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Impacto (para)</t>
         </is>
       </c>
       <c r="B3" s="18">
-        <f>'Mapa de Impacto'!C10&amp;CHAR(10)&amp;'Mapa de Impacto'!C13</f>
+        <f>'Mapa de Impacto'!C11</f>
         <v/>
       </c>
     </row>
@@ -4547,37 +6355,37 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18">
-        <f>Entregables!C23</f>
+        <f>Entregables!C21</f>
         <v/>
       </c>
       <c r="B8" s="18">
-        <f>Entregables!D23</f>
+        <f>Entregables!D21</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>Entregables!E23</f>
+        <f>Entregables!E21</f>
         <v/>
       </c>
       <c r="D8" s="18">
-        <f>Entregables!F23</f>
+        <f>Entregables!F21</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="18">
-        <f>Entregables!C24</f>
+        <f>Entregables!C22</f>
         <v/>
       </c>
       <c r="B9" s="18">
-        <f>Entregables!D24</f>
+        <f>Entregables!D22</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>Entregables!E24</f>
+        <f>Entregables!E22</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>Entregables!F24</f>
+        <f>Entregables!F22</f>
         <v/>
       </c>
     </row>

</xml_diff>